<commit_message>
Excel auditado: triangulación y recomendación restauradas; regla de recomendación en el motor
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01M3Z6Fw74B8ffLJq5CxcxMa
</commit_message>
<xml_diff>
--- a/excel/EXCEL FINAL PRO DEFINITIVO SORIANA - AUDITADO.xlsx
+++ b/excel/EXCEL FINAL PRO DEFINITIVO SORIANA - AUDITADO.xlsx
@@ -1430,7 +1430,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2871" uniqueCount="1588">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2902" uniqueCount="1616">
   <si>
     <t xml:space="preserve">1. VALUACIÓN (DCF, base FY2025)</t>
   </si>
@@ -4976,6 +4976,90 @@
   </si>
   <si>
     <t xml:space="preserve">Mediana (estadístico central robusto) en lugar de la media: con n pequeño y un atípico (Profi 21.3x) la media se desplaza al alza.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">6. TRIANGULACIÓN: MODELO, TRANSACCIONES Y OPINIÓN DE LOS EXPERTOS</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Fuente / método</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Precio (MXN)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">DCF (ValuFlow)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Valor intrínseco del modelo del equipo.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Múltiplos de empresas comparables (CIQ).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Transacciones CIQ (hoja Transacciones, media, n = 3) — histórico</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Muestra no defendible (1 de 3 en ventana); incluye prima de control.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Transacciones SDC — mediana (referencia oficial)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Estadístico central robusto de la muestra auditada.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Transacciones SDC — media sin atípicos</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Excluye atípicos por RIC.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Consenso de analistas (precio objetivo, S&amp;P Capital IQ)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Valuación combinada del proyecto (DCF 50% / Comps 50%)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Precio objetivo del proyecto.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Sensibilidad: DCF, Comps y Transacciones SDC (mediana) a ⅓</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Si se diera peso a transacciones con la nueva muestra.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Precio de mercado de referencia (25-sep-2026)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">7. CONCLUSIÓN, VALUACIÓN Y RECOMENDACIÓN</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Umbral para COMPRAR (potencial mayor a)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Umbral para VENDER (potencial menor a)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Precio objetivo (valuación combinada)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Potencial / (baja) vs. mercado</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Recomendación según el modelo</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Recomendación de los expertos</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Rango de valor razonable — bajo (mín. de DCF, Comps y SDC sin atípicos)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Rango de valor razonable — alto</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Precio objetivo de consenso de analistas</t>
   </si>
   <si>
     <t xml:space="preserve">CONTRASTE EXTERNO — S&amp;P Capital IQ, LSEG Refinitiv y modelos propios (referencias; no entran al precio oficial salvo DCF y Trading Comps)</t>
@@ -6662,7 +6746,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="276">
+  <cellXfs count="279">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -7691,6 +7775,18 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
+    <xf numFmtId="165" fontId="0" fillId="4" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="197" fontId="22" fillId="8" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="22" fillId="8" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
     <xf numFmtId="197" fontId="0" fillId="6" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -21668,7 +21764,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:AN81"/>
+  <dimension ref="A1:AN104"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="14"/>
@@ -25784,6 +25880,270 @@
     <row r="81" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A81" s="239" t="s">
         <v>1181</v>
+      </c>
+    </row>
+    <row r="83" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A83" s="240" t="s">
+        <v>1182</v>
+      </c>
+      <c r="B83" s="151"/>
+      <c r="C83" s="151"/>
+      <c r="D83" s="151"/>
+      <c r="E83" s="151"/>
+      <c r="F83" s="151"/>
+      <c r="G83" s="151"/>
+      <c r="H83" s="151"/>
+      <c r="I83" s="151"/>
+      <c r="J83" s="151"/>
+      <c r="K83" s="151"/>
+      <c r="L83" s="151"/>
+    </row>
+    <row r="84" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A84" s="244" t="s">
+        <v>1183</v>
+      </c>
+      <c r="B84" s="244"/>
+      <c r="C84" s="244" t="s">
+        <v>1184</v>
+      </c>
+      <c r="D84" s="244" t="s">
+        <v>1148</v>
+      </c>
+      <c r="E84" s="244" t="s">
+        <v>667</v>
+      </c>
+    </row>
+    <row r="85" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A85" s="0" t="s">
+        <v>1185</v>
+      </c>
+      <c r="C85" s="252" t="n">
+        <f aca="false">'Valuación Combinada'!B4</f>
+        <v>31.6168901445216</v>
+      </c>
+      <c r="D85" s="120" t="n">
+        <f aca="false">C85/$C$93-1</f>
+        <v>-0.0556484425172753</v>
+      </c>
+      <c r="E85" s="36" t="s">
+        <v>1186</v>
+      </c>
+    </row>
+    <row r="86" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A86" s="0" t="s">
+        <v>958</v>
+      </c>
+      <c r="C86" s="252" t="n">
+        <f aca="false">'Valuación Combinada'!B5</f>
+        <v>33.4928408544974</v>
+      </c>
+      <c r="D86" s="120" t="n">
+        <f aca="false">C86/$C$93-1</f>
+        <v>0.000383538067423972</v>
+      </c>
+      <c r="E86" s="36" t="s">
+        <v>1187</v>
+      </c>
+    </row>
+    <row r="87" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A87" s="0" t="s">
+        <v>1188</v>
+      </c>
+      <c r="C87" s="252" t="n">
+        <f aca="false">Transacciones!E49</f>
+        <v>40.7283951666667</v>
+      </c>
+      <c r="D87" s="120" t="n">
+        <f aca="false">C87/$C$93-1</f>
+        <v>0.21649925826364</v>
+      </c>
+      <c r="E87" s="36" t="s">
+        <v>1189</v>
+      </c>
+    </row>
+    <row r="88" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A88" s="0" t="s">
+        <v>1190</v>
+      </c>
+      <c r="C88" s="252" t="n">
+        <f aca="false">F53</f>
+        <v>23.7448001083333</v>
+      </c>
+      <c r="D88" s="120" t="n">
+        <f aca="false">C88/$C$93-1</f>
+        <v>-0.290776579798885</v>
+      </c>
+      <c r="E88" s="36" t="s">
+        <v>1191</v>
+      </c>
+    </row>
+    <row r="89" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A89" s="0" t="s">
+        <v>1192</v>
+      </c>
+      <c r="C89" s="252" t="n">
+        <f aca="false">F60</f>
+        <v>28.9893892547619</v>
+      </c>
+      <c r="D89" s="120" t="n">
+        <f aca="false">C89/$C$93-1</f>
+        <v>-0.13412815845992</v>
+      </c>
+      <c r="E89" s="36" t="s">
+        <v>1193</v>
+      </c>
+    </row>
+    <row r="90" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A90" s="0" t="s">
+        <v>1194</v>
+      </c>
+      <c r="C90" s="252" t="n">
+        <f aca="false">Comparativo!B18</f>
+        <v>23.357</v>
+      </c>
+      <c r="D90" s="120" t="n">
+        <f aca="false">C90/$C$93-1</f>
+        <v>-0.302359617682198</v>
+      </c>
+      <c r="E90" s="0" t="str">
+        <f aca="false">"Expertos: "&amp;Comparativo!B19&amp;" — sesgo vendedor."</f>
+        <v>Expertos: Venta (0 C / 1 M / 6 V) — sesgo vendedor.</v>
+      </c>
+    </row>
+    <row r="91" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A91" s="0" t="s">
+        <v>1195</v>
+      </c>
+      <c r="C91" s="252" t="n">
+        <f aca="false">'Valuación Combinada'!B9</f>
+        <v>32.5548654995095</v>
+      </c>
+      <c r="D91" s="120" t="n">
+        <f aca="false">C91/$C$93-1</f>
+        <v>-0.0276324522249256</v>
+      </c>
+      <c r="E91" s="36" t="s">
+        <v>1196</v>
+      </c>
+    </row>
+    <row r="92" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A92" s="0" t="s">
+        <v>1197</v>
+      </c>
+      <c r="C92" s="252" t="n">
+        <f aca="false">AVERAGE(C85,C86,C88)</f>
+        <v>29.6181770357841</v>
+      </c>
+      <c r="D92" s="120" t="n">
+        <f aca="false">C92/$C$93-1</f>
+        <v>-0.115347161416245</v>
+      </c>
+      <c r="E92" s="36" t="s">
+        <v>1198</v>
+      </c>
+    </row>
+    <row r="93" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A93" s="0" t="s">
+        <v>1199</v>
+      </c>
+      <c r="C93" s="252" t="n">
+        <f aca="false">'Valuación Combinada'!B10</f>
+        <v>33.48</v>
+      </c>
+    </row>
+    <row r="95" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A95" s="240" t="s">
+        <v>1200</v>
+      </c>
+      <c r="B95" s="151"/>
+      <c r="C95" s="151"/>
+      <c r="D95" s="151"/>
+      <c r="E95" s="151"/>
+      <c r="F95" s="151"/>
+      <c r="G95" s="151"/>
+      <c r="H95" s="151"/>
+      <c r="I95" s="151"/>
+      <c r="J95" s="151"/>
+      <c r="K95" s="151"/>
+      <c r="L95" s="151"/>
+    </row>
+    <row r="96" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A96" s="0" t="s">
+        <v>1201</v>
+      </c>
+      <c r="C96" s="257" t="n">
+        <v>0.1</v>
+      </c>
+    </row>
+    <row r="97" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A97" s="0" t="s">
+        <v>1202</v>
+      </c>
+      <c r="C97" s="257" t="n">
+        <v>-0.1</v>
+      </c>
+    </row>
+    <row r="98" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A98" s="0" t="s">
+        <v>1203</v>
+      </c>
+      <c r="C98" s="258" t="n">
+        <f aca="false">C91</f>
+        <v>32.5548654995095</v>
+      </c>
+    </row>
+    <row r="99" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A99" s="0" t="s">
+        <v>1204</v>
+      </c>
+      <c r="C99" s="120" t="n">
+        <f aca="false">C98/C93-1</f>
+        <v>-0.0276324522249256</v>
+      </c>
+    </row>
+    <row r="100" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A100" s="0" t="s">
+        <v>1205</v>
+      </c>
+      <c r="C100" s="259" t="str">
+        <f aca="false">IF(C99&gt;C96,"COMPRAR",IF(C99&lt;C97,"VENDER","MANTENER"))</f>
+        <v>MANTENER</v>
+      </c>
+    </row>
+    <row r="101" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A101" s="0" t="s">
+        <v>1206</v>
+      </c>
+      <c r="C101" s="0" t="str">
+        <f aca="false">Comparativo!B19</f>
+        <v>Venta (0 C / 1 M / 6 V)</v>
+      </c>
+    </row>
+    <row r="102" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A102" s="0" t="s">
+        <v>1207</v>
+      </c>
+      <c r="C102" s="252" t="n">
+        <f aca="false">MIN(C85,C86,C89)</f>
+        <v>28.9893892547619</v>
+      </c>
+    </row>
+    <row r="103" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A103" s="0" t="s">
+        <v>1208</v>
+      </c>
+      <c r="C103" s="252" t="n">
+        <f aca="false">MAX(C85,C86,C89)</f>
+        <v>33.4928408544974</v>
+      </c>
+    </row>
+    <row r="104" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A104" s="0" t="s">
+        <v>1209</v>
+      </c>
+      <c r="C104" s="252" t="n">
+        <f aca="false">C90</f>
+        <v>23.357</v>
       </c>
     </row>
   </sheetData>
@@ -25821,17 +26181,17 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="238" t="s">
-        <v>1182</v>
+        <v>1210</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="239" t="s">
-        <v>1183</v>
+        <v>1211</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="55.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="244" t="s">
-        <v>1184</v>
+        <v>1212</v>
       </c>
       <c r="B4" s="244" t="s">
         <v>721</v>
@@ -25840,16 +26200,16 @@
         <v>950</v>
       </c>
       <c r="D4" s="244" t="s">
-        <v>1185</v>
+        <v>1213</v>
       </c>
       <c r="E4" s="244" t="s">
         <v>311</v>
       </c>
       <c r="F4" s="244" t="s">
-        <v>1186</v>
+        <v>1214</v>
       </c>
       <c r="G4" s="244" t="s">
-        <v>1187</v>
+        <v>1215</v>
       </c>
       <c r="H4" s="244" t="s">
         <v>886</v>
@@ -25858,65 +26218,65 @@
         <v>206</v>
       </c>
       <c r="J4" s="244" t="s">
-        <v>1188</v>
+        <v>1216</v>
       </c>
       <c r="K4" s="244" t="s">
-        <v>1189</v>
+        <v>1217</v>
       </c>
       <c r="L4" s="244" t="s">
-        <v>1190</v>
+        <v>1218</v>
       </c>
       <c r="M4" s="244" t="s">
-        <v>1191</v>
+        <v>1219</v>
       </c>
       <c r="N4" s="244" t="s">
-        <v>1192</v>
+        <v>1220</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="0" t="s">
-        <v>1193</v>
+        <v>1221</v>
       </c>
       <c r="B5" s="0" t="s">
-        <v>1194</v>
+        <v>1222</v>
       </c>
       <c r="C5" s="0" t="s">
-        <v>1195</v>
+        <v>1223</v>
       </c>
       <c r="D5" s="0" t="s">
-        <v>1196</v>
-      </c>
-      <c r="E5" s="257" t="n">
+        <v>1224</v>
+      </c>
+      <c r="E5" s="260" t="n">
         <f aca="false">'Proyección Final Soriana'!B265</f>
         <v>31.6168901445216</v>
       </c>
-      <c r="F5" s="257" t="n">
+      <c r="F5" s="260" t="n">
         <f aca="false">'Valuación Combinada'!B18</f>
         <v>31.2773490371468</v>
       </c>
-      <c r="G5" s="257" t="n">
+      <c r="G5" s="260" t="n">
         <f aca="false">'Valuación Combinada'!D18</f>
         <v>32.289933097456</v>
       </c>
-      <c r="H5" s="257" t="n">
+      <c r="H5" s="260" t="n">
         <f aca="false">'Valuación Combinada'!B10</f>
         <v>33.48</v>
       </c>
       <c r="I5" s="36" t="s">
-        <v>1197</v>
+        <v>1225</v>
       </c>
       <c r="J5" s="120" t="n">
         <f aca="false">IF(AND(ISNUMBER(E5),ISNUMBER(H5)),E5/H5-1,"NA")</f>
         <v>-0.0556484425172753</v>
       </c>
       <c r="K5" s="36" t="s">
-        <v>1198</v>
+        <v>1226</v>
       </c>
       <c r="L5" s="36" t="s">
-        <v>1199</v>
+        <v>1227</v>
       </c>
       <c r="M5" s="36" t="s">
-        <v>1200</v>
+        <v>1228</v>
       </c>
       <c r="N5" s="36" t="s">
         <v>587</v>
@@ -25924,48 +26284,48 @@
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="0" t="s">
-        <v>1201</v>
+        <v>1229</v>
       </c>
       <c r="B6" s="0" t="s">
-        <v>1194</v>
+        <v>1222</v>
       </c>
       <c r="C6" s="0" t="s">
-        <v>1202</v>
+        <v>1230</v>
       </c>
       <c r="D6" s="0" t="s">
-        <v>1203</v>
-      </c>
-      <c r="E6" s="257" t="n">
+        <v>1231</v>
+      </c>
+      <c r="E6" s="260" t="n">
         <f aca="false">'Valuación Combinada'!B5</f>
         <v>33.4928408544974</v>
       </c>
-      <c r="F6" s="257" t="n">
+      <c r="F6" s="260" t="n">
         <f aca="false">'Valuación Combinada'!B19</f>
         <v>27.031161037037</v>
       </c>
-      <c r="G6" s="257" t="n">
+      <c r="G6" s="260" t="n">
         <f aca="false">'Valuación Combinada'!D19</f>
         <v>40.0699866203704</v>
       </c>
-      <c r="H6" s="257" t="n">
+      <c r="H6" s="260" t="n">
         <f aca="false">'Valuación Combinada'!B10</f>
         <v>33.48</v>
       </c>
       <c r="I6" s="36" t="s">
-        <v>1197</v>
+        <v>1225</v>
       </c>
       <c r="J6" s="120" t="n">
         <f aca="false">IF(AND(ISNUMBER(E6),ISNUMBER(H6)),E6/H6-1,"NA")</f>
         <v>0.000383538067423972</v>
       </c>
       <c r="K6" s="36" t="s">
-        <v>1204</v>
+        <v>1232</v>
       </c>
       <c r="L6" s="36" t="s">
-        <v>1205</v>
+        <v>1233</v>
       </c>
       <c r="M6" s="36" t="s">
-        <v>1200</v>
+        <v>1228</v>
       </c>
       <c r="N6" s="36" t="s">
         <v>587</v>
@@ -25973,48 +26333,48 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="0" t="s">
-        <v>1206</v>
+        <v>1234</v>
       </c>
       <c r="B7" s="0" t="s">
-        <v>1194</v>
+        <v>1222</v>
       </c>
       <c r="C7" s="0" t="s">
-        <v>1207</v>
+        <v>1235</v>
       </c>
       <c r="D7" s="0" t="s">
-        <v>1208</v>
-      </c>
-      <c r="E7" s="257" t="n">
+        <v>1236</v>
+      </c>
+      <c r="E7" s="260" t="n">
         <f aca="false">'Valuación Combinada'!B6</f>
         <v>23.7448001083333</v>
       </c>
-      <c r="F7" s="257" t="n">
+      <c r="F7" s="260" t="n">
         <f aca="false">'Valuación Combinada'!B20</f>
         <v>20.4147906458333</v>
       </c>
-      <c r="G7" s="257" t="n">
+      <c r="G7" s="260" t="n">
         <f aca="false">'Valuación Combinada'!D20</f>
         <v>49.1873847208333</v>
       </c>
-      <c r="H7" s="257" t="n">
+      <c r="H7" s="260" t="n">
         <f aca="false">'Valuación Combinada'!B10</f>
         <v>33.48</v>
       </c>
       <c r="I7" s="36" t="s">
-        <v>1197</v>
+        <v>1225</v>
       </c>
       <c r="J7" s="120" t="n">
         <f aca="false">IF(AND(ISNUMBER(E7),ISNUMBER(H7)),E7/H7-1,"NA")</f>
         <v>-0.290776579798885</v>
       </c>
       <c r="K7" s="36" t="s">
-        <v>1209</v>
+        <v>1237</v>
       </c>
       <c r="L7" s="36" t="s">
-        <v>1210</v>
+        <v>1238</v>
       </c>
       <c r="M7" s="36" t="s">
-        <v>1211</v>
+        <v>1239</v>
       </c>
       <c r="N7" s="36" t="s">
         <v>587</v>
@@ -26022,48 +26382,48 @@
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="0" t="s">
-        <v>1212</v>
+        <v>1240</v>
       </c>
       <c r="B8" s="0" t="s">
-        <v>1194</v>
+        <v>1222</v>
       </c>
       <c r="C8" s="0" t="s">
-        <v>1213</v>
+        <v>1241</v>
       </c>
       <c r="D8" s="0" t="s">
         <v>587</v>
       </c>
-      <c r="E8" s="257" t="n">
+      <c r="E8" s="260" t="n">
         <f aca="false">Transacciones!E49</f>
         <v>40.7283951666667</v>
       </c>
-      <c r="F8" s="257" t="n">
+      <c r="F8" s="260" t="n">
         <f aca="false">Transacciones!E28</f>
         <v>24.7618473333333</v>
       </c>
-      <c r="G8" s="257" t="n">
+      <c r="G8" s="260" t="n">
         <f aca="false">Transacciones!E33</f>
         <v>65.4437363333333</v>
       </c>
-      <c r="H8" s="257" t="n">
+      <c r="H8" s="260" t="n">
         <f aca="false">'Valuación Combinada'!B10</f>
         <v>33.48</v>
       </c>
       <c r="I8" s="36" t="s">
-        <v>1197</v>
+        <v>1225</v>
       </c>
       <c r="J8" s="120" t="n">
         <f aca="false">IF(AND(ISNUMBER(E8),ISNUMBER(H8)),E8/H8-1,"NA")</f>
         <v>0.21649925826364</v>
       </c>
       <c r="K8" s="36" t="s">
-        <v>1214</v>
+        <v>1242</v>
       </c>
       <c r="L8" s="36" t="s">
-        <v>1215</v>
+        <v>1243</v>
       </c>
       <c r="M8" s="36" t="s">
-        <v>1216</v>
+        <v>1244</v>
       </c>
       <c r="N8" s="36" t="s">
         <v>587</v>
@@ -26071,40 +26431,40 @@
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="0" t="s">
-        <v>1217</v>
+        <v>1245</v>
       </c>
       <c r="B9" s="0" t="s">
-        <v>1194</v>
+        <v>1222</v>
       </c>
       <c r="C9" s="0" t="s">
-        <v>1218</v>
+        <v>1246</v>
       </c>
       <c r="D9" s="0" t="s">
-        <v>1196</v>
-      </c>
-      <c r="E9" s="257" t="n">
+        <v>1224</v>
+      </c>
+      <c r="E9" s="260" t="n">
         <f aca="false">'Valuación Combinada'!B9</f>
         <v>32.5548654995095</v>
       </c>
-      <c r="H9" s="257" t="n">
+      <c r="H9" s="260" t="n">
         <f aca="false">'Valuación Combinada'!B10</f>
         <v>33.48</v>
       </c>
       <c r="I9" s="36" t="s">
-        <v>1197</v>
+        <v>1225</v>
       </c>
       <c r="J9" s="120" t="n">
         <f aca="false">IF(AND(ISNUMBER(E9),ISNUMBER(H9)),E9/H9-1,"NA")</f>
         <v>-0.0276324522249256</v>
       </c>
       <c r="K9" s="36" t="s">
-        <v>1219</v>
+        <v>1247</v>
       </c>
       <c r="L9" s="36" t="s">
         <v>587</v>
       </c>
       <c r="M9" s="36" t="s">
-        <v>1220</v>
+        <v>1248</v>
       </c>
       <c r="N9" s="36" t="s">
         <v>587</v>
@@ -26112,444 +26472,444 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="0" t="s">
-        <v>1221</v>
+        <v>1249</v>
       </c>
       <c r="B10" s="0" t="s">
-        <v>1222</v>
+        <v>1250</v>
       </c>
       <c r="C10" s="0" t="s">
         <v>973</v>
       </c>
       <c r="D10" s="0" t="s">
-        <v>1223</v>
-      </c>
-      <c r="E10" s="258" t="n">
+        <v>1251</v>
+      </c>
+      <c r="E10" s="261" t="n">
         <v>39.21</v>
       </c>
-      <c r="F10" s="258" t="n">
+      <c r="F10" s="261" t="n">
         <v>32.12</v>
       </c>
-      <c r="G10" s="258" t="n">
+      <c r="G10" s="261" t="n">
         <v>47.74</v>
       </c>
-      <c r="H10" s="258" t="n">
+      <c r="H10" s="261" t="n">
         <v>33.1</v>
       </c>
       <c r="I10" s="36" t="s">
-        <v>1223</v>
+        <v>1251</v>
       </c>
       <c r="J10" s="120" t="n">
         <f aca="false">IF(AND(ISNUMBER(E10),ISNUMBER(H10)),E10/H10-1,"NA")</f>
         <v>0.184592145015106</v>
       </c>
       <c r="K10" s="36" t="s">
-        <v>1224</v>
+        <v>1252</v>
       </c>
       <c r="L10" s="36" t="s">
-        <v>1225</v>
+        <v>1253</v>
       </c>
       <c r="M10" s="36" t="s">
-        <v>1226</v>
+        <v>1254</v>
       </c>
       <c r="N10" s="36" t="s">
-        <v>1227</v>
+        <v>1255</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="0" t="s">
-        <v>1228</v>
+        <v>1256</v>
       </c>
       <c r="B11" s="0" t="s">
-        <v>1229</v>
+        <v>1257</v>
       </c>
       <c r="C11" s="0" t="s">
-        <v>1230</v>
+        <v>1258</v>
       </c>
       <c r="D11" s="0" t="s">
-        <v>1223</v>
-      </c>
-      <c r="E11" s="258" t="n">
+        <v>1251</v>
+      </c>
+      <c r="E11" s="261" t="n">
         <v>36.35</v>
       </c>
-      <c r="H11" s="258" t="n">
+      <c r="H11" s="261" t="n">
         <v>33.1</v>
       </c>
       <c r="I11" s="36" t="s">
-        <v>1223</v>
+        <v>1251</v>
       </c>
       <c r="J11" s="120" t="n">
         <f aca="false">IF(AND(ISNUMBER(E11),ISNUMBER(H11)),E11/H11-1,"NA")</f>
         <v>0.0981873111782476</v>
       </c>
       <c r="K11" s="36" t="s">
-        <v>1219</v>
+        <v>1247</v>
       </c>
       <c r="L11" s="36" t="s">
-        <v>1231</v>
+        <v>1259</v>
       </c>
       <c r="M11" s="36" t="s">
-        <v>1232</v>
+        <v>1260</v>
       </c>
       <c r="N11" s="36" t="s">
-        <v>1233</v>
+        <v>1261</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="0" t="s">
-        <v>1234</v>
+        <v>1262</v>
       </c>
       <c r="B12" s="0" t="s">
-        <v>1235</v>
+        <v>1263</v>
       </c>
       <c r="C12" s="0" t="s">
         <v>973</v>
       </c>
       <c r="D12" s="0" t="s">
-        <v>1196</v>
-      </c>
-      <c r="E12" s="258" t="n">
+        <v>1224</v>
+      </c>
+      <c r="E12" s="261" t="n">
         <v>31.16</v>
       </c>
-      <c r="F12" s="258" t="n">
+      <c r="F12" s="261" t="n">
         <v>25.91</v>
       </c>
-      <c r="G12" s="258" t="n">
+      <c r="G12" s="261" t="n">
         <v>37.56</v>
       </c>
-      <c r="H12" s="258" t="n">
+      <c r="H12" s="261" t="n">
         <v>33.48</v>
       </c>
       <c r="I12" s="36" t="s">
-        <v>1197</v>
+        <v>1225</v>
       </c>
       <c r="J12" s="120" t="n">
         <f aca="false">IF(AND(ISNUMBER(E12),ISNUMBER(H12)),E12/H12-1,"NA")</f>
         <v>-0.069295101553166</v>
       </c>
       <c r="K12" s="36" t="s">
-        <v>1236</v>
+        <v>1264</v>
       </c>
       <c r="L12" s="36" t="s">
-        <v>1237</v>
+        <v>1265</v>
       </c>
       <c r="M12" s="36" t="s">
-        <v>1216</v>
+        <v>1244</v>
       </c>
       <c r="N12" s="36" t="s">
-        <v>1238</v>
+        <v>1266</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="0" t="s">
-        <v>1239</v>
+        <v>1267</v>
       </c>
       <c r="B13" s="0" t="s">
-        <v>1240</v>
+        <v>1268</v>
       </c>
       <c r="C13" s="0" t="s">
-        <v>1241</v>
+        <v>1269</v>
       </c>
       <c r="D13" s="0" t="s">
-        <v>1208</v>
-      </c>
-      <c r="E13" s="258" t="n">
+        <v>1236</v>
+      </c>
+      <c r="E13" s="261" t="n">
         <v>38.27</v>
       </c>
-      <c r="F13" s="258" t="n">
+      <c r="F13" s="261" t="n">
         <v>34.8</v>
       </c>
-      <c r="G13" s="258" t="n">
+      <c r="G13" s="261" t="n">
         <v>43</v>
       </c>
-      <c r="H13" s="258" t="n">
+      <c r="H13" s="261" t="n">
         <v>33.1</v>
       </c>
       <c r="I13" s="36" t="s">
-        <v>1223</v>
+        <v>1251</v>
       </c>
       <c r="J13" s="120" t="n">
         <f aca="false">IF(AND(ISNUMBER(E13),ISNUMBER(H13)),E13/H13-1,"NA")</f>
         <v>0.15619335347432</v>
       </c>
       <c r="K13" s="36" t="s">
-        <v>1242</v>
+        <v>1270</v>
       </c>
       <c r="L13" s="36" t="s">
-        <v>1243</v>
+        <v>1271</v>
       </c>
       <c r="M13" s="36" t="s">
-        <v>1232</v>
+        <v>1260</v>
       </c>
       <c r="N13" s="36" t="s">
-        <v>1244</v>
+        <v>1272</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="0" t="s">
-        <v>1245</v>
+        <v>1273</v>
       </c>
       <c r="B14" s="0" t="s">
-        <v>1246</v>
+        <v>1274</v>
       </c>
       <c r="C14" s="0" t="s">
-        <v>1247</v>
+        <v>1275</v>
       </c>
       <c r="D14" s="0" t="s">
-        <v>1208</v>
-      </c>
-      <c r="E14" s="258" t="n">
+        <v>1236</v>
+      </c>
+      <c r="E14" s="261" t="n">
         <v>29.7</v>
       </c>
-      <c r="F14" s="258" t="n">
+      <c r="F14" s="261" t="n">
         <v>25.3</v>
       </c>
-      <c r="G14" s="258" t="n">
+      <c r="G14" s="261" t="n">
         <v>33.8</v>
       </c>
-      <c r="H14" s="258" t="n">
+      <c r="H14" s="261" t="n">
         <v>33.1</v>
       </c>
       <c r="I14" s="36" t="s">
-        <v>1223</v>
+        <v>1251</v>
       </c>
       <c r="J14" s="120" t="n">
         <f aca="false">IF(AND(ISNUMBER(E14),ISNUMBER(H14)),E14/H14-1,"NA")</f>
         <v>-0.102719033232628</v>
       </c>
       <c r="K14" s="36" t="s">
-        <v>1248</v>
+        <v>1276</v>
       </c>
       <c r="L14" s="36" t="s">
-        <v>1249</v>
+        <v>1277</v>
       </c>
       <c r="M14" s="36" t="s">
-        <v>1232</v>
+        <v>1260</v>
       </c>
       <c r="N14" s="36" t="s">
-        <v>1250</v>
+        <v>1278</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="0" t="s">
+        <v>1279</v>
+      </c>
+      <c r="B15" s="0" t="s">
+        <v>1274</v>
+      </c>
+      <c r="C15" s="0" t="s">
+        <v>1280</v>
+      </c>
+      <c r="D15" s="0" t="s">
+        <v>1236</v>
+      </c>
+      <c r="E15" s="261" t="n">
+        <v>28.54</v>
+      </c>
+      <c r="F15" s="261" t="n">
+        <v>21.91</v>
+      </c>
+      <c r="G15" s="261" t="n">
+        <v>59.3</v>
+      </c>
+      <c r="H15" s="261" t="n">
+        <v>33.1</v>
+      </c>
+      <c r="I15" s="36" t="s">
         <v>1251</v>
-      </c>
-      <c r="B15" s="0" t="s">
-        <v>1246</v>
-      </c>
-      <c r="C15" s="0" t="s">
-        <v>1252</v>
-      </c>
-      <c r="D15" s="0" t="s">
-        <v>1208</v>
-      </c>
-      <c r="E15" s="258" t="n">
-        <v>28.54</v>
-      </c>
-      <c r="F15" s="258" t="n">
-        <v>21.91</v>
-      </c>
-      <c r="G15" s="258" t="n">
-        <v>59.3</v>
-      </c>
-      <c r="H15" s="258" t="n">
-        <v>33.1</v>
-      </c>
-      <c r="I15" s="36" t="s">
-        <v>1223</v>
       </c>
       <c r="J15" s="120" t="n">
         <f aca="false">IF(AND(ISNUMBER(E15),ISNUMBER(H15)),E15/H15-1,"NA")</f>
         <v>-0.137764350453172</v>
       </c>
       <c r="K15" s="36" t="s">
-        <v>1253</v>
+        <v>1281</v>
       </c>
       <c r="L15" s="36" t="s">
-        <v>1254</v>
+        <v>1282</v>
       </c>
       <c r="M15" s="36" t="s">
-        <v>1232</v>
+        <v>1260</v>
       </c>
       <c r="N15" s="36" t="s">
-        <v>1255</v>
+        <v>1283</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="0" t="s">
-        <v>1256</v>
+        <v>1284</v>
       </c>
       <c r="B16" s="0" t="s">
-        <v>1246</v>
+        <v>1274</v>
       </c>
       <c r="C16" s="0" t="s">
-        <v>1257</v>
+        <v>1285</v>
       </c>
       <c r="D16" s="0" t="s">
-        <v>1208</v>
-      </c>
-      <c r="E16" s="258" t="n">
+        <v>1236</v>
+      </c>
+      <c r="E16" s="261" t="n">
         <v>33.98</v>
       </c>
-      <c r="H16" s="258" t="n">
+      <c r="H16" s="261" t="n">
         <v>33.1</v>
       </c>
       <c r="I16" s="36" t="s">
-        <v>1223</v>
+        <v>1251</v>
       </c>
       <c r="J16" s="120" t="n">
         <f aca="false">IF(AND(ISNUMBER(E16),ISNUMBER(H16)),E16/H16-1,"NA")</f>
         <v>0.0265861027190331</v>
       </c>
       <c r="K16" s="36" t="s">
-        <v>1258</v>
+        <v>1286</v>
       </c>
       <c r="L16" s="36" t="s">
-        <v>1259</v>
+        <v>1287</v>
       </c>
       <c r="M16" s="36" t="s">
-        <v>1232</v>
+        <v>1260</v>
       </c>
       <c r="N16" s="36" t="s">
-        <v>1260</v>
+        <v>1288</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="0" t="s">
-        <v>1261</v>
+        <v>1289</v>
       </c>
       <c r="B17" s="0" t="s">
-        <v>1246</v>
+        <v>1274</v>
       </c>
       <c r="C17" s="0" t="s">
-        <v>1262</v>
+        <v>1290</v>
       </c>
       <c r="D17" s="0" t="s">
-        <v>1208</v>
-      </c>
-      <c r="E17" s="258" t="n">
+        <v>1236</v>
+      </c>
+      <c r="E17" s="261" t="n">
         <v>23.36</v>
       </c>
-      <c r="F17" s="258" t="n">
+      <c r="F17" s="261" t="n">
         <v>18.5</v>
       </c>
-      <c r="G17" s="258" t="n">
+      <c r="G17" s="261" t="n">
         <v>30</v>
       </c>
-      <c r="H17" s="258" t="n">
+      <c r="H17" s="261" t="n">
         <v>33.1</v>
       </c>
       <c r="I17" s="36" t="s">
-        <v>1223</v>
+        <v>1251</v>
       </c>
       <c r="J17" s="120" t="n">
         <f aca="false">IF(AND(ISNUMBER(E17),ISNUMBER(H17)),E17/H17-1,"NA")</f>
         <v>-0.294259818731118</v>
       </c>
       <c r="K17" s="36" t="s">
-        <v>1263</v>
+        <v>1291</v>
       </c>
       <c r="L17" s="36" t="s">
-        <v>1264</v>
+        <v>1292</v>
       </c>
       <c r="M17" s="36" t="s">
-        <v>1232</v>
+        <v>1260</v>
       </c>
       <c r="N17" s="36" t="s">
-        <v>1265</v>
+        <v>1293</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="0" t="s">
-        <v>1266</v>
+        <v>1294</v>
       </c>
       <c r="B18" s="0" t="s">
-        <v>1267</v>
+        <v>1295</v>
       </c>
       <c r="C18" s="0" t="s">
-        <v>1262</v>
+        <v>1290</v>
       </c>
       <c r="D18" s="0" t="s">
-        <v>1208</v>
-      </c>
-      <c r="E18" s="258" t="n">
+        <v>1236</v>
+      </c>
+      <c r="E18" s="261" t="n">
         <v>22.42</v>
       </c>
-      <c r="H18" s="258" t="n">
+      <c r="H18" s="261" t="n">
         <v>33.1</v>
       </c>
       <c r="I18" s="36" t="s">
-        <v>1223</v>
+        <v>1251</v>
       </c>
       <c r="J18" s="120" t="n">
         <f aca="false">IF(AND(ISNUMBER(E18),ISNUMBER(H18)),E18/H18-1,"NA")</f>
         <v>-0.322658610271903</v>
       </c>
       <c r="K18" s="36" t="s">
-        <v>1268</v>
+        <v>1296</v>
       </c>
       <c r="L18" s="36" t="s">
-        <v>1269</v>
+        <v>1297</v>
       </c>
       <c r="M18" s="36" t="s">
-        <v>1232</v>
+        <v>1260</v>
       </c>
       <c r="N18" s="36" t="s">
-        <v>1270</v>
+        <v>1298</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="0" t="s">
-        <v>1271</v>
+        <v>1299</v>
       </c>
       <c r="B19" s="0" t="s">
-        <v>1272</v>
+        <v>1300</v>
       </c>
       <c r="C19" s="0" t="s">
-        <v>1273</v>
+        <v>1301</v>
       </c>
       <c r="D19" s="0" t="s">
-        <v>1208</v>
-      </c>
-      <c r="E19" s="258" t="n">
+        <v>1236</v>
+      </c>
+      <c r="E19" s="261" t="n">
         <v>51</v>
       </c>
-      <c r="F19" s="258" t="n">
+      <c r="F19" s="261" t="n">
         <v>49.5</v>
       </c>
-      <c r="G19" s="258" t="n">
+      <c r="G19" s="261" t="n">
         <v>52.5</v>
       </c>
-      <c r="H19" s="258" t="n">
+      <c r="H19" s="261" t="n">
         <v>33.1</v>
       </c>
       <c r="I19" s="36" t="s">
-        <v>1223</v>
+        <v>1251</v>
       </c>
       <c r="J19" s="120" t="n">
         <f aca="false">IF(AND(ISNUMBER(E19),ISNUMBER(H19)),E19/H19-1,"NA")</f>
         <v>0.540785498489426</v>
       </c>
       <c r="K19" s="36" t="s">
-        <v>1274</v>
+        <v>1302</v>
       </c>
       <c r="L19" s="36" t="s">
-        <v>1275</v>
+        <v>1303</v>
       </c>
       <c r="M19" s="36" t="s">
-        <v>1232</v>
+        <v>1260</v>
       </c>
       <c r="N19" s="36" t="s">
-        <v>1276</v>
+        <v>1304</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="239" t="s">
-        <v>1277</v>
+        <v>1305</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="239" t="s">
-        <v>1278</v>
+        <v>1306</v>
       </c>
     </row>
   </sheetData>
@@ -26578,22 +26938,22 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="122" t="s">
-        <v>1279</v>
+        <v>1307</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="123" t="s">
-        <v>1280</v>
+        <v>1308</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="123" t="s">
-        <v>1281</v>
+        <v>1309</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="150" t="s">
-        <v>1282</v>
+        <v>1310</v>
       </c>
       <c r="B5" s="151"/>
       <c r="C5" s="151"/>
@@ -26606,68 +26966,68 @@
     </row>
     <row r="6" customFormat="false" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="129" t="s">
-        <v>1283</v>
+        <v>1311</v>
       </c>
       <c r="B6" s="129" t="s">
-        <v>1284</v>
+        <v>1312</v>
       </c>
       <c r="C6" s="129" t="s">
-        <v>1285</v>
+        <v>1313</v>
       </c>
       <c r="D6" s="129" t="s">
-        <v>1286</v>
+        <v>1314</v>
       </c>
       <c r="E6" s="129" t="s">
         <v>685</v>
       </c>
       <c r="F6" s="129" t="s">
-        <v>1287</v>
+        <v>1315</v>
       </c>
       <c r="G6" s="129" t="s">
         <v>691</v>
       </c>
       <c r="H6" s="129" t="s">
-        <v>1288</v>
+        <v>1316</v>
       </c>
       <c r="I6" s="129" t="s">
-        <v>1289</v>
+        <v>1317</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="57" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="0" t="s">
-        <v>1290</v>
+        <v>1318</v>
       </c>
       <c r="B7" s="0" t="s">
-        <v>1291</v>
-      </c>
-      <c r="C7" s="259" t="n">
+        <v>1319</v>
+      </c>
+      <c r="C7" s="262" t="n">
         <v>0.0393</v>
       </c>
-      <c r="D7" s="259" t="n">
+      <c r="D7" s="262" t="n">
         <v>0.0393</v>
       </c>
-      <c r="E7" s="259" t="n">
+      <c r="E7" s="262" t="n">
         <v>0.0326</v>
       </c>
-      <c r="F7" s="259" t="n">
+      <c r="F7" s="262" t="n">
         <v>0.0351</v>
       </c>
-      <c r="G7" s="259" t="n">
+      <c r="G7" s="262" t="n">
         <v>0.04</v>
       </c>
-      <c r="H7" s="259" t="n">
+      <c r="H7" s="262" t="n">
         <v>0.0351</v>
       </c>
       <c r="I7" s="132" t="s">
-        <v>1292</v>
+        <v>1320</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="0" t="s">
-        <v>1293</v>
+        <v>1321</v>
       </c>
       <c r="B8" s="36" t="s">
-        <v>1294</v>
+        <v>1322</v>
       </c>
       <c r="C8" s="148" t="n">
         <v>0.8</v>
@@ -26690,27 +27050,27 @@
     </row>
     <row r="9" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="0" t="s">
-        <v>1295</v>
+        <v>1323</v>
       </c>
       <c r="B9" s="0" t="s">
-        <v>1296</v>
-      </c>
-      <c r="C9" s="260" t="n">
+        <v>1324</v>
+      </c>
+      <c r="C9" s="263" t="n">
         <v>30.9318856931226</v>
       </c>
-      <c r="D9" s="260" t="n">
+      <c r="D9" s="263" t="n">
         <v>32.0220208160166</v>
       </c>
-      <c r="E9" s="260" t="n">
+      <c r="E9" s="263" t="n">
         <v>31.2773490371468</v>
       </c>
-      <c r="F9" s="260" t="n">
+      <c r="F9" s="263" t="n">
         <v>31.6168901445216</v>
       </c>
-      <c r="G9" s="260" t="n">
+      <c r="G9" s="263" t="n">
         <v>32.289933097456</v>
       </c>
-      <c r="H9" s="260" t="n">
+      <c r="H9" s="263" t="n">
         <v>30.5392473879664</v>
       </c>
     </row>
@@ -26719,24 +27079,24 @@
         <v>764</v>
       </c>
       <c r="B10" s="0" t="s">
-        <v>1297</v>
-      </c>
-      <c r="C10" s="261" t="n">
+        <v>1325</v>
+      </c>
+      <c r="C10" s="264" t="n">
         <v>55677.3942476206</v>
       </c>
-      <c r="D10" s="261" t="n">
+      <c r="D10" s="264" t="n">
         <v>57639.6374688299</v>
       </c>
-      <c r="E10" s="261" t="n">
+      <c r="E10" s="264" t="n">
         <v>56299.2282668643</v>
       </c>
-      <c r="F10" s="261" t="n">
+      <c r="F10" s="264" t="n">
         <v>56910.4022601389</v>
       </c>
-      <c r="G10" s="261" t="n">
+      <c r="G10" s="264" t="n">
         <v>58121.8795754208</v>
       </c>
-      <c r="H10" s="261" t="n">
+      <c r="H10" s="264" t="n">
         <v>54970.6452983396</v>
       </c>
     </row>
@@ -26745,24 +27105,24 @@
         <v>763</v>
       </c>
       <c r="B11" s="0" t="s">
-        <v>1298</v>
-      </c>
-      <c r="C11" s="261" t="n">
+        <v>1326</v>
+      </c>
+      <c r="C11" s="264" t="n">
         <v>65877.1203514794</v>
       </c>
-      <c r="D11" s="261" t="n">
+      <c r="D11" s="264" t="n">
         <v>67866.546878382</v>
       </c>
-      <c r="E11" s="261" t="n">
+      <c r="E11" s="264" t="n">
         <v>66638.4602735682</v>
       </c>
-      <c r="F11" s="261" t="n">
+      <c r="F11" s="264" t="n">
         <v>67198.4289751488</v>
       </c>
-      <c r="G11" s="261" t="n">
+      <c r="G11" s="264" t="n">
         <v>68308.3952361785</v>
       </c>
-      <c r="H11" s="261" t="n">
+      <c r="H11" s="264" t="n">
         <v>65231.572638484</v>
       </c>
     </row>
@@ -26771,24 +27131,24 @@
         <v>760</v>
       </c>
       <c r="B12" s="0" t="s">
-        <v>1299</v>
-      </c>
-      <c r="C12" s="262" t="n">
+        <v>1327</v>
+      </c>
+      <c r="C12" s="265" t="n">
         <v>0.117703264055937</v>
       </c>
-      <c r="D12" s="262" t="n">
+      <c r="D12" s="265" t="n">
         <v>0.113920331531273</v>
       </c>
-      <c r="E12" s="262" t="n">
+      <c r="E12" s="265" t="n">
         <v>0.113766977325831</v>
       </c>
-      <c r="F12" s="262" t="n">
+      <c r="F12" s="265" t="n">
         <v>0.113837026578705</v>
       </c>
-      <c r="G12" s="262" t="n">
+      <c r="G12" s="265" t="n">
         <v>0.113973014161891</v>
       </c>
-      <c r="H12" s="262" t="n">
+      <c r="H12" s="265" t="n">
         <v>0.117614347074452</v>
       </c>
     </row>
@@ -26797,24 +27157,24 @@
         <v>759</v>
       </c>
       <c r="B13" s="0" t="s">
-        <v>1300</v>
-      </c>
-      <c r="C13" s="262" t="n">
+        <v>1328</v>
+      </c>
+      <c r="C13" s="265" t="n">
         <v>0.140162655262051</v>
       </c>
-      <c r="D13" s="262" t="n">
+      <c r="D13" s="265" t="n">
         <v>0.13343472201868</v>
       </c>
-      <c r="E13" s="262" t="n">
+      <c r="E13" s="265" t="n">
         <v>0.133628639411916</v>
       </c>
-      <c r="F13" s="262" t="n">
+      <c r="F13" s="265" t="n">
         <v>0.133539746416858</v>
       </c>
-      <c r="G13" s="262" t="n">
+      <c r="G13" s="265" t="n">
         <v>0.133368687514593</v>
       </c>
-      <c r="H13" s="262" t="n">
+      <c r="H13" s="265" t="n">
         <v>0.140292132857991</v>
       </c>
     </row>
@@ -26823,7 +27183,7 @@
         <v>758</v>
       </c>
       <c r="B14" s="0" t="s">
-        <v>1301</v>
+        <v>1329</v>
       </c>
       <c r="C14" s="155" t="n">
         <v>1.06365615276715</v>
@@ -26849,24 +27209,24 @@
         <v>761</v>
       </c>
       <c r="B15" s="0" t="s">
-        <v>1302</v>
-      </c>
-      <c r="C15" s="262" t="n">
+        <v>1330</v>
+      </c>
+      <c r="C15" s="265" t="n">
         <v>0.125008009155719</v>
       </c>
-      <c r="D15" s="262" t="n">
+      <c r="D15" s="265" t="n">
         <v>0.120748041823037</v>
       </c>
-      <c r="E15" s="262" t="n">
+      <c r="E15" s="265" t="n">
         <v>0.120748041823037</v>
       </c>
-      <c r="F15" s="262" t="n">
+      <c r="F15" s="265" t="n">
         <v>0.120748041823037</v>
       </c>
-      <c r="G15" s="262" t="n">
+      <c r="G15" s="265" t="n">
         <v>0.120748041823037</v>
       </c>
-      <c r="H15" s="262" t="n">
+      <c r="H15" s="265" t="n">
         <v>0.125008009155719</v>
       </c>
     </row>
@@ -26875,76 +27235,76 @@
         <v>762</v>
       </c>
       <c r="B16" s="0" t="s">
-        <v>1303</v>
-      </c>
-      <c r="C16" s="262" t="n">
+        <v>1331</v>
+      </c>
+      <c r="C16" s="265" t="n">
         <v>0.138293538829152</v>
       </c>
-      <c r="D16" s="262" t="n">
+      <c r="D16" s="265" t="n">
         <v>0.132364052240143</v>
       </c>
-      <c r="E16" s="262" t="n">
+      <c r="E16" s="265" t="n">
         <v>0.132364052240143</v>
       </c>
-      <c r="F16" s="262" t="n">
+      <c r="F16" s="265" t="n">
         <v>0.132364052240143</v>
       </c>
-      <c r="G16" s="262" t="n">
+      <c r="G16" s="265" t="n">
         <v>0.132364052240143</v>
       </c>
-      <c r="H16" s="262" t="n">
+      <c r="H16" s="265" t="n">
         <v>0.138293538829152</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="0" t="s">
-        <v>1304</v>
+        <v>1332</v>
       </c>
       <c r="B17" s="0" t="s">
-        <v>1305</v>
-      </c>
-      <c r="C17" s="261" t="n">
+        <v>1333</v>
+      </c>
+      <c r="C17" s="264" t="n">
         <v>6784.70712387087</v>
       </c>
-      <c r="D17" s="261" t="n">
+      <c r="D17" s="264" t="n">
         <v>6784.70712387087</v>
       </c>
-      <c r="E17" s="261" t="n">
+      <c r="E17" s="264" t="n">
         <v>6636.24176035716</v>
       </c>
-      <c r="F17" s="261" t="n">
+      <c r="F17" s="264" t="n">
         <v>6704.44321602348</v>
       </c>
-      <c r="G17" s="261" t="n">
+      <c r="G17" s="264" t="n">
         <v>6839.71731193936</v>
       </c>
-      <c r="H17" s="261" t="n">
+      <c r="H17" s="264" t="n">
         <v>6704.44321602348</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="0" t="s">
-        <v>1306</v>
+        <v>1334</v>
       </c>
       <c r="B18" s="0" t="s">
-        <v>1307</v>
-      </c>
-      <c r="C18" s="261" t="n">
+        <v>1335</v>
+      </c>
+      <c r="C18" s="264" t="n">
         <v>195901.272736332</v>
       </c>
-      <c r="D18" s="261" t="n">
+      <c r="D18" s="264" t="n">
         <v>195901.272736332</v>
       </c>
-      <c r="E18" s="261" t="n">
+      <c r="E18" s="264" t="n">
         <v>191128.833926638</v>
       </c>
-      <c r="F18" s="261" t="n">
+      <c r="F18" s="264" t="n">
         <v>193343.68292541</v>
       </c>
-      <c r="G18" s="261" t="n">
+      <c r="G18" s="264" t="n">
         <v>197744.187774724</v>
       </c>
-      <c r="H18" s="261" t="n">
+      <c r="H18" s="264" t="n">
         <v>193343.68292541</v>
       </c>
     </row>
@@ -26953,30 +27313,30 @@
         <v>766</v>
       </c>
       <c r="B19" s="36" t="s">
-        <v>1308</v>
-      </c>
-      <c r="C19" s="260" t="n">
+        <v>1336</v>
+      </c>
+      <c r="C19" s="263" t="n">
         <v>32.21236327381</v>
       </c>
-      <c r="D19" s="260" t="n">
+      <c r="D19" s="263" t="n">
         <v>32.757430835257</v>
       </c>
-      <c r="E19" s="260" t="n">
+      <c r="E19" s="263" t="n">
         <v>32.3850949458221</v>
       </c>
-      <c r="F19" s="260" t="n">
+      <c r="F19" s="263" t="n">
         <v>32.5548654995095</v>
       </c>
-      <c r="G19" s="260" t="n">
+      <c r="G19" s="263" t="n">
         <v>32.8913869759767</v>
       </c>
-      <c r="H19" s="260" t="n">
+      <c r="H19" s="263" t="n">
         <v>32.0160441212319</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="150" t="s">
-        <v>1309</v>
+        <v>1337</v>
       </c>
       <c r="B21" s="151"/>
       <c r="C21" s="151"/>
@@ -26992,37 +27352,37 @@
         <v>1128</v>
       </c>
       <c r="B22" s="129" t="s">
-        <v>1310</v>
+        <v>1338</v>
       </c>
       <c r="C22" s="129" t="s">
-        <v>1311</v>
+        <v>1339</v>
       </c>
       <c r="D22" s="129" t="s">
         <v>772</v>
       </c>
       <c r="E22" s="129" t="s">
-        <v>1312</v>
+        <v>1340</v>
       </c>
       <c r="F22" s="129"/>
       <c r="G22" s="129" t="s">
         <v>854</v>
       </c>
       <c r="H22" s="129" t="s">
-        <v>1313</v>
+        <v>1341</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="28.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A23" s="0" t="s">
-        <v>1314</v>
-      </c>
-      <c r="B23" s="263" t="n">
+        <v>1342</v>
+      </c>
+      <c r="B23" s="266" t="n">
         <f aca="false">SUMPRODUCT(ABS('Proyección Final Soriana'!B97:G97))</f>
         <v>0</v>
       </c>
-      <c r="C23" s="263" t="n">
+      <c r="C23" s="266" t="n">
         <v>0</v>
       </c>
-      <c r="D23" s="264" t="n">
+      <c r="D23" s="267" t="n">
         <f aca="false">IF(AND(ISNUMBER(B23),ISNUMBER(C23)),B23-C23,"n/a")</f>
         <v>0</v>
       </c>
@@ -27034,40 +27394,40 @@
         <v>PASS</v>
       </c>
       <c r="H23" s="132" t="s">
-        <v>1315</v>
+        <v>1343</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="42.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A24" s="0" t="s">
-        <v>1316</v>
-      </c>
-      <c r="B24" s="263" t="n">
+        <v>1344</v>
+      </c>
+      <c r="B24" s="266" t="n">
         <f aca="false">'Proyección Final Soriana'!B126-'Proyección Final Soriana'!B123</f>
         <v>0.0788370265787054</v>
       </c>
-      <c r="C24" s="263" t="s">
-        <v>1317</v>
+      <c r="C24" s="266" t="s">
+        <v>1345</v>
       </c>
       <c r="G24" s="156" t="str">
         <f aca="false">IF(B24&gt;0,"PASS","FAIL")</f>
         <v>PASS</v>
       </c>
       <c r="H24" s="132" t="s">
-        <v>1318</v>
+        <v>1346</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="28.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A25" s="0" t="s">
-        <v>1319</v>
-      </c>
-      <c r="B25" s="263" t="n">
+        <v>1347</v>
+      </c>
+      <c r="B25" s="266" t="n">
         <f aca="false">ABS('Proyección Final Soriana'!G219-'Proyección Final Soriana'!G218)</f>
         <v>1.42513331427563E-007</v>
       </c>
-      <c r="C25" s="263" t="n">
+      <c r="C25" s="266" t="n">
         <v>0</v>
       </c>
-      <c r="D25" s="264" t="n">
+      <c r="D25" s="267" t="n">
         <f aca="false">IF(AND(ISNUMBER(B25),ISNUMBER(C25)),B25-C25,"n/a")</f>
         <v>1.42513331427563E-007</v>
       </c>
@@ -27079,22 +27439,22 @@
         <v>PASS</v>
       </c>
       <c r="H25" s="132" t="s">
-        <v>1320</v>
+        <v>1348</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="28.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A26" s="0" t="s">
-        <v>1321</v>
-      </c>
-      <c r="B26" s="263" t="n">
+        <v>1349</v>
+      </c>
+      <c r="B26" s="266" t="n">
         <f aca="false">'Proyección Final Soriana'!B134</f>
         <v>22451.0151511555</v>
       </c>
-      <c r="C26" s="263" t="n">
+      <c r="C26" s="266" t="n">
         <f aca="false">SUMPRODUCT('Proyección Final Soriana'!C117:G117,'Proyección Final Soriana'!C119:G119)</f>
         <v>22451.0151511555</v>
       </c>
-      <c r="D26" s="264" t="n">
+      <c r="D26" s="267" t="n">
         <f aca="false">IF(AND(ISNUMBER(B26),ISNUMBER(C26)),B26-C26,"n/a")</f>
         <v>0</v>
       </c>
@@ -27106,22 +27466,22 @@
         <v>PASS</v>
       </c>
       <c r="H26" s="132" t="s">
-        <v>1322</v>
+        <v>1350</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="28.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A27" s="0" t="s">
-        <v>1323</v>
-      </c>
-      <c r="B27" s="263" t="n">
+        <v>1351</v>
+      </c>
+      <c r="B27" s="266" t="n">
         <f aca="false">'Proyección Final Soriana'!G119</f>
         <v>0.583299690711079</v>
       </c>
-      <c r="C27" s="263" t="n">
+      <c r="C27" s="266" t="n">
         <f aca="false">1/(1+'Proyección Final Soriana'!B126)^5</f>
         <v>0.583299690711079</v>
       </c>
-      <c r="D27" s="264" t="n">
+      <c r="D27" s="267" t="n">
         <f aca="false">IF(AND(ISNUMBER(B27),ISNUMBER(C27)),B27-C27,"n/a")</f>
         <v>0</v>
       </c>
@@ -27133,22 +27493,22 @@
         <v>PASS</v>
       </c>
       <c r="H27" s="132" t="s">
-        <v>1324</v>
+        <v>1352</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="0" t="s">
-        <v>1325</v>
-      </c>
-      <c r="B28" s="263" t="n">
+        <v>1353</v>
+      </c>
+      <c r="B28" s="266" t="n">
         <f aca="false">'Proyección Final Soriana'!B129</f>
         <v>76153.1172746779</v>
       </c>
-      <c r="C28" s="263" t="n">
+      <c r="C28" s="266" t="n">
         <f aca="false">('Proyección Final Soriana'!G73*(1-'Proyección Final Soriana'!G55)+'Proyección Final Soriana'!G116)*(1+'Proyección Final Soriana'!B123)/('Proyección Final Soriana'!B126-'Proyección Final Soriana'!B123)</f>
         <v>76153.1172746779</v>
       </c>
-      <c r="D28" s="264" t="n">
+      <c r="D28" s="267" t="n">
         <f aca="false">IF(AND(ISNUMBER(B28),ISNUMBER(C28)),B28-C28,"n/a")</f>
         <v>0</v>
       </c>
@@ -27160,22 +27520,22 @@
         <v>PASS</v>
       </c>
       <c r="H28" s="132" t="s">
-        <v>1326</v>
+        <v>1354</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="28.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A29" s="0" t="s">
-        <v>1327</v>
-      </c>
-      <c r="B29" s="263" t="n">
+        <v>1355</v>
+      </c>
+      <c r="B29" s="266" t="n">
         <f aca="false">'Proyección Final Soriana'!G117</f>
         <v>6704.44321602348</v>
       </c>
-      <c r="C29" s="263" t="n">
+      <c r="C29" s="266" t="n">
         <f aca="false">'Proyección Final Soriana'!G73*(1-'Proyección Final Soriana'!G55)-'Proyección Final Soriana'!G72+'Proyección Final Soriana'!G104+('Proyección Final Soriana'!G102+'Proyección Final Soriana'!G103+'Proyección Final Soriana'!G105)</f>
         <v>6704.44321602348</v>
       </c>
-      <c r="D29" s="264" t="n">
+      <c r="D29" s="267" t="n">
         <f aca="false">IF(AND(ISNUMBER(B29),ISNUMBER(C29)),B29-C29,"n/a")</f>
         <v>0</v>
       </c>
@@ -27187,22 +27547,22 @@
         <v>PASS</v>
       </c>
       <c r="H29" s="132" t="s">
-        <v>1328</v>
+        <v>1356</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="28.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A30" s="0" t="s">
-        <v>1329</v>
-      </c>
-      <c r="B30" s="263" t="n">
+        <v>1357</v>
+      </c>
+      <c r="B30" s="266" t="n">
         <f aca="false">'Proyección Final Soriana'!B262</f>
         <v>55135.4919486144</v>
       </c>
-      <c r="C30" s="263" t="n">
+      <c r="C30" s="266" t="n">
         <f aca="false">'Proyección Final Soriana'!B258-(Datos!F25+Datos!F26)-(Datos!F27+Datos!F28)+Datos!F17</f>
         <v>55135.4919486144</v>
       </c>
-      <c r="D30" s="264" t="n">
+      <c r="D30" s="267" t="n">
         <f aca="false">IF(AND(ISNUMBER(B30),ISNUMBER(C30)),B30-C30,"n/a")</f>
         <v>0</v>
       </c>
@@ -27214,22 +27574,22 @@
         <v>PASS</v>
       </c>
       <c r="H30" s="132" t="s">
-        <v>1330</v>
+        <v>1358</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="57" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A31" s="0" t="s">
-        <v>1331</v>
-      </c>
-      <c r="B31" s="263" t="n">
+        <v>1359</v>
+      </c>
+      <c r="B31" s="266" t="n">
         <f aca="false">'Proyección Final Soriana'!B257</f>
         <v>1060.497</v>
       </c>
-      <c r="C31" s="263" t="n">
+      <c r="C31" s="266" t="n">
         <f aca="false">-((Datos!E15+Datos!F15)-(Datos!E16+Datos!F16))</f>
         <v>1060.497</v>
       </c>
-      <c r="D31" s="264" t="n">
+      <c r="D31" s="267" t="n">
         <f aca="false">IF(AND(ISNUMBER(B31),ISNUMBER(C31)),B31-C31,"n/a")</f>
         <v>0</v>
       </c>
@@ -27241,22 +27601,22 @@
         <v>PASS</v>
       </c>
       <c r="H31" s="132" t="s">
-        <v>1332</v>
+        <v>1360</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="0" t="s">
-        <v>1333</v>
-      </c>
-      <c r="B32" s="263" t="n">
+        <v>1361</v>
+      </c>
+      <c r="B32" s="266" t="n">
         <f aca="false">'Proyección Final Soriana'!B265</f>
         <v>31.6168901445216</v>
       </c>
-      <c r="C32" s="263" t="n">
+      <c r="C32" s="266" t="n">
         <f aca="false">'Proyección Final Soriana'!B263/WACC!B17</f>
         <v>31.6168901445216</v>
       </c>
-      <c r="D32" s="264" t="n">
+      <c r="D32" s="267" t="n">
         <f aca="false">IF(AND(ISNUMBER(B32),ISNUMBER(C32)),B32-C32,"n/a")</f>
         <v>0</v>
       </c>
@@ -27268,22 +27628,22 @@
         <v>PASS</v>
       </c>
       <c r="H32" s="132" t="s">
-        <v>1334</v>
+        <v>1362</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="72" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A33" s="0" t="s">
-        <v>1335</v>
-      </c>
-      <c r="B33" s="263" t="n">
+        <v>1363</v>
+      </c>
+      <c r="B33" s="266" t="n">
         <f aca="false">'Proyección Final Soriana'!B265</f>
         <v>31.6168901445216</v>
       </c>
-      <c r="C33" s="263" t="n">
+      <c r="C33" s="266" t="n">
         <f aca="false">IF(AND(Inflación!$E$6=0,'Beta y Kd'!$B$18=0),C9,IF(AND(Inflación!$E$6=0,'Beta y Kd'!$B$18=1),D9,IF(AND(Inflación!$E$6=1,'Beta y Kd'!$B$18=1),E9,IF(AND(Inflación!$E$6=2,'Beta y Kd'!$B$18=1),F9,IF(AND(Inflación!$E$6=3,'Beta y Kd'!$B$18=1),G9,IF(AND(Inflación!$E$6=2,'Beta y Kd'!$B$18=0),H9,"sin registro"))))))</f>
         <v>31.6168901445216</v>
       </c>
-      <c r="D33" s="264" t="n">
+      <c r="D33" s="267" t="n">
         <f aca="false">IF(AND(ISNUMBER(B33),ISNUMBER(C33)),B33-C33,"n/a")</f>
         <v>0</v>
       </c>
@@ -27295,21 +27655,21 @@
         <v>PASS</v>
       </c>
       <c r="H33" s="132" t="s">
-        <v>1336</v>
+        <v>1364</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="100.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A34" s="0" t="s">
-        <v>1337</v>
-      </c>
-      <c r="B34" s="263" t="n">
+        <v>1365</v>
+      </c>
+      <c r="B34" s="266" t="n">
         <f aca="false">C9</f>
         <v>30.9318856931226</v>
       </c>
-      <c r="C34" s="263" t="n">
+      <c r="C34" s="266" t="n">
         <v>30.9318856931226</v>
       </c>
-      <c r="D34" s="264" t="n">
+      <c r="D34" s="267" t="n">
         <f aca="false">IF(AND(ISNUMBER(B34),ISNUMBER(C34)),B34-C34,"n/a")</f>
         <v>0</v>
       </c>
@@ -27321,21 +27681,21 @@
         <v>PASS</v>
       </c>
       <c r="H34" s="132" t="s">
-        <v>1338</v>
+        <v>1366</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="100.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A35" s="0" t="s">
-        <v>1339</v>
-      </c>
-      <c r="B35" s="263" t="n">
+        <v>1367</v>
+      </c>
+      <c r="B35" s="266" t="n">
         <f aca="false">IF(AND(E9&lt;F9,F9&lt;G9),1,0)</f>
         <v>1</v>
       </c>
-      <c r="C35" s="263" t="n">
+      <c r="C35" s="266" t="n">
         <v>1</v>
       </c>
-      <c r="D35" s="264" t="n">
+      <c r="D35" s="267" t="n">
         <f aca="false">IF(AND(ISNUMBER(B35),ISNUMBER(C35)),B35-C35,"n/a")</f>
         <v>0</v>
       </c>
@@ -27347,22 +27707,22 @@
         <v>PASS</v>
       </c>
       <c r="H35" s="132" t="s">
-        <v>1340</v>
+        <v>1368</v>
       </c>
     </row>
     <row r="36" customFormat="false" ht="42.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A36" s="0" t="s">
-        <v>1341</v>
-      </c>
-      <c r="B36" s="263" t="n">
+        <v>1369</v>
+      </c>
+      <c r="B36" s="266" t="n">
         <f aca="false">'Beta y Kd'!B14</f>
         <v>0.647803675992488</v>
       </c>
-      <c r="C36" s="263" t="n">
+      <c r="C36" s="266" t="n">
         <f aca="false">'Beta y Kd'!B11</f>
         <v>0.65</v>
       </c>
-      <c r="D36" s="264" t="n">
+      <c r="D36" s="267" t="n">
         <f aca="false">IF(AND(ISNUMBER(B36),ISNUMBER(C36)),B36-C36,"n/a")</f>
         <v>-0.00219632400751191</v>
       </c>
@@ -27374,22 +27734,22 @@
         <v>PASS</v>
       </c>
       <c r="H36" s="132" t="s">
-        <v>1342</v>
+        <v>1370</v>
       </c>
     </row>
     <row r="37" customFormat="false" ht="28.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A37" s="0" t="s">
-        <v>1343</v>
-      </c>
-      <c r="B37" s="263" t="n">
+        <v>1371</v>
+      </c>
+      <c r="B37" s="266" t="n">
         <f aca="false">'Beta y Kd'!B19</f>
         <v>0.69</v>
       </c>
-      <c r="C37" s="263" t="n">
+      <c r="C37" s="266" t="n">
         <f aca="false">IF('Beta y Kd'!$B$18=1,'Beta y Kd'!B13,'Beta y Kd'!B17)</f>
         <v>0.69</v>
       </c>
-      <c r="D37" s="264" t="n">
+      <c r="D37" s="267" t="n">
         <f aca="false">IF(AND(ISNUMBER(B37),ISNUMBER(C37)),B37-C37,"n/a")</f>
         <v>0</v>
       </c>
@@ -27401,22 +27761,22 @@
         <v>PASS</v>
       </c>
       <c r="H37" s="132" t="s">
-        <v>1344</v>
+        <v>1372</v>
       </c>
     </row>
     <row r="38" customFormat="false" ht="57" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A38" s="0" t="s">
-        <v>1345</v>
-      </c>
-      <c r="B38" s="263" t="n">
+        <v>1373</v>
+      </c>
+      <c r="B38" s="266" t="n">
         <f aca="false">WACC!B28</f>
         <v>0.879292015133413</v>
       </c>
-      <c r="C38" s="263" t="n">
+      <c r="C38" s="266" t="n">
         <f aca="false">WACC!B9*(1+(1-WACC!B10)*WACC!B23)</f>
         <v>0.879292015133413</v>
       </c>
-      <c r="D38" s="264" t="n">
+      <c r="D38" s="267" t="n">
         <f aca="false">IF(AND(ISNUMBER(B38),ISNUMBER(C38)),B38-C38,"n/a")</f>
         <v>0</v>
       </c>
@@ -27428,22 +27788,22 @@
         <v>PASS</v>
       </c>
       <c r="H38" s="132" t="s">
-        <v>1346</v>
+        <v>1374</v>
       </c>
     </row>
     <row r="39" customFormat="false" ht="57" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A39" s="0" t="s">
-        <v>1347</v>
-      </c>
-      <c r="B39" s="263" t="n">
+        <v>1375</v>
+      </c>
+      <c r="B39" s="266" t="n">
         <f aca="false">'Proyección Final Soriana'!E219</f>
         <v>0.907086203708222</v>
       </c>
-      <c r="C39" s="263" t="n">
+      <c r="C39" s="266" t="n">
         <f aca="false">'Proyección Final Soriana'!B212*(1+(1-'Proyección Final Soriana'!B207)*'Proyección Final Soriana'!B209/'Proyección Final Soriana'!C219)</f>
         <v>0.907086203708222</v>
       </c>
-      <c r="D39" s="264" t="n">
+      <c r="D39" s="267" t="n">
         <f aca="false">IF(AND(ISNUMBER(B39),ISNUMBER(C39)),B39-C39,"n/a")</f>
         <v>0</v>
       </c>
@@ -27455,22 +27815,22 @@
         <v>PASS</v>
       </c>
       <c r="H39" s="132" t="s">
-        <v>1348</v>
+        <v>1376</v>
       </c>
     </row>
     <row r="40" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A40" s="0" t="s">
-        <v>1349</v>
-      </c>
-      <c r="B40" s="263" t="n">
+        <v>1377</v>
+      </c>
+      <c r="B40" s="266" t="n">
         <f aca="false">'Proyección Final Soriana'!F219</f>
         <v>0.133539746416858</v>
       </c>
-      <c r="C40" s="263" t="n">
+      <c r="C40" s="266" t="n">
         <f aca="false">'Proyección Final Soriana'!B210+'Proyección Final Soriana'!E219*'Proyección Final Soriana'!B211</f>
         <v>0.133539746416858</v>
       </c>
-      <c r="D40" s="264" t="n">
+      <c r="D40" s="267" t="n">
         <f aca="false">IF(AND(ISNUMBER(B40),ISNUMBER(C40)),B40-C40,"n/a")</f>
         <v>0</v>
       </c>
@@ -27482,22 +27842,22 @@
         <v>PASS</v>
       </c>
       <c r="H40" s="132" t="s">
-        <v>1350</v>
+        <v>1378</v>
       </c>
     </row>
     <row r="41" customFormat="false" ht="57" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A41" s="0" t="s">
-        <v>1351</v>
-      </c>
-      <c r="B41" s="263" t="n">
+        <v>1379</v>
+      </c>
+      <c r="B41" s="266" t="n">
         <f aca="false">'Proyección Final Soriana'!C61</f>
         <v>0.1</v>
       </c>
-      <c r="C41" s="263" t="n">
+      <c r="C41" s="266" t="n">
         <f aca="false">(Datos!E10+Datos!F10)*2/Datos!F29</f>
         <v>0.0986484820696688</v>
       </c>
-      <c r="D41" s="264" t="n">
+      <c r="D41" s="267" t="n">
         <f aca="false">IF(AND(ISNUMBER(B41),ISNUMBER(C41)),B41-C41,"n/a")</f>
         <v>0.00135151793033124</v>
       </c>
@@ -27509,21 +27869,21 @@
         <v>PASS</v>
       </c>
       <c r="H41" s="132" t="s">
-        <v>1352</v>
+        <v>1380</v>
       </c>
     </row>
     <row r="42" customFormat="false" ht="42.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A42" s="0" t="s">
-        <v>1353</v>
-      </c>
-      <c r="B42" s="263" t="n">
+        <v>1381</v>
+      </c>
+      <c r="B42" s="266" t="n">
         <f aca="false">SUMPRODUCT(ABS('Proyección Final Soriana'!C10:G10-Inflación!B13:F13))</f>
         <v>0</v>
       </c>
-      <c r="C42" s="263" t="n">
+      <c r="C42" s="266" t="n">
         <v>0</v>
       </c>
-      <c r="D42" s="264" t="n">
+      <c r="D42" s="267" t="n">
         <f aca="false">IF(AND(ISNUMBER(B42),ISNUMBER(C42)),B42-C42,"n/a")</f>
         <v>0</v>
       </c>
@@ -27535,22 +27895,22 @@
         <v>PASS</v>
       </c>
       <c r="H42" s="132" t="s">
-        <v>1354</v>
+        <v>1382</v>
       </c>
     </row>
     <row r="43" customFormat="false" ht="28.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A43" s="0" t="s">
-        <v>1355</v>
-      </c>
-      <c r="B43" s="263" t="n">
+        <v>1383</v>
+      </c>
+      <c r="B43" s="266" t="n">
         <f aca="false">Inflación!B34</f>
         <v>0.0351</v>
       </c>
-      <c r="C43" s="263" t="n">
+      <c r="C43" s="266" t="n">
         <f aca="false">ROUND(Inflación!C21*EXP(Inflación!D21*5),2)/100</f>
         <v>0.0351</v>
       </c>
-      <c r="D43" s="264" t="n">
+      <c r="D43" s="267" t="n">
         <f aca="false">IF(AND(ISNUMBER(B43),ISNUMBER(C43)),B43-C43,"n/a")</f>
         <v>0</v>
       </c>
@@ -27562,21 +27922,21 @@
         <v>PASS</v>
       </c>
       <c r="H43" s="132" t="s">
-        <v>1356</v>
+        <v>1384</v>
       </c>
     </row>
     <row r="44" customFormat="false" ht="42.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A44" s="0" t="s">
-        <v>1357</v>
-      </c>
-      <c r="B44" s="263" t="n">
+        <v>1385</v>
+      </c>
+      <c r="B44" s="266" t="n">
         <f aca="false">Inflación!G21</f>
         <v>0.0350871363974646</v>
       </c>
-      <c r="C44" s="263" t="n">
+      <c r="C44" s="266" t="n">
         <v>0.0351</v>
       </c>
-      <c r="D44" s="264" t="n">
+      <c r="D44" s="267" t="n">
         <f aca="false">IF(AND(ISNUMBER(B44),ISNUMBER(C44)),B44-C44,"n/a")</f>
         <v>-1.2863602535447E-005</v>
       </c>
@@ -27588,21 +27948,21 @@
         <v>PASS</v>
       </c>
       <c r="H44" s="132" t="s">
-        <v>1358</v>
+        <v>1386</v>
       </c>
     </row>
     <row r="45" customFormat="false" ht="28.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A45" s="0" t="s">
-        <v>1359</v>
-      </c>
-      <c r="B45" s="263" t="n">
+        <v>1387</v>
+      </c>
+      <c r="B45" s="266" t="n">
         <f aca="false">Inflación!G20</f>
         <v>0.0350405233912861</v>
       </c>
-      <c r="C45" s="263" t="n">
+      <c r="C45" s="266" t="n">
         <v>0.0350807936283421</v>
       </c>
-      <c r="D45" s="264" t="n">
+      <c r="D45" s="267" t="n">
         <f aca="false">IF(AND(ISNUMBER(B45),ISNUMBER(C45)),B45-C45,"n/a")</f>
         <v>-4.02702370559671E-005</v>
       </c>
@@ -27614,21 +27974,21 @@
         <v>PASS</v>
       </c>
       <c r="H45" s="132" t="s">
-        <v>1360</v>
+        <v>1388</v>
       </c>
     </row>
     <row r="46" customFormat="false" ht="28.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A46" s="0" t="s">
-        <v>1361</v>
-      </c>
-      <c r="B46" s="263" t="n">
+        <v>1389</v>
+      </c>
+      <c r="B46" s="266" t="n">
         <f aca="false">Inflación!G24</f>
         <v>0.0326787650364365</v>
       </c>
-      <c r="C46" s="263" t="n">
+      <c r="C46" s="266" t="n">
         <v>0.0326787671112565</v>
       </c>
-      <c r="D46" s="264" t="n">
+      <c r="D46" s="267" t="n">
         <f aca="false">IF(AND(ISNUMBER(B46),ISNUMBER(C46)),B46-C46,"n/a")</f>
         <v>-2.07481998942827E-009</v>
       </c>
@@ -27640,21 +28000,21 @@
         <v>PASS</v>
       </c>
       <c r="H46" s="132" t="s">
-        <v>1362</v>
+        <v>1390</v>
       </c>
     </row>
     <row r="47" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A47" s="0" t="s">
-        <v>1363</v>
-      </c>
-      <c r="B47" s="263" t="n">
+        <v>1391</v>
+      </c>
+      <c r="B47" s="266" t="n">
         <f aca="false">VF_BETA_HISTORICA</f>
         <v>0.0414619566109314</v>
       </c>
-      <c r="C47" s="263" t="n">
+      <c r="C47" s="266" t="n">
         <v>0.0414619566109315</v>
       </c>
-      <c r="D47" s="264" t="n">
+      <c r="D47" s="267" t="n">
         <f aca="false">IF(AND(ISNUMBER(B47),ISNUMBER(C47)),B47-C47,"n/a")</f>
         <v>0</v>
       </c>
@@ -27666,21 +28026,21 @@
         <v>PASS</v>
       </c>
       <c r="H47" s="132" t="s">
-        <v>1364</v>
+        <v>1392</v>
       </c>
     </row>
     <row r="48" customFormat="false" ht="172.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A48" s="0" t="s">
-        <v>1365</v>
-      </c>
-      <c r="B48" s="263" t="n">
+        <v>1393</v>
+      </c>
+      <c r="B48" s="266" t="n">
         <f aca="false">COUNT(Multiplos!N5:N14)+COUNT(Multiplos!P5:P14)</f>
         <v>20</v>
       </c>
-      <c r="C48" s="263" t="n">
+      <c r="C48" s="266" t="n">
         <v>20</v>
       </c>
-      <c r="D48" s="264" t="n">
+      <c r="D48" s="267" t="n">
         <f aca="false">IF(AND(ISNUMBER(B48),ISNUMBER(C48)),B48-C48,"n/a")</f>
         <v>0</v>
       </c>
@@ -27692,22 +28052,22 @@
         <v>PASS</v>
       </c>
       <c r="H48" s="132" t="s">
-        <v>1366</v>
+        <v>1394</v>
       </c>
     </row>
     <row r="49" customFormat="false" ht="72" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A49" s="0" t="s">
-        <v>1367</v>
-      </c>
-      <c r="B49" s="263" t="n">
+        <v>1395</v>
+      </c>
+      <c r="B49" s="266" t="n">
         <f aca="false">Multiplos!E60</f>
         <v>14.5142857142857</v>
       </c>
-      <c r="C49" s="263" t="n">
+      <c r="C49" s="266" t="n">
         <f aca="false">SUMPRODUCT(Multiplos!P5:P14,Multiplos!K5:K14)/SUM(Multiplos!K5:K14)</f>
         <v>14.5142857142857</v>
       </c>
-      <c r="D49" s="264" t="n">
+      <c r="D49" s="267" t="n">
         <f aca="false">IF(AND(ISNUMBER(B49),ISNUMBER(C49)),B49-C49,"n/a")</f>
         <v>0</v>
       </c>
@@ -27719,22 +28079,22 @@
         <v>PASS</v>
       </c>
       <c r="H49" s="132" t="s">
-        <v>1368</v>
+        <v>1396</v>
       </c>
     </row>
     <row r="50" customFormat="false" ht="42.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A50" s="0" t="s">
-        <v>1369</v>
-      </c>
-      <c r="B50" s="263" t="n">
+        <v>1397</v>
+      </c>
+      <c r="B50" s="266" t="n">
         <f aca="false">Multiplos!C60</f>
         <v>7.04285714285714</v>
       </c>
-      <c r="C50" s="263" t="n">
+      <c r="C50" s="266" t="n">
         <f aca="false">SUMPRODUCT(Multiplos!N5:N14,Multiplos!K5:K14)/SUM(Multiplos!K5:K14)</f>
         <v>7.04285714285714</v>
       </c>
-      <c r="D50" s="264" t="n">
+      <c r="D50" s="267" t="n">
         <f aca="false">IF(AND(ISNUMBER(B50),ISNUMBER(C50)),B50-C50,"n/a")</f>
         <v>0</v>
       </c>
@@ -27746,22 +28106,22 @@
         <v>PASS</v>
       </c>
       <c r="H50" s="132" t="s">
-        <v>1370</v>
+        <v>1398</v>
       </c>
     </row>
     <row r="51" customFormat="false" ht="42.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A51" s="0" t="s">
-        <v>1371</v>
-      </c>
-      <c r="B51" s="263" t="n">
+        <v>1399</v>
+      </c>
+      <c r="B51" s="266" t="n">
         <f aca="false">Multiplos!H60</f>
         <v>36.853929547619</v>
       </c>
-      <c r="C51" s="263" t="n">
+      <c r="C51" s="266" t="n">
         <f aca="false">(Multiplos!C60*Multiplos!B21+Multiplos!B30)/Multiplos!B23</f>
         <v>36.853929547619</v>
       </c>
-      <c r="D51" s="264" t="n">
+      <c r="D51" s="267" t="n">
         <f aca="false">IF(AND(ISNUMBER(B51),ISNUMBER(C51)),B51-C51,"n/a")</f>
         <v>0</v>
       </c>
@@ -27773,22 +28133,22 @@
         <v>PASS</v>
       </c>
       <c r="H51" s="132" t="s">
-        <v>1372</v>
+        <v>1400</v>
       </c>
     </row>
     <row r="52" customFormat="false" ht="42.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A52" s="0" t="s">
-        <v>1373</v>
-      </c>
-      <c r="B52" s="263" t="n">
+        <v>1401</v>
+      </c>
+      <c r="B52" s="266" t="n">
         <f aca="false">Multiplos!D73</f>
         <v>33.4928408544974</v>
       </c>
-      <c r="C52" s="263" t="n">
+      <c r="C52" s="266" t="n">
         <f aca="false">AVERAGE(Multiplos!H60:J60)</f>
         <v>33.4928408544974</v>
       </c>
-      <c r="D52" s="264" t="n">
+      <c r="D52" s="267" t="n">
         <f aca="false">IF(AND(ISNUMBER(B52),ISNUMBER(C52)),B52-C52,"n/a")</f>
         <v>0</v>
       </c>
@@ -27800,21 +28160,21 @@
         <v>PASS</v>
       </c>
       <c r="H52" s="132" t="s">
-        <v>1374</v>
+        <v>1402</v>
       </c>
     </row>
     <row r="53" customFormat="false" ht="28.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A53" s="0" t="s">
-        <v>1375</v>
-      </c>
-      <c r="B53" s="263" t="n">
+        <v>1403</v>
+      </c>
+      <c r="B53" s="266" t="n">
         <f aca="false">Multiplos!C64</f>
         <v>7</v>
       </c>
-      <c r="C53" s="263" t="n">
+      <c r="C53" s="266" t="n">
         <v>7</v>
       </c>
-      <c r="D53" s="264" t="n">
+      <c r="D53" s="267" t="n">
         <f aca="false">IF(AND(ISNUMBER(B53),ISNUMBER(C53)),B53-C53,"n/a")</f>
         <v>0</v>
       </c>
@@ -27826,22 +28186,22 @@
         <v>PASS</v>
       </c>
       <c r="H53" s="132" t="s">
-        <v>1376</v>
+        <v>1404</v>
       </c>
     </row>
     <row r="54" customFormat="false" ht="28.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A54" s="0" t="s">
-        <v>1377</v>
-      </c>
-      <c r="B54" s="263" t="n">
+        <v>1405</v>
+      </c>
+      <c r="B54" s="266" t="n">
         <f aca="false">Transacciones!C30</f>
         <v>7.63333333333333</v>
       </c>
-      <c r="C54" s="263" t="n">
+      <c r="C54" s="266" t="n">
         <f aca="false">Transacciones!I15</f>
         <v>7.6</v>
       </c>
-      <c r="D54" s="264" t="n">
+      <c r="D54" s="267" t="n">
         <f aca="false">IF(AND(ISNUMBER(B54),ISNUMBER(C54)),B54-C54,"n/a")</f>
         <v>0.0333333333333332</v>
       </c>
@@ -27853,22 +28213,22 @@
         <v>PASS</v>
       </c>
       <c r="H54" s="132" t="s">
-        <v>1378</v>
+        <v>1406</v>
       </c>
     </row>
     <row r="55" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A55" s="0" t="s">
-        <v>1379</v>
-      </c>
-      <c r="B55" s="263" t="n">
+        <v>1407</v>
+      </c>
+      <c r="B55" s="266" t="n">
         <f aca="false">Transacciones!B30</f>
         <v>0.733333333333333</v>
       </c>
-      <c r="C55" s="263" t="n">
+      <c r="C55" s="266" t="n">
         <f aca="false">Transacciones!H15</f>
         <v>0.7</v>
       </c>
-      <c r="D55" s="264" t="n">
+      <c r="D55" s="267" t="n">
         <f aca="false">IF(AND(ISNUMBER(B55),ISNUMBER(C55)),B55-C55,"n/a")</f>
         <v>0.0333333333333334</v>
       </c>
@@ -27880,21 +28240,21 @@
         <v>PASS</v>
       </c>
       <c r="H55" s="132" t="s">
-        <v>1380</v>
+        <v>1408</v>
       </c>
     </row>
     <row r="56" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A56" s="0" t="s">
-        <v>1381</v>
-      </c>
-      <c r="B56" s="263" t="n">
+        <v>1409</v>
+      </c>
+      <c r="B56" s="266" t="n">
         <f aca="false">'Valuación Combinada'!C7</f>
         <v>1</v>
       </c>
-      <c r="C56" s="263" t="n">
+      <c r="C56" s="266" t="n">
         <v>1</v>
       </c>
-      <c r="D56" s="264" t="n">
+      <c r="D56" s="267" t="n">
         <f aca="false">IF(AND(ISNUMBER(B56),ISNUMBER(C56)),B56-C56,"n/a")</f>
         <v>0</v>
       </c>
@@ -27906,22 +28266,22 @@
         <v>PASS</v>
       </c>
       <c r="H56" s="132" t="s">
-        <v>1382</v>
+        <v>1410</v>
       </c>
     </row>
     <row r="57" customFormat="false" ht="42.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A57" s="0" t="s">
-        <v>1383</v>
-      </c>
-      <c r="B57" s="263" t="n">
+        <v>1411</v>
+      </c>
+      <c r="B57" s="266" t="n">
         <f aca="false">'Valuación Combinada'!B9</f>
         <v>32.5548654995095</v>
       </c>
-      <c r="C57" s="263" t="n">
+      <c r="C57" s="266" t="n">
         <f aca="false">'Valuación Combinada'!B4*'Valuación Combinada'!C4+'Valuación Combinada'!B5*'Valuación Combinada'!C5+IF(ISNUMBER('Valuación Combinada'!B6),'Valuación Combinada'!B6*'Valuación Combinada'!C6,0)</f>
         <v>32.5548654995095</v>
       </c>
-      <c r="D57" s="264" t="n">
+      <c r="D57" s="267" t="n">
         <f aca="false">IF(AND(ISNUMBER(B57),ISNUMBER(C57)),B57-C57,"n/a")</f>
         <v>0</v>
       </c>
@@ -27933,22 +28293,22 @@
         <v>PASS</v>
       </c>
       <c r="H57" s="132" t="s">
-        <v>1384</v>
+        <v>1412</v>
       </c>
     </row>
     <row r="58" customFormat="false" ht="42.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A58" s="0" t="s">
-        <v>1385</v>
-      </c>
-      <c r="B58" s="263" t="n">
+        <v>1413</v>
+      </c>
+      <c r="B58" s="266" t="n">
         <f aca="false">Transacciones!E30</f>
         <v>40.7283951666667</v>
       </c>
-      <c r="C58" s="263" t="n">
+      <c r="C58" s="266" t="n">
         <f aca="false">(Transacciones!C30*Multiplos!B21+Multiplos!B30)/Multiplos!B23</f>
         <v>40.7283951666667</v>
       </c>
-      <c r="D58" s="264" t="n">
+      <c r="D58" s="267" t="n">
         <f aca="false">IF(AND(ISNUMBER(B58),ISNUMBER(C58)),B58-C58,"n/a")</f>
         <v>0</v>
       </c>
@@ -27960,22 +28320,22 @@
         <v>PASS</v>
       </c>
       <c r="H58" s="132" t="s">
-        <v>1386</v>
+        <v>1414</v>
       </c>
     </row>
     <row r="59" customFormat="false" ht="28.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A59" s="0" t="s">
-        <v>1387</v>
-      </c>
-      <c r="B59" s="263" t="n">
+        <v>1415</v>
+      </c>
+      <c r="B59" s="266" t="n">
         <f aca="false">Transacciones!C41</f>
         <v>73311.1113</v>
       </c>
-      <c r="C59" s="263" t="n">
+      <c r="C59" s="266" t="n">
         <f aca="false">Transacciones!C39+Multiplos!B30</f>
         <v>73311.1113</v>
       </c>
-      <c r="D59" s="264" t="n">
+      <c r="D59" s="267" t="n">
         <f aca="false">IF(AND(ISNUMBER(B59),ISNUMBER(C59)),B59-C59,"n/a")</f>
         <v>0</v>
       </c>
@@ -27987,22 +28347,22 @@
         <v>PASS</v>
       </c>
       <c r="H59" s="132" t="s">
-        <v>1388</v>
+        <v>1416</v>
       </c>
     </row>
     <row r="60" customFormat="false" ht="28.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A60" s="0" t="s">
-        <v>1389</v>
-      </c>
-      <c r="B60" s="263" t="n">
+        <v>1417</v>
+      </c>
+      <c r="B60" s="266" t="n">
         <f aca="false">Multiplos!C69</f>
         <v>66337.0731857143</v>
       </c>
-      <c r="C60" s="263" t="n">
+      <c r="C60" s="266" t="n">
         <f aca="false">Multiplos!C68+Multiplos!B30</f>
         <v>66337.0731857143</v>
       </c>
-      <c r="D60" s="264" t="n">
+      <c r="D60" s="267" t="n">
         <f aca="false">IF(AND(ISNUMBER(B60),ISNUMBER(C60)),B60-C60,"n/a")</f>
         <v>0</v>
       </c>
@@ -28014,21 +28374,21 @@
         <v>PASS</v>
       </c>
       <c r="H60" s="132" t="s">
-        <v>1388</v>
+        <v>1416</v>
       </c>
     </row>
     <row r="61" customFormat="false" ht="28.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A61" s="0" t="s">
-        <v>1390</v>
-      </c>
-      <c r="B61" s="263" t="n">
+        <v>1418</v>
+      </c>
+      <c r="B61" s="266" t="n">
         <f aca="false">'Valuación Combinada'!C6</f>
         <v>0</v>
       </c>
-      <c r="C61" s="263" t="n">
+      <c r="C61" s="266" t="n">
         <v>0</v>
       </c>
-      <c r="D61" s="264" t="n">
+      <c r="D61" s="267" t="n">
         <f aca="false">IF(AND(ISNUMBER(B61),ISNUMBER(C61)),B61-C61,"n/a")</f>
         <v>0</v>
       </c>
@@ -28040,12 +28400,12 @@
         <v>PASS</v>
       </c>
       <c r="H61" s="132" t="s">
-        <v>1391</v>
+        <v>1419</v>
       </c>
     </row>
     <row r="62" customFormat="false" ht="201" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A62" s="0" t="s">
-        <v>1392</v>
+        <v>1420</v>
       </c>
       <c r="B62" s="251" t="n">
         <f aca="false">'Transacciones SDC'!C56</f>
@@ -28055,7 +28415,7 @@
         <f aca="false">SUMPRODUCT(('Transacciones SDC'!AB23:AB45=1)*ISNUMBER('Transacciones SDC'!N23:N45))</f>
         <v>8</v>
       </c>
-      <c r="D62" s="265" t="n">
+      <c r="D62" s="268" t="n">
         <f aca="false">IF(AND(ISNUMBER(B62),ISNUMBER(C62)),B62-C62,"n/a")</f>
         <v>0</v>
       </c>
@@ -28067,14 +28427,14 @@
         <v>PASS</v>
       </c>
       <c r="H62" s="132" t="s">
-        <v>1393</v>
+        <v>1421</v>
       </c>
     </row>
     <row r="63" customFormat="false" ht="100.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A63" s="156" t="s">
-        <v>1394</v>
-      </c>
-      <c r="B63" s="266" t="n">
+        <v>1422</v>
+      </c>
+      <c r="B63" s="269" t="n">
         <f aca="false">'Transacciones SDC'!C52</f>
         <v>7.7775</v>
       </c>
@@ -28094,12 +28454,12 @@
         <v>PASS</v>
       </c>
       <c r="H63" s="132" t="s">
-        <v>1395</v>
+        <v>1423</v>
       </c>
     </row>
     <row r="64" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A64" s="0" t="s">
-        <v>1396</v>
+        <v>1424</v>
       </c>
       <c r="B64" s="251" t="n">
         <f aca="false">'Transacciones SDC'!C53</f>
@@ -28121,12 +28481,12 @@
         <v>PASS</v>
       </c>
       <c r="H64" s="36" t="s">
-        <v>1397</v>
+        <v>1425</v>
       </c>
     </row>
     <row r="65" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A65" s="0" t="s">
-        <v>1398</v>
+        <v>1426</v>
       </c>
       <c r="B65" s="0" t="n">
         <f aca="false">SUMPRODUCT(('Transacciones SDC'!AB23:AB45=1)*('Transacciones SDC'!T23:T45&lt;'Transacciones SDC'!$C$9))</f>
@@ -28147,12 +28507,12 @@
         <v>PASS</v>
       </c>
       <c r="H65" s="0" t="s">
-        <v>1399</v>
+        <v>1427</v>
       </c>
     </row>
     <row r="66" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A66" s="0" t="s">
-        <v>1400</v>
+        <v>1428</v>
       </c>
       <c r="B66" s="0" t="n">
         <f aca="false">SUMPRODUCT(('Transacciones SDC'!AB23:AB45=1)*(('Transacciones SDC'!B23:B45&lt;'Transacciones SDC'!$C$8)+('Transacciones SDC'!B23:B45&gt;'Transacciones SDC'!$C$6)))</f>
@@ -28173,12 +28533,12 @@
         <v>PASS</v>
       </c>
       <c r="H66" s="0" t="s">
-        <v>1401</v>
+        <v>1429</v>
       </c>
     </row>
     <row r="67" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A67" s="0" t="s">
-        <v>1402</v>
+        <v>1430</v>
       </c>
       <c r="B67" s="0" t="n">
         <f aca="false">SUMPRODUCT(('Transacciones SDC'!AB23:AB45=1)*('Transacciones SDC'!X23:X45="Sí"))</f>
@@ -28199,12 +28559,12 @@
         <v>PASS</v>
       </c>
       <c r="H67" s="0" t="s">
-        <v>1403</v>
+        <v>1431</v>
       </c>
     </row>
     <row r="68" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A68" s="0" t="s">
-        <v>1404</v>
+        <v>1432</v>
       </c>
       <c r="B68" s="0" t="n">
         <f aca="false">COUNTIF('Transacciones SDC'!AE23:AE45,0)+COUNTIF('Transacciones SDC'!AF23:AF45,0)</f>
@@ -28225,12 +28585,12 @@
         <v>PASS</v>
       </c>
       <c r="H68" s="0" t="s">
-        <v>1405</v>
+        <v>1433</v>
       </c>
     </row>
     <row r="69" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A69" s="0" t="s">
-        <v>1406</v>
+        <v>1434</v>
       </c>
       <c r="B69" s="252" t="n">
         <f aca="false">'Transacciones SDC'!F53</f>
@@ -28252,14 +28612,14 @@
         <v>PASS</v>
       </c>
       <c r="H69" s="36" t="s">
-        <v>1407</v>
+        <v>1435</v>
       </c>
     </row>
     <row r="70" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A70" s="0" t="s">
-        <v>1408</v>
-      </c>
-      <c r="B70" s="267" t="n">
+        <v>1436</v>
+      </c>
+      <c r="B70" s="270" t="n">
         <f aca="false">'Valuación Combinada'!B6</f>
         <v>23.7448001083333</v>
       </c>
@@ -28279,18 +28639,18 @@
         <v>PASS</v>
       </c>
       <c r="H70" s="36" t="s">
-        <v>1409</v>
+        <v>1437</v>
       </c>
     </row>
     <row r="71" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A71" s="0" t="s">
-        <v>1410</v>
+        <v>1438</v>
       </c>
       <c r="B71" s="121" t="n">
         <f aca="false">'Proyección Final Soriana'!D277</f>
         <v>31.6168901445216</v>
       </c>
-      <c r="C71" s="268" t="n">
+      <c r="C71" s="271" t="n">
         <f aca="false">'Proyección Final Soriana'!B265</f>
         <v>31.6168901445216</v>
       </c>
@@ -28306,14 +28666,14 @@
         <v>PASS</v>
       </c>
       <c r="H71" s="36" t="s">
-        <v>1411</v>
+        <v>1439</v>
       </c>
     </row>
     <row r="73" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A73" s="0" t="s">
-        <v>1412</v>
-      </c>
-      <c r="B73" s="269" t="n">
+        <v>1440</v>
+      </c>
+      <c r="B73" s="272" t="n">
         <f aca="false">Multiplos!C60</f>
         <v>7.04285714285714</v>
       </c>
@@ -28329,19 +28689,19 @@
         <v>RAZONABLE</v>
       </c>
       <c r="H73" s="36" t="s">
-        <v>1413</v>
+        <v>1441</v>
       </c>
     </row>
     <row r="74" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A74" s="119" t="s">
-        <v>1414</v>
+        <v>1442</v>
       </c>
       <c r="B74" s="0" t="str">
         <f aca="false">COUNTIF(G23:G71,"PASS")&amp;" PASS de "&amp;COUNTA(A23:A71)</f>
         <v>49 PASS de 49</v>
       </c>
       <c r="H74" s="36" t="s">
-        <v>1415</v>
+        <v>1443</v>
       </c>
     </row>
   </sheetData>
@@ -28374,25 +28734,25 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="122" t="s">
-        <v>1416</v>
+        <v>1444</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="123" t="s">
-        <v>1417</v>
+        <v>1445</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="123" t="s">
-        <v>1281</v>
+        <v>1309</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="129" t="s">
-        <v>1418</v>
+        <v>1446</v>
       </c>
       <c r="B5" s="129" t="s">
-        <v>1419</v>
+        <v>1447</v>
       </c>
       <c r="C5" s="129" t="s">
         <v>78</v>
@@ -28401,7 +28761,7 @@
         <v>60</v>
       </c>
       <c r="E5" s="129" t="s">
-        <v>1420</v>
+        <v>1448</v>
       </c>
       <c r="F5" s="129" t="s">
         <v>851</v>
@@ -28412,209 +28772,209 @@
     </row>
     <row r="6" customFormat="false" ht="28.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="132" t="s">
-        <v>1421</v>
+        <v>1449</v>
       </c>
       <c r="B6" s="132" t="s">
-        <v>1422</v>
+        <v>1450</v>
       </c>
       <c r="C6" s="132" t="s">
-        <v>1423</v>
+        <v>1451</v>
       </c>
       <c r="D6" s="132" t="s">
-        <v>1223</v>
+        <v>1251</v>
       </c>
       <c r="E6" s="132" t="s">
-        <v>1424</v>
+        <v>1452</v>
       </c>
       <c r="F6" s="132" t="s">
-        <v>1425</v>
+        <v>1453</v>
       </c>
       <c r="G6" s="132" t="s">
-        <v>1426</v>
+        <v>1454</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="132" t="s">
-        <v>1427</v>
+        <v>1455</v>
       </c>
       <c r="B7" s="132" t="s">
-        <v>1428</v>
+        <v>1456</v>
       </c>
       <c r="C7" s="132" t="s">
-        <v>1429</v>
+        <v>1457</v>
       </c>
       <c r="D7" s="132" t="s">
-        <v>1223</v>
+        <v>1251</v>
       </c>
       <c r="E7" s="132" t="s">
-        <v>1424</v>
+        <v>1452</v>
       </c>
       <c r="F7" s="132" t="s">
         <v>661</v>
       </c>
       <c r="G7" s="132" t="s">
-        <v>1430</v>
+        <v>1458</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="28.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="132" t="s">
-        <v>1431</v>
+        <v>1459</v>
       </c>
       <c r="B8" s="132" t="s">
-        <v>1432</v>
+        <v>1460</v>
       </c>
       <c r="C8" s="132" t="s">
-        <v>1433</v>
+        <v>1461</v>
       </c>
       <c r="D8" s="132" t="s">
-        <v>1223</v>
+        <v>1251</v>
       </c>
       <c r="E8" s="132" t="s">
-        <v>1424</v>
+        <v>1452</v>
       </c>
       <c r="F8" s="132" t="s">
-        <v>1434</v>
+        <v>1462</v>
       </c>
       <c r="G8" s="132" t="s">
-        <v>1435</v>
+        <v>1463</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="28.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="132" t="s">
-        <v>1436</v>
+        <v>1464</v>
       </c>
       <c r="B9" s="132" t="s">
-        <v>1437</v>
+        <v>1465</v>
       </c>
       <c r="C9" s="132" t="s">
-        <v>1438</v>
+        <v>1466</v>
       </c>
       <c r="D9" s="132" t="s">
         <v>587</v>
       </c>
       <c r="E9" s="132" t="s">
-        <v>1424</v>
+        <v>1452</v>
       </c>
       <c r="F9" s="132" t="s">
-        <v>1434</v>
+        <v>1462</v>
       </c>
       <c r="G9" s="132" t="s">
-        <v>1439</v>
+        <v>1467</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="28.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="132" t="s">
-        <v>1440</v>
+        <v>1468</v>
       </c>
       <c r="B10" s="132" t="s">
-        <v>1441</v>
+        <v>1469</v>
       </c>
       <c r="C10" s="132" t="s">
-        <v>1442</v>
+        <v>1470</v>
       </c>
       <c r="D10" s="132" t="s">
-        <v>1443</v>
+        <v>1471</v>
       </c>
       <c r="E10" s="132" t="s">
-        <v>1424</v>
+        <v>1452</v>
       </c>
       <c r="F10" s="132" t="s">
-        <v>1444</v>
+        <v>1472</v>
       </c>
       <c r="G10" s="132" t="s">
-        <v>1445</v>
+        <v>1473</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="72" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A11" s="132" t="s">
-        <v>1446</v>
+        <v>1474</v>
       </c>
       <c r="B11" s="132" t="s">
-        <v>1447</v>
+        <v>1475</v>
       </c>
       <c r="C11" s="132" t="n">
         <v>0.69</v>
       </c>
       <c r="D11" s="132" t="s">
-        <v>1448</v>
+        <v>1476</v>
       </c>
       <c r="E11" s="132" t="s">
-        <v>1449</v>
+        <v>1477</v>
       </c>
       <c r="F11" s="132" t="s">
-        <v>1425</v>
+        <v>1453</v>
       </c>
       <c r="G11" s="132" t="s">
-        <v>1450</v>
+        <v>1478</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="132" t="s">
-        <v>1451</v>
+        <v>1479</v>
       </c>
       <c r="B12" s="132" t="s">
-        <v>1452</v>
+        <v>1480</v>
       </c>
       <c r="C12" s="132" t="s">
-        <v>1453</v>
+        <v>1481</v>
       </c>
       <c r="D12" s="132" t="s">
         <v>587</v>
       </c>
       <c r="E12" s="132" t="s">
-        <v>1449</v>
+        <v>1477</v>
       </c>
       <c r="F12" s="132" t="s">
-        <v>1444</v>
+        <v>1472</v>
       </c>
       <c r="G12" s="132" t="s">
-        <v>1454</v>
+        <v>1482</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="42.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A13" s="132" t="s">
-        <v>1455</v>
+        <v>1483</v>
       </c>
       <c r="B13" s="132" t="s">
-        <v>1456</v>
+        <v>1484</v>
       </c>
       <c r="C13" s="132" t="s">
-        <v>1457</v>
+        <v>1485</v>
       </c>
       <c r="D13" s="132" t="s">
-        <v>1443</v>
+        <v>1471</v>
       </c>
       <c r="E13" s="132" t="s">
-        <v>1458</v>
+        <v>1486</v>
       </c>
       <c r="F13" s="132" t="s">
-        <v>1434</v>
+        <v>1462</v>
       </c>
       <c r="G13" s="132" t="s">
-        <v>1459</v>
+        <v>1487</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="57" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A14" s="132" t="s">
-        <v>1460</v>
+        <v>1488</v>
       </c>
       <c r="B14" s="132" t="s">
-        <v>1461</v>
+        <v>1489</v>
       </c>
       <c r="C14" s="132" t="s">
-        <v>1462</v>
-      </c>
-      <c r="D14" s="270" t="s">
-        <v>1197</v>
+        <v>1490</v>
+      </c>
+      <c r="D14" s="273" t="s">
+        <v>1225</v>
       </c>
       <c r="E14" s="132" t="s">
-        <v>1424</v>
+        <v>1452</v>
       </c>
       <c r="F14" s="132" t="s">
-        <v>1425</v>
+        <v>1453</v>
       </c>
       <c r="G14" s="132" t="s">
-        <v>1463</v>
+        <v>1491</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="57" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -28622,252 +28982,252 @@
         <v>747</v>
       </c>
       <c r="B15" s="132" t="s">
-        <v>1464</v>
+        <v>1492</v>
       </c>
       <c r="C15" s="132" t="s">
-        <v>1465</v>
+        <v>1493</v>
       </c>
       <c r="D15" s="132" t="s">
-        <v>1448</v>
+        <v>1476</v>
       </c>
       <c r="E15" s="132" t="s">
-        <v>1424</v>
+        <v>1452</v>
       </c>
       <c r="F15" s="132" t="s">
-        <v>1425</v>
+        <v>1453</v>
       </c>
       <c r="G15" s="132" t="s">
-        <v>1466</v>
+        <v>1494</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="57" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A16" s="132" t="s">
-        <v>1467</v>
+        <v>1495</v>
       </c>
       <c r="B16" s="132" t="s">
-        <v>1468</v>
+        <v>1496</v>
       </c>
       <c r="C16" s="132" t="s">
-        <v>1469</v>
-      </c>
-      <c r="D16" s="271" t="s">
-        <v>1470</v>
+        <v>1497</v>
+      </c>
+      <c r="D16" s="274" t="s">
+        <v>1498</v>
       </c>
       <c r="E16" s="132" t="s">
-        <v>1424</v>
+        <v>1452</v>
       </c>
       <c r="F16" s="132" t="s">
-        <v>1434</v>
+        <v>1462</v>
       </c>
       <c r="G16" s="132" t="s">
-        <v>1471</v>
+        <v>1499</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="132" t="s">
-        <v>1472</v>
+        <v>1500</v>
       </c>
       <c r="B17" s="132" t="s">
         <v>958</v>
       </c>
       <c r="C17" s="132" t="s">
-        <v>1473</v>
+        <v>1501</v>
       </c>
       <c r="D17" s="132" t="s">
-        <v>1203</v>
+        <v>1231</v>
       </c>
       <c r="E17" s="132" t="s">
-        <v>1449</v>
+        <v>1477</v>
       </c>
       <c r="F17" s="132" t="s">
-        <v>1425</v>
+        <v>1453</v>
       </c>
       <c r="G17" s="132" t="s">
-        <v>1474</v>
+        <v>1502</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="132" t="s">
-        <v>1475</v>
+        <v>1503</v>
       </c>
       <c r="B18" s="132" t="s">
-        <v>1476</v>
+        <v>1504</v>
       </c>
       <c r="C18" s="132" t="s">
-        <v>1477</v>
+        <v>1505</v>
       </c>
       <c r="D18" s="132" t="s">
         <v>587</v>
       </c>
       <c r="E18" s="132" t="s">
-        <v>1478</v>
+        <v>1506</v>
       </c>
       <c r="F18" s="132" t="s">
-        <v>1425</v>
+        <v>1453</v>
       </c>
       <c r="G18" s="132" t="s">
-        <v>1479</v>
+        <v>1507</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="132" t="s">
-        <v>1480</v>
+        <v>1508</v>
       </c>
       <c r="B19" s="132" t="s">
-        <v>1481</v>
+        <v>1509</v>
       </c>
       <c r="C19" s="132" t="s">
-        <v>1482</v>
+        <v>1510</v>
       </c>
       <c r="D19" s="132" t="s">
-        <v>1203</v>
+        <v>1231</v>
       </c>
       <c r="E19" s="132" t="s">
-        <v>1483</v>
+        <v>1511</v>
       </c>
       <c r="F19" s="132" t="s">
-        <v>1425</v>
+        <v>1453</v>
       </c>
       <c r="G19" s="132" t="s">
-        <v>1484</v>
+        <v>1512</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="57" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A20" s="132" t="s">
-        <v>1485</v>
+        <v>1513</v>
       </c>
       <c r="B20" s="132" t="s">
-        <v>1486</v>
+        <v>1514</v>
       </c>
       <c r="C20" s="132" t="s">
-        <v>1487</v>
+        <v>1515</v>
       </c>
       <c r="D20" s="132" t="s">
         <v>587</v>
       </c>
       <c r="E20" s="132" t="s">
-        <v>1458</v>
+        <v>1486</v>
       </c>
       <c r="F20" s="132" t="s">
-        <v>1434</v>
+        <v>1462</v>
       </c>
       <c r="G20" s="132" t="s">
-        <v>1488</v>
+        <v>1516</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="245" t="s">
-        <v>1489</v>
+        <v>1517</v>
       </c>
       <c r="B21" s="245" t="s">
-        <v>1490</v>
+        <v>1518</v>
       </c>
       <c r="C21" s="245" t="s">
-        <v>1491</v>
+        <v>1519</v>
       </c>
       <c r="D21" s="245" t="s">
-        <v>1208</v>
+        <v>1236</v>
       </c>
       <c r="E21" s="245" t="s">
-        <v>1492</v>
+        <v>1520</v>
       </c>
       <c r="F21" s="245" t="s">
-        <v>1425</v>
+        <v>1453</v>
       </c>
       <c r="G21" s="245" t="s">
-        <v>1493</v>
+        <v>1521</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="245" t="s">
-        <v>1494</v>
+        <v>1522</v>
       </c>
       <c r="B22" s="245" t="s">
-        <v>1495</v>
+        <v>1523</v>
       </c>
       <c r="C22" s="245" t="s">
-        <v>1496</v>
+        <v>1524</v>
       </c>
       <c r="D22" s="245" t="s">
-        <v>1208</v>
+        <v>1236</v>
       </c>
       <c r="E22" s="245" t="s">
-        <v>1497</v>
+        <v>1525</v>
       </c>
       <c r="F22" s="245" t="s">
-        <v>1444</v>
+        <v>1472</v>
       </c>
       <c r="G22" s="245" t="s">
-        <v>1498</v>
+        <v>1526</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A23" s="272" t="s">
-        <v>1499</v>
-      </c>
-      <c r="B23" s="272" t="s">
-        <v>1500</v>
-      </c>
-      <c r="C23" s="272" t="n">
+      <c r="A23" s="275" t="s">
+        <v>1527</v>
+      </c>
+      <c r="B23" s="275" t="s">
+        <v>1528</v>
+      </c>
+      <c r="C23" s="275" t="n">
         <v>18.48</v>
       </c>
-      <c r="D23" s="272" t="s">
-        <v>1501</v>
-      </c>
-      <c r="E23" s="272" t="s">
-        <v>1502</v>
-      </c>
-      <c r="F23" s="272" t="s">
-        <v>1503</v>
-      </c>
-      <c r="G23" s="272" t="s">
-        <v>1504</v>
+      <c r="D23" s="275" t="s">
+        <v>1529</v>
+      </c>
+      <c r="E23" s="275" t="s">
+        <v>1530</v>
+      </c>
+      <c r="F23" s="275" t="s">
+        <v>1531</v>
+      </c>
+      <c r="G23" s="275" t="s">
+        <v>1532</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A24" s="273"/>
-      <c r="B24" s="273"/>
-      <c r="C24" s="273"/>
-      <c r="D24" s="273"/>
-      <c r="E24" s="273"/>
-      <c r="F24" s="273"/>
-      <c r="G24" s="273"/>
+      <c r="A24" s="276"/>
+      <c r="B24" s="276"/>
+      <c r="C24" s="276"/>
+      <c r="D24" s="276"/>
+      <c r="E24" s="276"/>
+      <c r="F24" s="276"/>
+      <c r="G24" s="276"/>
     </row>
     <row r="25" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A25" s="274" t="s">
-        <v>1505</v>
-      </c>
-      <c r="B25" s="274"/>
-      <c r="C25" s="274"/>
-      <c r="D25" s="274"/>
-      <c r="E25" s="274"/>
-      <c r="F25" s="274"/>
-      <c r="G25" s="274"/>
+      <c r="A25" s="277" t="s">
+        <v>1533</v>
+      </c>
+      <c r="B25" s="277"/>
+      <c r="C25" s="277"/>
+      <c r="D25" s="277"/>
+      <c r="E25" s="277"/>
+      <c r="F25" s="277"/>
+      <c r="G25" s="277"/>
     </row>
     <row r="26" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A26" s="275" t="s">
-        <v>1506</v>
-      </c>
-      <c r="B26" s="275"/>
-      <c r="C26" s="275"/>
-      <c r="D26" s="275"/>
-      <c r="E26" s="275"/>
-      <c r="F26" s="275"/>
-      <c r="G26" s="275"/>
+      <c r="A26" s="278" t="s">
+        <v>1534</v>
+      </c>
+      <c r="B26" s="278"/>
+      <c r="C26" s="278"/>
+      <c r="D26" s="278"/>
+      <c r="E26" s="278"/>
+      <c r="F26" s="278"/>
+      <c r="G26" s="278"/>
     </row>
     <row r="27" customFormat="false" ht="82.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="132" t="s">
-        <v>1507</v>
+        <v>1535</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="82.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="132" t="s">
-        <v>1508</v>
+        <v>1536</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="55.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="132" t="s">
-        <v>1509</v>
+        <v>1537</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -29886,12 +30246,12 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="238" t="s">
-        <v>1510</v>
+        <v>1538</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="239" t="s">
-        <v>1511</v>
+        <v>1539</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -29899,22 +30259,22 @@
         <v>359</v>
       </c>
       <c r="B4" s="244" t="s">
-        <v>1512</v>
+        <v>1540</v>
       </c>
       <c r="C4" s="244" t="s">
         <v>851</v>
       </c>
       <c r="D4" s="244" t="s">
-        <v>1513</v>
+        <v>1541</v>
       </c>
       <c r="E4" s="244" t="s">
-        <v>1514</v>
+        <v>1542</v>
       </c>
       <c r="F4" s="244" t="s">
-        <v>1515</v>
+        <v>1543</v>
       </c>
       <c r="G4" s="244" t="s">
-        <v>1516</v>
+        <v>1544</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -29922,22 +30282,22 @@
         <v>1</v>
       </c>
       <c r="B5" s="132" t="s">
-        <v>1490</v>
+        <v>1518</v>
       </c>
       <c r="C5" s="132" t="s">
-        <v>1517</v>
+        <v>1545</v>
       </c>
       <c r="D5" s="132" t="s">
-        <v>1518</v>
+        <v>1546</v>
       </c>
       <c r="E5" s="132" t="s">
-        <v>1519</v>
+        <v>1547</v>
       </c>
       <c r="F5" s="132" t="s">
-        <v>1520</v>
+        <v>1548</v>
       </c>
       <c r="G5" s="132" t="s">
-        <v>1521</v>
+        <v>1549</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="41.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -29945,22 +30305,22 @@
         <v>2</v>
       </c>
       <c r="B6" s="132" t="s">
-        <v>1490</v>
+        <v>1518</v>
       </c>
       <c r="C6" s="132" t="s">
         <v>46</v>
       </c>
       <c r="D6" s="132" t="s">
-        <v>1522</v>
+        <v>1550</v>
       </c>
       <c r="E6" s="132" t="s">
-        <v>1523</v>
+        <v>1551</v>
       </c>
       <c r="F6" s="132" t="s">
-        <v>1524</v>
+        <v>1552</v>
       </c>
       <c r="G6" s="132" t="s">
-        <v>1525</v>
+        <v>1553</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="55.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -29968,22 +30328,22 @@
         <v>3</v>
       </c>
       <c r="B7" s="132" t="s">
-        <v>1490</v>
+        <v>1518</v>
       </c>
       <c r="C7" s="132" t="s">
-        <v>1526</v>
+        <v>1554</v>
       </c>
       <c r="D7" s="132" t="s">
-        <v>1527</v>
+        <v>1555</v>
       </c>
       <c r="E7" s="132" t="s">
-        <v>1528</v>
+        <v>1556</v>
       </c>
       <c r="F7" s="132" t="s">
-        <v>1529</v>
+        <v>1557</v>
       </c>
       <c r="G7" s="132" t="s">
-        <v>1530</v>
+        <v>1558</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -29991,22 +30351,22 @@
         <v>4</v>
       </c>
       <c r="B8" s="132" t="s">
-        <v>1490</v>
+        <v>1518</v>
       </c>
       <c r="C8" s="132" t="s">
-        <v>1531</v>
+        <v>1559</v>
       </c>
       <c r="D8" s="132" t="s">
-        <v>1532</v>
+        <v>1560</v>
       </c>
       <c r="E8" s="132" t="s">
-        <v>1533</v>
+        <v>1561</v>
       </c>
       <c r="F8" s="132" t="s">
-        <v>1534</v>
+        <v>1562</v>
       </c>
       <c r="G8" s="132" t="s">
-        <v>1535</v>
+        <v>1563</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="41.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -30014,22 +30374,22 @@
         <v>5</v>
       </c>
       <c r="B9" s="132" t="s">
-        <v>1490</v>
+        <v>1518</v>
       </c>
       <c r="C9" s="132" t="s">
-        <v>1536</v>
+        <v>1564</v>
       </c>
       <c r="D9" s="132" t="s">
-        <v>1537</v>
+        <v>1565</v>
       </c>
       <c r="E9" s="132" t="s">
-        <v>1538</v>
+        <v>1566</v>
       </c>
       <c r="F9" s="132" t="s">
-        <v>1539</v>
+        <v>1567</v>
       </c>
       <c r="G9" s="132" t="s">
-        <v>1540</v>
+        <v>1568</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -30037,22 +30397,22 @@
         <v>6</v>
       </c>
       <c r="B10" s="132" t="s">
-        <v>1490</v>
+        <v>1518</v>
       </c>
       <c r="C10" s="132" t="s">
-        <v>1531</v>
+        <v>1559</v>
       </c>
       <c r="D10" s="132" t="s">
-        <v>1541</v>
+        <v>1569</v>
       </c>
       <c r="E10" s="132" t="s">
-        <v>1542</v>
+        <v>1570</v>
       </c>
       <c r="F10" s="132" t="s">
-        <v>1543</v>
+        <v>1571</v>
       </c>
       <c r="G10" s="132" t="s">
-        <v>1544</v>
+        <v>1572</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -30060,22 +30420,22 @@
         <v>7</v>
       </c>
       <c r="B11" s="132" t="s">
-        <v>1490</v>
+        <v>1518</v>
       </c>
       <c r="C11" s="132" t="s">
-        <v>1545</v>
+        <v>1573</v>
       </c>
       <c r="D11" s="132" t="s">
-        <v>1546</v>
+        <v>1574</v>
       </c>
       <c r="E11" s="132" t="s">
-        <v>1547</v>
+        <v>1575</v>
       </c>
       <c r="F11" s="132" t="s">
-        <v>1548</v>
+        <v>1576</v>
       </c>
       <c r="G11" s="132" t="s">
-        <v>1549</v>
+        <v>1577</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -30083,22 +30443,22 @@
         <v>8</v>
       </c>
       <c r="B12" s="132" t="s">
-        <v>1550</v>
+        <v>1578</v>
       </c>
       <c r="C12" s="132" t="s">
-        <v>1551</v>
+        <v>1579</v>
       </c>
       <c r="D12" s="132" t="s">
-        <v>1552</v>
+        <v>1580</v>
       </c>
       <c r="E12" s="132" t="s">
-        <v>1553</v>
+        <v>1581</v>
       </c>
       <c r="F12" s="132" t="s">
-        <v>1554</v>
+        <v>1582</v>
       </c>
       <c r="G12" s="132" t="s">
-        <v>1555</v>
+        <v>1583</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -30106,22 +30466,22 @@
         <v>9</v>
       </c>
       <c r="B13" s="132" t="s">
-        <v>1556</v>
+        <v>1584</v>
       </c>
       <c r="C13" s="132" t="s">
-        <v>1557</v>
+        <v>1585</v>
       </c>
       <c r="D13" s="132" t="s">
-        <v>1558</v>
+        <v>1586</v>
       </c>
       <c r="E13" s="132" t="s">
-        <v>1559</v>
+        <v>1587</v>
       </c>
       <c r="F13" s="132" t="s">
-        <v>1560</v>
+        <v>1588</v>
       </c>
       <c r="G13" s="132" t="s">
-        <v>1561</v>
+        <v>1589</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -30129,22 +30489,22 @@
         <v>10</v>
       </c>
       <c r="B14" s="132" t="s">
-        <v>1562</v>
+        <v>1590</v>
       </c>
       <c r="C14" s="132" t="s">
-        <v>1562</v>
+        <v>1590</v>
       </c>
       <c r="D14" s="132" t="s">
-        <v>1563</v>
+        <v>1591</v>
       </c>
       <c r="E14" s="132" t="s">
-        <v>1564</v>
+        <v>1592</v>
       </c>
       <c r="F14" s="132" t="s">
-        <v>1565</v>
+        <v>1593</v>
       </c>
       <c r="G14" s="132" t="s">
-        <v>1566</v>
+        <v>1594</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="41.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -30155,19 +30515,19 @@
         <v>374</v>
       </c>
       <c r="C15" s="132" t="s">
-        <v>1557</v>
+        <v>1585</v>
       </c>
       <c r="D15" s="132" t="s">
-        <v>1567</v>
+        <v>1595</v>
       </c>
       <c r="E15" s="132" t="s">
-        <v>1568</v>
+        <v>1596</v>
       </c>
       <c r="F15" s="132" t="s">
-        <v>1569</v>
+        <v>1597</v>
       </c>
       <c r="G15" s="132" t="s">
-        <v>1570</v>
+        <v>1598</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="41.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -30175,19 +30535,19 @@
         <v>12</v>
       </c>
       <c r="B16" s="132" t="s">
-        <v>1571</v>
+        <v>1599</v>
       </c>
       <c r="C16" s="132" t="s">
-        <v>1444</v>
+        <v>1472</v>
       </c>
       <c r="D16" s="132" t="s">
-        <v>1572</v>
+        <v>1600</v>
       </c>
       <c r="E16" s="132" t="s">
-        <v>1573</v>
+        <v>1601</v>
       </c>
       <c r="F16" s="132" t="s">
-        <v>1574</v>
+        <v>1602</v>
       </c>
       <c r="G16" s="132" t="s">
         <v>587</v>
@@ -30198,22 +30558,22 @@
         <v>13</v>
       </c>
       <c r="B17" s="132" t="s">
-        <v>1575</v>
+        <v>1603</v>
       </c>
       <c r="C17" s="132" t="s">
-        <v>1576</v>
+        <v>1604</v>
       </c>
       <c r="D17" s="132" t="s">
-        <v>1577</v>
+        <v>1605</v>
       </c>
       <c r="E17" s="132" t="s">
-        <v>1578</v>
+        <v>1606</v>
       </c>
       <c r="F17" s="132" t="s">
-        <v>1579</v>
+        <v>1607</v>
       </c>
       <c r="G17" s="132" t="s">
-        <v>1580</v>
+        <v>1608</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="55.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -30224,19 +30584,19 @@
         <v>973</v>
       </c>
       <c r="C18" s="132" t="s">
-        <v>1576</v>
+        <v>1604</v>
       </c>
       <c r="D18" s="132" t="s">
-        <v>1581</v>
+        <v>1609</v>
       </c>
       <c r="E18" s="132" t="s">
         <v>587</v>
       </c>
       <c r="F18" s="132" t="s">
-        <v>1582</v>
+        <v>1610</v>
       </c>
       <c r="G18" s="132" t="s">
-        <v>1583</v>
+        <v>1611</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="55.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -30244,19 +30604,19 @@
         <v>15</v>
       </c>
       <c r="B19" s="132" t="s">
-        <v>1584</v>
+        <v>1612</v>
       </c>
       <c r="C19" s="132" t="s">
-        <v>1576</v>
+        <v>1604</v>
       </c>
       <c r="D19" s="132" t="s">
-        <v>1585</v>
+        <v>1613</v>
       </c>
       <c r="E19" s="132" t="s">
-        <v>1586</v>
+        <v>1614</v>
       </c>
       <c r="F19" s="132" t="s">
-        <v>1587</v>
+        <v>1615</v>
       </c>
       <c r="G19" s="132" t="s">
         <v>587</v>

</xml_diff>

<commit_message>
Precio de referencia: cierre del 30-jun-2026 (MXN 30.25) desde el Excel auditado (WACC!B13 = Inflación!B183); ratios de mercado leídos del Excel
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01M3Z6Fw74B8ffLJq5CxcxMa
</commit_message>
<xml_diff>
--- a/excel/EXCEL FINAL PRO DEFINITIVO SORIANA - AUDITADO.xlsx
+++ b/excel/EXCEL FINAL PRO DEFINITIVO SORIANA - AUDITADO.xlsx
@@ -1430,7 +1430,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2923" uniqueCount="1635">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2929" uniqueCount="1641">
   <si>
     <t xml:space="preserve">1. VALUACIÓN (DCF, base FY2025)</t>
   </si>
@@ -2047,7 +2047,7 @@
     <t xml:space="preserve">DATOS DE MERCADO</t>
   </si>
   <si>
-    <t xml:space="preserve">Precio actual por acción (MXN)</t>
+    <t xml:space="preserve">Precio de referencia por acción (MXN) — cierre del 30-jun-2026 (serie mensual, hoja Inflación fila 183)</t>
   </si>
   <si>
     <t xml:space="preserve">Fecha del precio</t>
@@ -4375,7 +4375,7 @@
     <t xml:space="preserve">PRECIO COMBINADO (MXN por acción)</t>
   </si>
   <si>
-    <t xml:space="preserve">Precio de mercado (MXN, 25-sep-2026)</t>
+    <t xml:space="preserve">Precio de mercado de referencia (MXN, cierre 30-jun-2026)</t>
   </si>
   <si>
     <t xml:space="preserve">Diferencia vs. precio (MXN)</t>
@@ -5080,7 +5080,7 @@
     <t xml:space="preserve">Si se diera peso a transacciones con la nueva muestra.</t>
   </si>
   <si>
-    <t xml:space="preserve">Precio de mercado de referencia (25-sep-2026)</t>
+    <t xml:space="preserve">Precio de mercado de referencia (30-jun-2026)</t>
   </si>
   <si>
     <t xml:space="preserve">7. CONCLUSIÓN, VALUACIÓN Y RECOMENDACIÓN</t>
@@ -5158,123 +5158,123 @@
     <t xml:space="preserve">01-oct-2026</t>
   </si>
   <si>
+    <t xml:space="preserve">30-jun-2026</t>
+  </si>
+  <si>
+    <t xml:space="preserve">βU 0.1705 (regresión semanal desapalancada; βL observada 0.2178), WACC iterado, g 3.5%, múltiplo de salida 5.81x</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Rango = escenarios de inflación Cautela–Alcista.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Sí (50%)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">team_comps</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Trading Comps (7 pares CIQ, promedio de 3 múltiplos a la media)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">EV/EBITDA, EV/EBIT y P/U LTM; puente al 2T26</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Múltiplos CIQ y precio de referencia al 30-jun-2026.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">team_sdc</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Precedent Transactions LSEG/SDC (mediana EV/EBITDA)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">19-oct-2026</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Muestra global auditada; rango P25–P75</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Sin operaciones mexicanas; control mixto; dispersión amplia.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">No (0%, referencia)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">team_ciq_trans</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Precedent Transactions CIQ (3 operaciones, media)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Media de EV/EBITDA 7.63x</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Histórico: 1 de 3 en la ventana; no defendible.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">No (histórico)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">team_combined</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Valuación combinada (DCF 50% / Comps 50%)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Transacciones 0%</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Sí (precio objetivo)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">indiv_dcf</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Modelo individual del autor del reporte (SORIANA_FINAL)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">07-oct-2026</t>
+  </si>
+  <si>
+    <t xml:space="preserve">βU 0.1705 (regresión, no significativa al 95%), WACC 9.63%, Ke 10.39%, g 3.5%</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Misma βU que el equipo desde el 19-oct-2026; la diferencia restante es proyección, fecha y precio de referencia.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">No (otro modelo)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1, 5–7</t>
+  </si>
+  <si>
+    <t xml:space="preserve">indiv_combined</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Modelo individual del autor del reporte</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Valuación combinada (50% DCF / 50% comps)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Modelo distinto del equipo.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">No</t>
+  </si>
+  <si>
+    <t xml:space="preserve">8</t>
+  </si>
+  <si>
+    <t xml:space="preserve">app_hist</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ValuFlow (app del equipo, versión anterior)</t>
+  </si>
+  <si>
     <t xml:space="preserve">25-sep-2026</t>
   </si>
   <si>
-    <t xml:space="preserve">βU 0.1705 (regresión semanal desapalancada; βL observada 0.2178), WACC iterado, g 3.5%, múltiplo de salida 5.81x</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Rango = escenarios de inflación Cautela–Alcista.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Sí (50%)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">team_comps</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Trading Comps (7 pares CIQ, promedio de 3 múltiplos a la media)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">30-jun-2026</t>
-  </si>
-  <si>
-    <t xml:space="preserve">EV/EBITDA, EV/EBIT y P/U LTM; puente al 2T26</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Múltiplos CIQ al 30-jun-2026; precio de mercado de otra fecha.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">team_sdc</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Precedent Transactions LSEG/SDC (mediana EV/EBITDA)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">19-oct-2026</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Muestra global auditada; rango P25–P75</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Sin operaciones mexicanas; control mixto; dispersión amplia.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">No (0%, referencia)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">team_ciq_trans</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Precedent Transactions CIQ (3 operaciones, media)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Media de EV/EBITDA 7.63x</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Histórico: 1 de 3 en la ventana; no defendible.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">No (histórico)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">team_combined</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Valuación combinada (DCF 50% / Comps 50%)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Transacciones 0%</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Sí (precio objetivo)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">indiv_dcf</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Modelo individual del autor del reporte (SORIANA_FINAL)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">07-oct-2026</t>
-  </si>
-  <si>
-    <t xml:space="preserve">βU 0.1705 (regresión, no significativa al 95%), WACC 9.63%, Ke 10.39%, g 3.5%</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Misma βU que el equipo desde el 19-oct-2026; la diferencia restante es proyección, fecha y precio de referencia.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">No (otro modelo)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1, 5–7</t>
-  </si>
-  <si>
-    <t xml:space="preserve">indiv_combined</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Modelo individual del autor del reporte</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Valuación combinada (50% DCF / 50% comps)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Modelo distinto del equipo.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">No</t>
-  </si>
-  <si>
-    <t xml:space="preserve">8</t>
-  </si>
-  <si>
-    <t xml:space="preserve">app_hist</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ValuFlow (app del equipo, versión anterior)</t>
-  </si>
-  <si>
     <t xml:space="preserve">βU 0.80 (heredada), WACC 11.88%, Ke 13.95%</t>
   </si>
   <si>
@@ -5956,7 +5956,7 @@
     <t xml:space="preserve">9.517%</t>
   </si>
   <si>
-    <t xml:space="preserve">Cierre del Bono M 10 años el 25-sep-2026 (misma fecha que el precio de Soriana, WACC!B14): 9.517%. Fuente consultada: Investing.com, histórico Mexico 10Y (no oficial); confirmar en Banxico SIE (vector de precios de valores gubernamentales). Al usar el Bono M en pesos, el Rf ya incorpora el riesgo soberano de México.</t>
+    <t xml:space="preserve">Cierre del Bono M 10 años el 25-sep-2026 (cercano a la fecha de valuación; el precio de referencia de Soriana es el cierre del 30-jun-2026, WACC!B14): 9.517%. Fuente consultada: Investing.com, histórico Mexico 10Y (no oficial); confirmar en Banxico SIE (vector de precios de valores gubernamentales). Al usar el Bono M en pesos, el Rf ya incorpora el riesgo soberano de México.</t>
   </si>
   <si>
     <t xml:space="preserve">WACC!B6</t>
@@ -6328,13 +6328,31 @@
     <t xml:space="preserve">Fechas</t>
   </si>
   <si>
-    <t xml:space="preserve">Fecha de valuación 01-oct-2026; precio 33.48 MXN del 25-sep-2026 (último cierre antes de la valuación); balance 2T26; comparables CIQ al 30-jun-2026; pantalla SDC 19-oct-2026; reporte comparativo 19-oct-2026 con precio 33.10 MXN del 7-oct-2026.</t>
+    <t xml:space="preserve">Fecha de valuación 01-oct-2026; precio de referencia 30.25 MXN del 30-jun-2026 (antes 33.48 MXN del 25-sep-2026; ver hallazgo de precio); balance 2T26; comparables CIQ al 30-jun-2026; pantalla SDC 19-oct-2026; reporte comparativo 19-oct-2026 con precio 33.10 MXN del 7-oct-2026.</t>
   </si>
   <si>
     <t xml:space="preserve">Cada fecha cumple una función distinta.</t>
   </si>
   <si>
     <t xml:space="preserve">Se rotulan en cada salida; el precio nunca se presenta como "del día".</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Precio de referencia</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Cambio de supuesto (retroalimentación del profesor, 20-oct-2026)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">El precio de comparación era 33.48 MXN (cierre 25-sep-2026). El profesor pidió usar 30.25 MXN, cierre del 30-jun-2026.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Cambia la capitalización de mercado (E = precio × acciones), el WACC a mercado (punto de partida de la iteración), el potencial y la recomendación. El WACC iterado converge al mismo punto fijo, así que el DCF casi no cambia.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">WACC!B13 = Inflación!B183 (30.25, cierre de junio 2026) y WACC!B14 = 30-jun-2026. Fecha de valuación, balance, proyección, comparables y transacciones sin cambio. El Rf (Bono M) se conserva al 25-sep-2026.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Recálculo en LibreOffice; tabla A y controles de Validación.</t>
   </si>
 </sst>
 </file>
@@ -8222,7 +8240,7 @@
       </c>
       <c r="B5" s="4" t="n">
         <f aca="false">Valuación!B15</f>
-        <v>0.100630184051038</v>
+        <v>0.10049964337765</v>
       </c>
       <c r="C5" s="4" t="n">
         <f aca="false">Valuación!B53</f>
@@ -8285,7 +8303,7 @@
       </c>
       <c r="B8" s="5" t="n">
         <f aca="false">Valuación!B31</f>
-        <v>27698.2061852259</v>
+        <v>27707.6609242111</v>
       </c>
       <c r="C8" s="5" t="n">
         <f aca="false">Valuación!B69</f>
@@ -8306,7 +8324,7 @@
       </c>
       <c r="B9" s="5" t="n">
         <f aca="false">Valuación!B33</f>
-        <v>124303.410482692</v>
+        <v>124551.146959902</v>
       </c>
       <c r="C9" s="5" t="n">
         <f aca="false">Valuación!B71</f>
@@ -8327,7 +8345,7 @@
       </c>
       <c r="B10" s="5" t="n">
         <f aca="false">Valuación!B34</f>
-        <v>76961.9299902015</v>
+        <v>77161.0627174786</v>
       </c>
       <c r="C10" s="5" t="n">
         <f aca="false">Valuación!B72</f>
@@ -8348,7 +8366,7 @@
       </c>
       <c r="B11" s="5" t="n">
         <f aca="false">Valuación!B35</f>
-        <v>104660.136175427</v>
+        <v>104868.72364169</v>
       </c>
       <c r="C11" s="5" t="n">
         <f aca="false">Valuación!B73</f>
@@ -8411,7 +8429,7 @@
       </c>
       <c r="B14" s="5" t="n">
         <f aca="false">Valuación!B39</f>
-        <v>90337.1361754274</v>
+        <v>90545.7236416897</v>
       </c>
       <c r="C14" s="5" t="n">
         <f aca="false">Valuación!B77</f>
@@ -8432,7 +8450,7 @@
       </c>
       <c r="B15" s="6" t="n">
         <f aca="false">Valuación!B41</f>
-        <v>50.1872978752374</v>
+        <v>50.3031798009387</v>
       </c>
       <c r="C15" s="6" t="n">
         <f aca="false">Valuación!B79</f>
@@ -8453,7 +8471,7 @@
       </c>
       <c r="B16" s="6" t="n">
         <f aca="false">Valuación!B42</f>
-        <v>33.48</v>
+        <v>30.25</v>
       </c>
       <c r="C16" s="6" t="n">
         <f aca="false">Valuación!B80</f>
@@ -8474,7 +8492,7 @@
       </c>
       <c r="B17" s="7" t="n">
         <f aca="false">Valuación!B43</f>
-        <v>0.499023234027403</v>
+        <v>0.662915034741776</v>
       </c>
       <c r="C17" s="7" t="n">
         <f aca="false">Valuación!B81</f>
@@ -11938,23 +11956,23 @@
       <c r="B119" s="105"/>
       <c r="C119" s="107" t="n">
         <f aca="false">1/(1+$B$126)^C118</f>
-        <v>0.912718730291208</v>
+        <v>0.912718730384644</v>
       </c>
       <c r="D119" s="107" t="n">
         <f aca="false">1/(1+$B$126)^D118</f>
-        <v>0.833055480624394</v>
+        <v>0.833055480794956</v>
       </c>
       <c r="E119" s="107" t="n">
         <f aca="false">1/(1+$B$126)^E118</f>
-        <v>0.760345340537629</v>
+        <v>0.760345340771142</v>
       </c>
       <c r="F119" s="107" t="n">
         <f aca="false">1/(1+$B$126)^F118</f>
-        <v>0.69398143379834</v>
+        <v>0.693981434082516</v>
       </c>
       <c r="G119" s="107" t="n">
         <f aca="false">1/(1+$B$126)^G118</f>
-        <v>0.633409853102093</v>
+        <v>0.633409853426309</v>
       </c>
     </row>
     <row r="120" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -11964,23 +11982,23 @@
       <c r="B120" s="105"/>
       <c r="C120" s="100" t="n">
         <f aca="false">C117*C119</f>
-        <v>5081.85076486183</v>
+        <v>5081.85076538207</v>
       </c>
       <c r="D120" s="100" t="n">
         <f aca="false">D117*D119</f>
-        <v>4905.91250427151</v>
+        <v>4905.91250527596</v>
       </c>
       <c r="E120" s="100" t="n">
         <f aca="false">E117*E119</f>
-        <v>4884.30809162533</v>
+        <v>4884.30809312537</v>
       </c>
       <c r="F120" s="100" t="n">
         <f aca="false">F117*F119</f>
-        <v>4428.64950288821</v>
+        <v>4428.64950470168</v>
       </c>
       <c r="G120" s="100" t="n">
         <f aca="false">G117*G119</f>
-        <v>4246.66039259276</v>
+        <v>4246.66039476644</v>
       </c>
     </row>
     <row r="121" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -12024,7 +12042,7 @@
       </c>
       <c r="B124" s="99" t="n">
         <f aca="false">B220</f>
-        <v>0.0956277841268195</v>
+        <v>0.0956277840146585</v>
       </c>
       <c r="C124" s="105"/>
       <c r="D124" s="105"/>
@@ -12051,7 +12069,7 @@
       </c>
       <c r="B126" s="99" t="n">
         <f aca="false">B124+B125</f>
-        <v>0.0956277841268195</v>
+        <v>0.0956277840146585</v>
       </c>
       <c r="C126" s="105"/>
       <c r="D126" s="105"/>
@@ -12093,7 +12111,7 @@
       </c>
       <c r="B129" s="104" t="n">
         <f aca="false">IF(B126&gt;B123,B128/(B126-B123),"REVISAR WACC/g")</f>
-        <v>99025.313510992</v>
+        <v>99025.3136941883</v>
       </c>
       <c r="C129" s="103"/>
       <c r="D129" s="103"/>
@@ -12107,7 +12125,7 @@
       </c>
       <c r="B130" s="107" t="n">
         <f aca="false">G119</f>
-        <v>0.633409853102093</v>
+        <v>0.633409853426309</v>
       </c>
       <c r="C130" s="105"/>
       <c r="D130" s="105"/>
@@ -12121,7 +12139,7 @@
       </c>
       <c r="B131" s="100" t="n">
         <f aca="false">B129*B130</f>
-        <v>62723.6092843861</v>
+        <v>62723.60943253</v>
       </c>
       <c r="C131" s="105"/>
       <c r="D131" s="105"/>
@@ -12157,7 +12175,7 @@
       </c>
       <c r="B134" s="100" t="n">
         <f aca="false">SUM(C120:G120)</f>
-        <v>23547.3812562396</v>
+        <v>23547.3812632515</v>
       </c>
       <c r="C134" s="105"/>
       <c r="D134" s="105"/>
@@ -12171,7 +12189,7 @@
       </c>
       <c r="B135" s="100" t="n">
         <f aca="false">B131</f>
-        <v>62723.6092843861</v>
+        <v>62723.60943253</v>
       </c>
       <c r="C135" s="105"/>
       <c r="D135" s="105"/>
@@ -12185,7 +12203,7 @@
       </c>
       <c r="B136" s="104" t="n">
         <f aca="false">B134+B135</f>
-        <v>86270.9905406258</v>
+        <v>86270.9906957815</v>
       </c>
       <c r="C136" s="103"/>
       <c r="D136" s="103"/>
@@ -12199,7 +12217,7 @@
       </c>
       <c r="B137" s="98" t="n">
         <f aca="false">B135/B136</f>
-        <v>0.727053310635735</v>
+        <v>0.727053311045344</v>
       </c>
       <c r="C137" s="105"/>
       <c r="D137" s="105"/>
@@ -12235,7 +12253,7 @@
       </c>
       <c r="B140" s="100" t="n">
         <f aca="false">B136</f>
-        <v>86270.9905406258</v>
+        <v>86270.9906957815</v>
       </c>
       <c r="C140" s="105"/>
       <c r="D140" s="105"/>
@@ -12305,7 +12323,7 @@
       </c>
       <c r="B145" s="104" t="n">
         <f aca="false">SUM(B140:B143)</f>
-        <v>71947.9905406258</v>
+        <v>71947.9906957815</v>
       </c>
       <c r="C145" s="103"/>
       <c r="D145" s="103"/>
@@ -12341,7 +12359,7 @@
       </c>
       <c r="B148" s="100" t="n">
         <f aca="false">B145</f>
-        <v>71947.9905406258</v>
+        <v>71947.9906957815</v>
       </c>
       <c r="C148" s="105"/>
       <c r="D148" s="105"/>
@@ -12369,7 +12387,7 @@
       </c>
       <c r="B150" s="109" t="n">
         <f aca="false">B148/B149</f>
-        <v>39.9711058559032</v>
+        <v>39.9711059421009</v>
       </c>
       <c r="C150" s="103"/>
       <c r="D150" s="103"/>
@@ -12383,7 +12401,7 @@
       </c>
       <c r="B151" s="110" t="n">
         <f aca="false">Valuación!B42</f>
-        <v>33.48</v>
+        <v>30.25</v>
       </c>
       <c r="C151" s="105"/>
       <c r="D151" s="105"/>
@@ -12397,7 +12415,7 @@
       </c>
       <c r="B152" s="98" t="n">
         <f aca="false">B150/B151-1</f>
-        <v>0.193880103222915</v>
+        <v>0.321358874119037</v>
       </c>
       <c r="C152" s="105"/>
       <c r="D152" s="105"/>
@@ -12411,7 +12429,7 @@
       </c>
       <c r="B153" s="110" t="n">
         <f aca="false">'Proyección Soriana'!B85</f>
-        <v>50.1811650263689</v>
+        <v>50.2970347293132</v>
       </c>
       <c r="C153" s="105"/>
       <c r="D153" s="105"/>
@@ -12425,7 +12443,7 @@
       </c>
       <c r="B154" s="98" t="n">
         <f aca="false">B150/B153-1</f>
-        <v>-0.203463972291208</v>
+        <v>-0.205298957339812</v>
       </c>
       <c r="C154" s="105"/>
       <c r="D154" s="105"/>
@@ -12551,135 +12569,135 @@
     <row r="163" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A163" s="111" t="n">
         <f aca="false">$B$126-2*$B$161</f>
-        <v>0.0856277841268195</v>
+        <v>0.0856277840146585</v>
       </c>
       <c r="B163" s="110" t="n">
         <f aca="false" t="array" ref="B163:B163">(SUMPRODUCT($C$117:$G$117,1/(1+$A163)^$C$118:$G$118)+$B$127*(1+B$162)/($A163-B$162)/(1+$A163)^$G$118+$B$141+$B$142+$B$143)/$B$149</f>
-        <v>41.6080851373411</v>
+        <v>41.6080852269052</v>
       </c>
       <c r="C163" s="110" t="n">
         <f aca="false" t="array" ref="C163:C163">(SUMPRODUCT($C$117:$G$117,1/(1+$A163)^$C$118:$G$118)+$B$127*(1+C$162)/($A163-C$162)/(1+$A163)^$G$118+$B$141+$B$142+$B$143)/$B$149</f>
-        <v>45.0475257623403</v>
+        <v>45.0475258666236</v>
       </c>
       <c r="D163" s="110" t="n">
         <f aca="false" t="array" ref="D163:D163">(SUMPRODUCT($C$117:$G$117,1/(1+$A163)^$C$118:$G$118)+$B$127*(1+D$162)/($A163-D$162)/(1+$A163)^$G$118+$B$141+$B$142+$B$143)/$B$149</f>
-        <v>49.1663247049746</v>
+        <v>49.1663248283895</v>
       </c>
       <c r="E163" s="110" t="n">
         <f aca="false" t="array" ref="E163:E163">(SUMPRODUCT($C$117:$G$117,1/(1+$A163)^$C$118:$G$118)+$B$127*(1+E$162)/($A163-E$162)/(1+$A163)^$G$118+$B$141+$B$142+$B$143)/$B$149</f>
-        <v>54.1878190165504</v>
+        <v>54.1878191655088</v>
       </c>
       <c r="F163" s="110" t="n">
         <f aca="false" t="array" ref="F163:F163">(SUMPRODUCT($C$117:$G$117,1/(1+$A163)^$C$118:$G$118)+$B$127*(1+F$162)/($A163-F$162)/(1+$A163)^$G$118+$B$141+$B$142+$B$143)/$B$149</f>
-        <v>60.4452887620561</v>
+        <v>60.4452889462574</v>
       </c>
       <c r="G163" s="105"/>
     </row>
     <row r="164" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A164" s="111" t="n">
         <f aca="false">A163+$B$161</f>
-        <v>0.0906277841268195</v>
+        <v>0.0906277840146585</v>
       </c>
       <c r="B164" s="110" t="n">
         <f aca="false" t="array" ref="B164:B164">(SUMPRODUCT($C$117:$G$117,1/(1+$A164)^$C$118:$G$118)+$B$127*(1+B$162)/($A164-B$162)/(1+$A164)^$G$118+$B$141+$B$142+$B$143)/$B$149</f>
-        <v>37.9182273719414</v>
+        <v>37.9182274484378</v>
       </c>
       <c r="C164" s="110" t="n">
         <f aca="false" t="array" ref="C164:C164">(SUMPRODUCT($C$117:$G$117,1/(1+$A164)^$C$118:$G$118)+$B$127*(1+C$162)/($A164-C$162)/(1+$A164)^$G$118+$B$141+$B$142+$B$143)/$B$149</f>
-        <v>40.7804895076976</v>
+        <v>40.7804895955583</v>
       </c>
       <c r="D164" s="110" t="n">
         <f aca="false" t="array" ref="D164:D164">(SUMPRODUCT($C$117:$G$117,1/(1+$A164)^$C$118:$G$118)+$B$127*(1+D$162)/($A164-D$162)/(1+$A164)^$G$118+$B$141+$B$142+$B$143)/$B$149</f>
-        <v>44.1572898693933</v>
+        <v>44.1572899716987</v>
       </c>
       <c r="E164" s="110" t="n">
         <f aca="false" t="array" ref="E164:E164">(SUMPRODUCT($C$117:$G$117,1/(1+$A164)^$C$118:$G$118)+$B$127*(1+E$162)/($A164-E$162)/(1+$A164)^$G$118+$B$141+$B$142+$B$143)/$B$149</f>
-        <v>48.2010758438184</v>
+        <v>48.2010759648993</v>
       </c>
       <c r="F164" s="110" t="n">
         <f aca="false" t="array" ref="F164:F164">(SUMPRODUCT($C$117:$G$117,1/(1+$A164)^$C$118:$G$118)+$B$127*(1+F$162)/($A164-F$162)/(1+$A164)^$G$118+$B$141+$B$142+$B$143)/$B$149</f>
-        <v>53.1311169918863</v>
+        <v>53.1311171380362</v>
       </c>
       <c r="G164" s="105"/>
     </row>
     <row r="165" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A165" s="111" t="n">
         <f aca="false">A164+$B$161</f>
-        <v>0.0956277841268195</v>
+        <v>0.0956277840146585</v>
       </c>
       <c r="B165" s="110" t="n">
         <f aca="false" t="array" ref="B165:B165">(SUMPRODUCT($C$117:$G$117,1/(1+$A165)^$C$118:$G$118)+$B$127*(1+B$162)/($A165-B$162)/(1+$A165)^$G$118+$B$141+$B$142+$B$143)/$B$149</f>
-        <v>34.7482788379517</v>
+        <v>34.7482789040543</v>
       </c>
       <c r="C165" s="110" t="n">
         <f aca="false" t="array" ref="C165:C165">(SUMPRODUCT($C$117:$G$117,1/(1+$A165)^$C$118:$G$118)+$B$127*(1+C$162)/($A165-C$162)/(1+$A165)^$G$118+$B$141+$B$142+$B$143)/$B$149</f>
-        <v>37.1607359488317</v>
+        <v>37.1607360238763</v>
       </c>
       <c r="D165" s="112" t="n">
         <f aca="false" t="array" ref="D165:D165">(SUMPRODUCT($C$117:$G$117,1/(1+$A165)^$C$118:$G$118)+$B$127*(1+D$162)/($A165-D$162)/(1+$A165)^$G$118+$B$141+$B$142+$B$143)/$B$149</f>
-        <v>39.9711058559032</v>
+        <v>39.9711059421009</v>
       </c>
       <c r="E165" s="110" t="n">
         <f aca="false" t="array" ref="E165:E165">(SUMPRODUCT($C$117:$G$117,1/(1+$A165)^$C$118:$G$118)+$B$127*(1+E$162)/($A165-E$162)/(1+$A165)^$G$118+$B$141+$B$142+$B$143)/$B$149</f>
-        <v>43.2866855158321</v>
+        <v>43.2866856162064</v>
       </c>
       <c r="F165" s="110" t="n">
         <f aca="false" t="array" ref="F165:F165">(SUMPRODUCT($C$117:$G$117,1/(1+$A165)^$C$118:$G$118)+$B$127*(1+F$162)/($A165-F$162)/(1+$A165)^$G$118+$B$141+$B$142+$B$143)/$B$149</f>
-        <v>47.2571584753816</v>
+        <v>47.2571585941835</v>
       </c>
       <c r="G165" s="105"/>
     </row>
     <row r="166" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A166" s="111" t="n">
         <f aca="false">A165+$B$161</f>
-        <v>0.10062778412682</v>
+        <v>0.100627784014659</v>
       </c>
       <c r="B166" s="110" t="n">
         <f aca="false" t="array" ref="B166:B166">(SUMPRODUCT($C$117:$G$117,1/(1+$A166)^$C$118:$G$118)+$B$127*(1+B$162)/($A166-B$162)/(1+$A166)^$G$118+$B$141+$B$142+$B$143)/$B$149</f>
-        <v>31.9951991973123</v>
+        <v>31.995199255012</v>
       </c>
       <c r="C166" s="110" t="n">
         <f aca="false" t="array" ref="C166:C166">(SUMPRODUCT($C$117:$G$117,1/(1+$A166)^$C$118:$G$118)+$B$127*(1+C$162)/($A166-C$162)/(1+$A166)^$G$118+$B$141+$B$142+$B$143)/$B$149</f>
-        <v>34.050882586818</v>
+        <v>34.0508826516688</v>
       </c>
       <c r="D166" s="110" t="n">
         <f aca="false" t="array" ref="D166:D166">(SUMPRODUCT($C$117:$G$117,1/(1+$A166)^$C$118:$G$118)+$B$127*(1+D$162)/($A166-D$162)/(1+$A166)^$G$118+$B$141+$B$142+$B$143)/$B$149</f>
-        <v>36.4197996801362</v>
+        <v>36.4197997537633</v>
       </c>
       <c r="E166" s="110" t="n">
         <f aca="false" t="array" ref="E166:E166">(SUMPRODUCT($C$117:$G$117,1/(1+$A166)^$C$118:$G$118)+$B$127*(1+E$162)/($A166-E$162)/(1+$A166)^$G$118+$B$141+$B$142+$B$143)/$B$149</f>
-        <v>39.1794480408817</v>
+        <v>39.1794481254554</v>
       </c>
       <c r="F166" s="110" t="n">
         <f aca="false" t="array" ref="F166:F166">(SUMPRODUCT($C$117:$G$117,1/(1+$A166)^$C$118:$G$118)+$B$127*(1+F$162)/($A166-F$162)/(1+$A166)^$G$118+$B$141+$B$142+$B$143)/$B$149</f>
-        <v>42.4351881306191</v>
+        <v>42.4351882291075</v>
       </c>
       <c r="G166" s="105"/>
     </row>
     <row r="167" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A167" s="111" t="n">
         <f aca="false">A166+$B$161</f>
-        <v>0.10562778412682</v>
+        <v>0.105627784014659</v>
       </c>
       <c r="B167" s="110" t="n">
         <f aca="false" t="array" ref="B167:B167">(SUMPRODUCT($C$117:$G$117,1/(1+$A167)^$C$118:$G$118)+$B$127*(1+B$162)/($A167-B$162)/(1+$A167)^$G$118+$B$141+$B$142+$B$143)/$B$149</f>
-        <v>29.581504922679</v>
+        <v>29.5815049734885</v>
       </c>
       <c r="C167" s="110" t="n">
         <f aca="false" t="array" ref="C167:C167">(SUMPRODUCT($C$117:$G$117,1/(1+$A167)^$C$118:$G$118)+$B$127*(1+C$162)/($A167-C$162)/(1+$A167)^$G$118+$B$141+$B$142+$B$143)/$B$149</f>
-        <v>31.3498751538021</v>
+        <v>31.3498752104118</v>
       </c>
       <c r="D167" s="110" t="n">
         <f aca="false" t="array" ref="D167:D167">(SUMPRODUCT($C$117:$G$117,1/(1+$A167)^$C$118:$G$118)+$B$127*(1+D$162)/($A167-D$162)/(1+$A167)^$G$118+$B$141+$B$142+$B$143)/$B$149</f>
-        <v>33.3686242199666</v>
+        <v>33.3686242835953</v>
       </c>
       <c r="E167" s="110" t="n">
         <f aca="false" t="array" ref="E167:E167">(SUMPRODUCT($C$117:$G$117,1/(1+$A167)^$C$118:$G$118)+$B$127*(1+E$162)/($A167-E$162)/(1+$A167)^$G$118+$B$141+$B$142+$B$143)/$B$149</f>
-        <v>35.6949791413377</v>
+        <v>35.6949792135806</v>
       </c>
       <c r="F167" s="110" t="n">
         <f aca="false" t="array" ref="F167:F167">(SUMPRODUCT($C$117:$G$117,1/(1+$A167)^$C$118:$G$118)+$B$127*(1+F$162)/($A167-F$162)/(1+$A167)^$G$118+$B$141+$B$142+$B$143)/$B$149</f>
-        <v>38.405045088087</v>
+        <v>38.4050451710749</v>
       </c>
       <c r="G167" s="105"/>
     </row>
@@ -13595,27 +13613,27 @@
       </c>
       <c r="B214" s="99" t="n">
         <f aca="false">WACC!B33</f>
-        <v>0.100630184051038</v>
+        <v>0.10049964337765</v>
       </c>
       <c r="C214" s="100" t="n">
         <f aca="false" t="array" ref="C214:C214">SUMPRODUCT($C$117:$G$117,1/(1+B214)^$C$118:$G$118)+$B$127*(1+$B$123)/(B214-$B$123)/(1+B214)^$G$118-$B$144</f>
-        <v>65552.8037920425</v>
+        <v>65707.3442223899</v>
       </c>
       <c r="D214" s="107" t="n">
         <f aca="false">$B$209/C214</f>
-        <v>0.360289699810934</v>
+        <v>0.359442316220599</v>
       </c>
       <c r="E214" s="107" t="n">
         <f aca="false">$B$212*(1+(1-$B$207)*D214)</f>
-        <v>0.213526641210658</v>
+        <v>0.213425493631905</v>
       </c>
       <c r="F214" s="99" t="n">
         <f aca="false">$B$210+E214*$B$211</f>
-        <v>0.104202176923211</v>
+        <v>0.10419789838063</v>
       </c>
       <c r="G214" s="99" t="n">
         <f aca="false">C214/(C214+$B$209)*F214+$B$209/(C214+$B$209)*$B$208</f>
-        <v>0.0951433036124324</v>
+        <v>0.0951558289547022</v>
       </c>
     </row>
     <row r="215" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -13624,27 +13642,27 @@
       </c>
       <c r="B215" s="99" t="n">
         <f aca="false">G214</f>
-        <v>0.0951433036124324</v>
+        <v>0.0951558289547022</v>
       </c>
       <c r="C215" s="100" t="n">
         <f aca="false" t="array" ref="C215:C215">SUMPRODUCT($C$117:$G$117,1/(1+B215)^$C$118:$G$118)+$B$127*(1+$B$123)/(B215-$B$123)/(1+B215)^$G$118-$B$144</f>
-        <v>72623.5581022153</v>
+        <v>72605.9562287197</v>
       </c>
       <c r="D215" s="107" t="n">
         <f aca="false">$B$209/C215</f>
-        <v>0.325211276026416</v>
+        <v>0.325290117047694</v>
       </c>
       <c r="E215" s="107" t="n">
         <f aca="false">$B$212*(1+(1-$B$207)*D215)</f>
-        <v>0.209339520203425</v>
+        <v>0.209348931028109</v>
       </c>
       <c r="F215" s="99" t="n">
         <f aca="false">$B$210+E215*$B$211</f>
-        <v>0.104025061704605</v>
+        <v>0.104025459782489</v>
       </c>
       <c r="G215" s="99" t="n">
         <f aca="false">C215/(C215+$B$209)*F215+$B$209/(C215+$B$209)*$B$208</f>
-        <v>0.0956751978496798</v>
+        <v>0.0956739708119807</v>
       </c>
     </row>
     <row r="216" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -13653,27 +13671,27 @@
       </c>
       <c r="B216" s="99" t="n">
         <f aca="false">G215</f>
-        <v>0.0956751978496798</v>
+        <v>0.0956739708119807</v>
       </c>
       <c r="C216" s="100" t="n">
         <f aca="false" t="array" ref="C216:C216">SUMPRODUCT($C$117:$G$117,1/(1+B216)^$C$118:$G$118)+$B$127*(1+$B$123)/(B216-$B$123)/(1+B216)^$G$118-$B$144</f>
-        <v>71882.4527069998</v>
+        <v>71884.1475009234</v>
       </c>
       <c r="D216" s="107" t="n">
         <f aca="false">$B$209/C216</f>
-        <v>0.3285641921022</v>
+        <v>0.32855644562936</v>
       </c>
       <c r="E216" s="107" t="n">
         <f aca="false">$B$212*(1+(1-$B$207)*D216)</f>
-        <v>0.20973973959249</v>
+        <v>0.209738814938083</v>
       </c>
       <c r="F216" s="99" t="n">
         <f aca="false">$B$210+E216*$B$211</f>
-        <v>0.104041990984762</v>
+        <v>0.104041951871881</v>
       </c>
       <c r="G216" s="99" t="n">
         <f aca="false">C216/(C216+$B$209)*F216+$B$209/(C216+$B$209)*$B$208</f>
-        <v>0.0956231435312865</v>
+        <v>0.0956232634931478</v>
       </c>
     </row>
     <row r="217" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -13682,27 +13700,27 @@
       </c>
       <c r="B217" s="99" t="n">
         <f aca="false">G216</f>
-        <v>0.0956231435312865</v>
+        <v>0.0956232634931478</v>
       </c>
       <c r="C217" s="100" t="n">
         <f aca="false" t="array" ref="C217:C217">SUMPRODUCT($C$117:$G$117,1/(1+B217)^$C$118:$G$118)+$B$127*(1+$B$123)/(B217-$B$123)/(1+B217)^$G$118-$B$144</f>
-        <v>71954.410504547</v>
+        <v>71954.2445327548</v>
       </c>
       <c r="D217" s="107" t="n">
         <f aca="false">$B$209/C217</f>
-        <v>0.328235612443903</v>
+        <v>0.328236369561892</v>
       </c>
       <c r="E217" s="107" t="n">
         <f aca="false">$B$212*(1+(1-$B$207)*D217)</f>
-        <v>0.209700518822531</v>
+        <v>0.209700609195594</v>
       </c>
       <c r="F217" s="99" t="n">
         <f aca="false">$B$210+E217*$B$211</f>
-        <v>0.104040331946193</v>
+        <v>0.104040335768974</v>
       </c>
       <c r="G217" s="99" t="n">
         <f aca="false">C217/(C217+$B$209)*F217+$B$209/(C217+$B$209)*$B$208</f>
-        <v>0.0956282331442387</v>
+        <v>0.0956282214137846</v>
       </c>
     </row>
     <row r="218" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -13711,27 +13729,27 @@
       </c>
       <c r="B218" s="99" t="n">
         <f aca="false">G217</f>
-        <v>0.0956282331442387</v>
+        <v>0.0956282214137846</v>
       </c>
       <c r="C218" s="100" t="n">
         <f aca="false" t="array" ref="C218:C218">SUMPRODUCT($C$117:$G$117,1/(1+B218)^$C$118:$G$118)+$B$127*(1+$B$123)/(B218-$B$123)/(1+B218)^$G$118-$B$144</f>
-        <v>71947.3694059349</v>
+        <v>71947.3856327879</v>
       </c>
       <c r="D218" s="107" t="n">
         <f aca="false">$B$209/C218</f>
-        <v>0.32826773508208</v>
+        <v>0.328267661045307</v>
       </c>
       <c r="E218" s="107" t="n">
         <f aca="false">$B$212*(1+(1-$B$207)*D218)</f>
-        <v>0.209704353127457</v>
+        <v>0.209704344290089</v>
       </c>
       <c r="F218" s="99" t="n">
         <f aca="false">$B$210+E218*$B$211</f>
-        <v>0.104040494137291</v>
+        <v>0.104040493763471</v>
       </c>
       <c r="G218" s="99" t="n">
         <f aca="false">C218/(C218+$B$209)*F218+$B$209/(C218+$B$209)*$B$208</f>
-        <v>0.0956277354619232</v>
+        <v>0.0956277366089617</v>
       </c>
     </row>
     <row r="219" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -13740,27 +13758,27 @@
       </c>
       <c r="B219" s="99" t="n">
         <f aca="false">G218</f>
-        <v>0.0956277354619232</v>
+        <v>0.0956277366089617</v>
       </c>
       <c r="C219" s="100" t="n">
         <f aca="false" t="array" ref="C219:C219">SUMPRODUCT($C$117:$G$117,1/(1+B219)^$C$118:$G$118)+$B$127*(1+$B$123)/(B219-$B$123)/(1+B219)^$G$118-$B$144</f>
-        <v>71948.0578602907</v>
+        <v>71948.0562735554</v>
       </c>
       <c r="D219" s="107" t="n">
         <f aca="false">$B$209/C219</f>
-        <v>0.328264593963907</v>
+        <v>0.328264601203422</v>
       </c>
       <c r="E219" s="107" t="n">
         <f aca="false">$B$212*(1+(1-$B$207)*D219)</f>
-        <v>0.209703978189233</v>
+        <v>0.209703979053375</v>
       </c>
       <c r="F219" s="99" t="n">
         <f aca="false">$B$210+E219*$B$211</f>
-        <v>0.104040478277405</v>
+        <v>0.104040478313958</v>
       </c>
       <c r="G219" s="99" t="n">
         <f aca="false">C219/(C219+$B$209)*F219+$B$209/(C219+$B$209)*$B$208</f>
-        <v>0.0956277841268195</v>
+        <v>0.0956277840146585</v>
       </c>
     </row>
     <row r="220" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -13769,7 +13787,7 @@
       </c>
       <c r="B220" s="111" t="n">
         <f aca="false">G219</f>
-        <v>0.0956277841268195</v>
+        <v>0.0956277840146585</v>
       </c>
       <c r="C220" s="103"/>
       <c r="D220" s="103"/>
@@ -13783,7 +13801,7 @@
       </c>
       <c r="B221" s="111" t="n">
         <f aca="false">F219</f>
-        <v>0.104040478277405</v>
+        <v>0.104040478313958</v>
       </c>
       <c r="C221" s="103"/>
       <c r="D221" s="103"/>
@@ -13797,7 +13815,7 @@
       </c>
       <c r="B222" s="113" t="n">
         <f aca="false">(G219-G218)*10000</f>
-        <v>0.00048664896321049</v>
+        <v>0.000474056967569858</v>
       </c>
       <c r="C222" s="106"/>
       <c r="D222" s="106"/>
@@ -13848,7 +13866,7 @@
       </c>
       <c r="B226" s="100" t="n">
         <f aca="false">WACC!B18</f>
-        <v>60264</v>
+        <v>54450</v>
       </c>
       <c r="C226" s="100" t="n">
         <f aca="false">WACC!C18</f>
@@ -13917,7 +13935,7 @@
       </c>
       <c r="B229" s="100" t="n">
         <f aca="false">SUM(B226:B228)</f>
-        <v>74587</v>
+        <v>68773</v>
       </c>
       <c r="C229" s="100" t="n">
         <f aca="false">SUM(C226:C228)</f>
@@ -13963,7 +13981,7 @@
       </c>
       <c r="B231" s="115" t="n">
         <f aca="false">B229/B230</f>
-        <v>6.27097696317471</v>
+        <v>5.78215907180091</v>
       </c>
       <c r="C231" s="115" t="n">
         <f aca="false">C229/C230</f>
@@ -14055,7 +14073,7 @@
       </c>
       <c r="B237" s="100" t="n">
         <f aca="false">B236*G119</f>
-        <v>48947.0225397703</v>
+        <v>48947.0225648243</v>
       </c>
       <c r="C237" s="105"/>
       <c r="D237" s="105"/>
@@ -14069,7 +14087,7 @@
       </c>
       <c r="B238" s="104" t="n">
         <f aca="false">B134+B237</f>
-        <v>72494.40379601</v>
+        <v>72494.4038280758</v>
       </c>
       <c r="C238" s="105"/>
       <c r="D238" s="105"/>
@@ -14083,7 +14101,7 @@
       </c>
       <c r="B239" s="100" t="n">
         <f aca="false">B238-B144</f>
-        <v>58171.40379601</v>
+        <v>58171.4038280758</v>
       </c>
       <c r="C239" s="105"/>
       <c r="D239" s="105"/>
@@ -14097,7 +14115,7 @@
       </c>
       <c r="B240" s="109" t="n">
         <f aca="false">B239/B149</f>
-        <v>32.3174465533389</v>
+        <v>32.3174465711532</v>
       </c>
       <c r="C240" s="105"/>
       <c r="D240" s="105"/>
@@ -14111,7 +14129,7 @@
       </c>
       <c r="B241" s="117" t="n">
         <f aca="false">B129/G71</f>
-        <v>7.44626689247961</v>
+        <v>7.44626690625516</v>
       </c>
       <c r="C241" s="105"/>
       <c r="D241" s="105"/>
@@ -14125,7 +14143,7 @@
       </c>
       <c r="B242" s="99" t="n">
         <f aca="false">(B236*B126-B127)/(B236+B127)</f>
-        <v>0.0191272410371974</v>
+        <v>0.0191272409328678</v>
       </c>
       <c r="C242" s="105"/>
       <c r="D242" s="105"/>
@@ -14166,7 +14184,7 @@
       </c>
       <c r="B245" s="100" t="n">
         <f aca="false">B243*B136+B244*B238</f>
-        <v>79382.6971683179</v>
+        <v>79382.6972619287</v>
       </c>
       <c r="C245" s="105"/>
       <c r="D245" s="105"/>
@@ -14180,7 +14198,7 @@
       </c>
       <c r="B246" s="109" t="n">
         <f aca="false">B243*B150+B244*B240</f>
-        <v>36.144276204621</v>
+        <v>36.144276256627</v>
       </c>
       <c r="C246" s="105"/>
       <c r="D246" s="105"/>
@@ -14295,7 +14313,7 @@
       </c>
       <c r="B255" s="100" t="n">
         <f aca="false">B245</f>
-        <v>79382.6971683179</v>
+        <v>79382.6972619287</v>
       </c>
       <c r="C255" s="105"/>
       <c r="D255" s="105"/>
@@ -14309,7 +14327,7 @@
       </c>
       <c r="B256" s="100" t="n">
         <f aca="false">B255*(1+B126)^B253</f>
-        <v>83091.6473540494</v>
+        <v>83091.6474477808</v>
       </c>
       <c r="C256" s="105"/>
       <c r="D256" s="105"/>
@@ -14337,7 +14355,7 @@
       </c>
       <c r="B258" s="100" t="n">
         <f aca="false">B256+B257</f>
-        <v>84152.1443540494</v>
+        <v>84152.1444477808</v>
       </c>
       <c r="C258" s="105"/>
       <c r="D258" s="105"/>
@@ -14393,7 +14411,7 @@
       </c>
       <c r="B262" s="104" t="n">
         <f aca="false">SUM(B258:B261)</f>
-        <v>67306.9403540494</v>
+        <v>67306.9404477808</v>
       </c>
       <c r="C262" s="105"/>
       <c r="D262" s="105"/>
@@ -14407,7 +14425,7 @@
       </c>
       <c r="B263" s="104" t="n">
         <f aca="false">B262*(1+B221)^B254</f>
-        <v>69012.1409597606</v>
+        <v>69012.1410564443</v>
       </c>
       <c r="C263" s="105"/>
       <c r="D263" s="105"/>
@@ -14435,7 +14453,7 @@
       </c>
       <c r="B265" s="109" t="n">
         <f aca="false">B263/B264</f>
-        <v>38.3400783109781</v>
+        <v>38.3400783646913</v>
       </c>
       <c r="C265" s="105"/>
       <c r="D265" s="105"/>
@@ -14449,7 +14467,7 @@
       </c>
       <c r="B266" s="110" t="n">
         <f aca="false">B151</f>
-        <v>33.48</v>
+        <v>30.25</v>
       </c>
       <c r="C266" s="105"/>
       <c r="D266" s="105"/>
@@ -14463,7 +14481,7 @@
       </c>
       <c r="B267" s="98" t="n">
         <f aca="false">B265/B266-1</f>
-        <v>0.145163629360159</v>
+        <v>0.267440607097232</v>
       </c>
       <c r="C267" s="105"/>
       <c r="D267" s="105"/>
@@ -14505,7 +14523,7 @@
       </c>
       <c r="B270" s="98" t="n">
         <f aca="false">B265/B269-1</f>
-        <v>0.641481282312717</v>
+        <v>0.641481284612376</v>
       </c>
       <c r="C270" s="105"/>
       <c r="D270" s="105"/>
@@ -14546,131 +14564,131 @@
     <row r="275" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A275" s="120" t="n">
         <f aca="false">$B$126+(0-2)*$B$161</f>
-        <v>0.0856277841268195</v>
+        <v>0.0856277840146585</v>
       </c>
       <c r="B275" s="121" t="n">
         <f aca="false">(($B$243*(SUMPRODUCT($C$117:$G$117,1/(1+$A275)^$C$118:$G$118)+$B$127*(1+B$274)/($A275-B$274)/(1+$A275)^$G$118)+$B$244*(SUMPRODUCT($C$117:$G$117,1/(1+$A275)^$C$118:$G$118)+$B$234*$G$71/(1+$A275)^$G$118))*(1+$A275)^$B$253+$B$257+$B$259+$B$260+$B$261)*(1+$B$221)^$B$254/$B$264</f>
-        <v>39.8689044782261</v>
+        <v>39.8689045339037</v>
       </c>
       <c r="C275" s="121" t="n">
         <f aca="false">(($B$243*(SUMPRODUCT($C$117:$G$117,1/(1+$A275)^$C$118:$G$118)+$B$127*(1+C$274)/($A275-C$274)/(1+$A275)^$G$118)+$B$244*(SUMPRODUCT($C$117:$G$117,1/(1+$A275)^$C$118:$G$118)+$B$234*$G$71/(1+$A275)^$G$118))*(1+$A275)^$B$253+$B$257+$B$259+$B$260+$B$261)*(1+$B$221)^$B$254/$B$264</f>
-        <v>41.7061362519603</v>
+        <v>41.7061363154208</v>
       </c>
       <c r="D275" s="121" t="n">
         <f aca="false">(($B$243*(SUMPRODUCT($C$117:$G$117,1/(1+$A275)^$C$118:$G$118)+$B$127*(1+D$274)/($A275-D$274)/(1+$A275)^$G$118)+$B$244*(SUMPRODUCT($C$117:$G$117,1/(1+$A275)^$C$118:$G$118)+$B$234*$G$71/(1+$A275)^$G$118))*(1+$A275)^$B$253+$B$257+$B$259+$B$260+$B$261)*(1+$B$221)^$B$254/$B$264</f>
-        <v>43.9062580485191</v>
+        <v>43.9062581221039</v>
       </c>
       <c r="E275" s="121" t="n">
         <f aca="false">(($B$243*(SUMPRODUCT($C$117:$G$117,1/(1+$A275)^$C$118:$G$118)+$B$127*(1+E$274)/($A275-E$274)/(1+$A275)^$G$118)+$B$244*(SUMPRODUCT($C$117:$G$117,1/(1+$A275)^$C$118:$G$118)+$B$234*$G$71/(1+$A275)^$G$118))*(1+$A275)^$B$253+$B$257+$B$259+$B$260+$B$261)*(1+$B$221)^$B$254/$B$264</f>
-        <v>46.5885688969162</v>
+        <v>46.5885689840293</v>
       </c>
       <c r="F275" s="121" t="n">
         <f aca="false">(($B$243*(SUMPRODUCT($C$117:$G$117,1/(1+$A275)^$C$118:$G$118)+$B$127*(1+F$274)/($A275-F$274)/(1+$A275)^$G$118)+$B$244*(SUMPRODUCT($C$117:$G$117,1/(1+$A275)^$C$118:$G$118)+$B$234*$G$71/(1+$A275)^$G$118))*(1+$A275)^$B$253+$B$257+$B$259+$B$260+$B$261)*(1+$B$221)^$B$254/$B$264</f>
-        <v>49.9310956310785</v>
+        <v>49.9310957368725</v>
       </c>
     </row>
     <row r="276" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A276" s="120" t="n">
         <f aca="false">$B$126+(1-2)*$B$161</f>
-        <v>0.0906277841268195</v>
+        <v>0.0906277840146585</v>
       </c>
       <c r="B276" s="121" t="n">
         <f aca="false">(($B$243*(SUMPRODUCT($C$117:$G$117,1/(1+$A276)^$C$118:$G$118)+$B$127*(1+B$274)/($A276-B$274)/(1+$A276)^$G$118)+$B$244*(SUMPRODUCT($C$117:$G$117,1/(1+$A276)^$C$118:$G$118)+$B$234*$G$71/(1+$A276)^$G$118))*(1+$A276)^$B$253+$B$257+$B$259+$B$260+$B$261)*(1+$B$221)^$B$254/$B$264</f>
-        <v>37.5636113649666</v>
+        <v>37.5636114136321</v>
       </c>
       <c r="C276" s="121" t="n">
         <f aca="false">(($B$243*(SUMPRODUCT($C$117:$G$117,1/(1+$A276)^$C$118:$G$118)+$B$127*(1+C$274)/($A276-C$274)/(1+$A276)^$G$118)+$B$244*(SUMPRODUCT($C$117:$G$117,1/(1+$A276)^$C$118:$G$118)+$B$234*$G$71/(1+$A276)^$G$118))*(1+$A276)^$B$253+$B$257+$B$259+$B$260+$B$261)*(1+$B$221)^$B$254/$B$264</f>
-        <v>39.09605087388</v>
+        <v>39.0960509285639</v>
       </c>
       <c r="D276" s="121" t="n">
         <f aca="false">(($B$243*(SUMPRODUCT($C$117:$G$117,1/(1+$A276)^$C$118:$G$118)+$B$127*(1+D$274)/($A276-D$274)/(1+$A276)^$G$118)+$B$244*(SUMPRODUCT($C$117:$G$117,1/(1+$A276)^$C$118:$G$118)+$B$234*$G$71/(1+$A276)^$G$118))*(1+$A276)^$B$253+$B$257+$B$259+$B$260+$B$261)*(1+$B$221)^$B$254/$B$264</f>
-        <v>40.9039713376737</v>
+        <v>40.9039714000134</v>
       </c>
       <c r="E276" s="121" t="n">
         <f aca="false">(($B$243*(SUMPRODUCT($C$117:$G$117,1/(1+$A276)^$C$118:$G$118)+$B$127*(1+E$274)/($A276-E$274)/(1+$A276)^$G$118)+$B$244*(SUMPRODUCT($C$117:$G$117,1/(1+$A276)^$C$118:$G$118)+$B$234*$G$71/(1+$A276)^$G$118))*(1+$A276)^$B$253+$B$257+$B$259+$B$260+$B$261)*(1+$B$221)^$B$254/$B$264</f>
-        <v>43.0689922543067</v>
+        <v>43.0689923266055</v>
       </c>
       <c r="F276" s="121" t="n">
         <f aca="false">(($B$243*(SUMPRODUCT($C$117:$G$117,1/(1+$A276)^$C$118:$G$118)+$B$127*(1+F$274)/($A276-F$274)/(1+$A276)^$G$118)+$B$244*(SUMPRODUCT($C$117:$G$117,1/(1+$A276)^$C$118:$G$118)+$B$234*$G$71/(1+$A276)^$G$118))*(1+$A276)^$B$253+$B$257+$B$259+$B$260+$B$261)*(1+$B$221)^$B$254/$B$264</f>
-        <v>45.7085093486668</v>
+        <v>45.7085094342737</v>
       </c>
     </row>
     <row r="277" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A277" s="120" t="n">
         <f aca="false">$B$126+(2-2)*$B$161</f>
-        <v>0.0956277841268195</v>
+        <v>0.0956277840146585</v>
       </c>
       <c r="B277" s="121" t="n">
         <f aca="false">(($B$243*(SUMPRODUCT($C$117:$G$117,1/(1+$A277)^$C$118:$G$118)+$B$127*(1+B$274)/($A277-B$274)/(1+$A277)^$G$118)+$B$244*(SUMPRODUCT($C$117:$G$117,1/(1+$A277)^$C$118:$G$118)+$B$234*$G$71/(1+$A277)^$G$118))*(1+$A277)^$B$253+$B$257+$B$259+$B$260+$B$261)*(1+$B$221)^$B$254/$B$264</f>
-        <v>35.5374028126272</v>
+        <v>35.5374028556769</v>
       </c>
       <c r="C277" s="121" t="n">
         <f aca="false">(($B$243*(SUMPRODUCT($C$117:$G$117,1/(1+$A277)^$C$118:$G$118)+$B$127*(1+C$274)/($A277-C$274)/(1+$A277)^$G$118)+$B$244*(SUMPRODUCT($C$117:$G$117,1/(1+$A277)^$C$118:$G$118)+$B$234*$G$71/(1+$A277)^$G$118))*(1+$A277)^$B$253+$B$257+$B$259+$B$260+$B$261)*(1+$B$221)^$B$254/$B$264</f>
-        <v>36.8319765008321</v>
+        <v>36.8319765486248</v>
       </c>
       <c r="D277" s="121" t="n">
         <f aca="false">(($B$243*(SUMPRODUCT($C$117:$G$117,1/(1+$A277)^$C$118:$G$118)+$B$127*(1+D$274)/($A277-D$274)/(1+$A277)^$G$118)+$B$244*(SUMPRODUCT($C$117:$G$117,1/(1+$A277)^$C$118:$G$118)+$B$234*$G$71/(1+$A277)^$G$118))*(1+$A277)^$B$253+$B$257+$B$259+$B$260+$B$261)*(1+$B$221)^$B$254/$B$264</f>
-        <v>38.3400783109781</v>
+        <v>38.3400783646913</v>
       </c>
       <c r="E277" s="121" t="n">
         <f aca="false">(($B$243*(SUMPRODUCT($C$117:$G$117,1/(1+$A277)^$C$118:$G$118)+$B$127*(1+E$274)/($A277-E$274)/(1+$A277)^$G$118)+$B$244*(SUMPRODUCT($C$117:$G$117,1/(1+$A277)^$C$118:$G$118)+$B$234*$G$71/(1+$A277)^$G$118))*(1+$A277)^$B$253+$B$257+$B$259+$B$260+$B$261)*(1+$B$221)^$B$254/$B$264</f>
-        <v>40.1192859783533</v>
+        <v>40.1192860395977</v>
       </c>
       <c r="F277" s="121" t="n">
         <f aca="false">(($B$243*(SUMPRODUCT($C$117:$G$117,1/(1+$A277)^$C$118:$G$118)+$B$127*(1+F$274)/($A277-F$274)/(1+$A277)^$G$118)+$B$244*(SUMPRODUCT($C$117:$G$117,1/(1+$A277)^$C$118:$G$118)+$B$234*$G$71/(1+$A277)^$G$118))*(1+$A277)^$B$253+$B$257+$B$259+$B$260+$B$261)*(1+$B$221)^$B$254/$B$264</f>
-        <v>42.2499227469743</v>
+        <v>42.2499228180161</v>
       </c>
     </row>
     <row r="278" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A278" s="120" t="n">
         <f aca="false">$B$126+(3-2)*$B$161</f>
-        <v>0.10062778412682</v>
+        <v>0.100627784014658</v>
       </c>
       <c r="B278" s="121" t="n">
         <f aca="false">(($B$243*(SUMPRODUCT($C$117:$G$117,1/(1+$A278)^$C$118:$G$118)+$B$127*(1+B$274)/($A278-B$274)/(1+$A278)^$G$118)+$B$244*(SUMPRODUCT($C$117:$G$117,1/(1+$A278)^$C$118:$G$118)+$B$234*$G$71/(1+$A278)^$G$118))*(1+$A278)^$B$253+$B$257+$B$259+$B$260+$B$261)*(1+$B$221)^$B$254/$B$264</f>
-        <v>33.7365334061119</v>
+        <v>33.7365334445868</v>
       </c>
       <c r="C278" s="121" t="n">
         <f aca="false">(($B$243*(SUMPRODUCT($C$117:$G$117,1/(1+$A278)^$C$118:$G$118)+$B$127*(1+C$274)/($A278-C$274)/(1+$A278)^$G$118)+$B$244*(SUMPRODUCT($C$117:$G$117,1/(1+$A278)^$C$118:$G$118)+$B$234*$G$71/(1+$A278)^$G$118))*(1+$A278)^$B$253+$B$257+$B$259+$B$260+$B$261)*(1+$B$221)^$B$254/$B$264</f>
-        <v>34.8421692731812</v>
+        <v>34.8421693154553</v>
       </c>
       <c r="D278" s="121" t="n">
         <f aca="false">(($B$243*(SUMPRODUCT($C$117:$G$117,1/(1+$A278)^$C$118:$G$118)+$B$127*(1+D$274)/($A278-D$274)/(1+$A278)^$G$118)+$B$244*(SUMPRODUCT($C$117:$G$117,1/(1+$A278)^$C$118:$G$118)+$B$234*$G$71/(1+$A278)^$G$118))*(1+$A278)^$B$253+$B$257+$B$259+$B$260+$B$261)*(1+$B$221)^$B$254/$B$264</f>
-        <v>36.1162758393272</v>
+        <v>36.1162758862672</v>
       </c>
       <c r="E278" s="121" t="n">
         <f aca="false">(($B$243*(SUMPRODUCT($C$117:$G$117,1/(1+$A278)^$C$118:$G$118)+$B$127*(1+E$274)/($A278-E$274)/(1+$A278)^$G$118)+$B$244*(SUMPRODUCT($C$117:$G$117,1/(1+$A278)^$C$118:$G$118)+$B$234*$G$71/(1+$A278)^$G$118))*(1+$A278)^$B$253+$B$257+$B$259+$B$260+$B$261)*(1+$B$221)^$B$254/$B$264</f>
-        <v>37.6005346623132</v>
+        <v>37.6005347150776</v>
       </c>
       <c r="F278" s="121" t="n">
         <f aca="false">(($B$243*(SUMPRODUCT($C$117:$G$117,1/(1+$A278)^$C$118:$G$118)+$B$127*(1+F$274)/($A278-F$274)/(1+$A278)^$G$118)+$B$244*(SUMPRODUCT($C$117:$G$117,1/(1+$A278)^$C$118:$G$118)+$B$234*$G$71/(1+$A278)^$G$118))*(1+$A278)^$B$253+$B$257+$B$259+$B$260+$B$261)*(1+$B$221)^$B$254/$B$264</f>
-        <v>39.3516131773441</v>
+        <v>39.3516132375178</v>
       </c>
     </row>
     <row r="279" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A279" s="120" t="n">
         <f aca="false">$B$126+(4-2)*$B$161</f>
-        <v>0.10562778412682</v>
+        <v>0.105627784014658</v>
       </c>
       <c r="B279" s="121" t="n">
         <f aca="false">(($B$243*(SUMPRODUCT($C$117:$G$117,1/(1+$A279)^$C$118:$G$118)+$B$127*(1+B$274)/($A279-B$274)/(1+$A279)^$G$118)+$B$244*(SUMPRODUCT($C$117:$G$117,1/(1+$A279)^$C$118:$G$118)+$B$234*$G$71/(1+$A279)^$G$118))*(1+$A279)^$B$253+$B$257+$B$259+$B$260+$B$261)*(1+$B$221)^$B$254/$B$264</f>
-        <v>32.1205313788558</v>
+        <v>32.1205314135483</v>
       </c>
       <c r="C279" s="121" t="n">
         <f aca="false">(($B$243*(SUMPRODUCT($C$117:$G$117,1/(1+$A279)^$C$118:$G$118)+$B$127*(1+C$274)/($A279-C$274)/(1+$A279)^$G$118)+$B$244*(SUMPRODUCT($C$117:$G$117,1/(1+$A279)^$C$118:$G$118)+$B$234*$G$71/(1+$A279)^$G$118))*(1+$A279)^$B$253+$B$257+$B$259+$B$260+$B$261)*(1+$B$221)^$B$254/$B$264</f>
-        <v>33.0737956670992</v>
+        <v>33.073795704878</v>
       </c>
       <c r="D279" s="121" t="n">
         <f aca="false">(($B$243*(SUMPRODUCT($C$117:$G$117,1/(1+$A279)^$C$118:$G$118)+$B$127*(1+D$274)/($A279-D$274)/(1+$A279)^$G$118)+$B$244*(SUMPRODUCT($C$117:$G$117,1/(1+$A279)^$C$118:$G$118)+$B$234*$G$71/(1+$A279)^$G$118))*(1+$A279)^$B$253+$B$257+$B$259+$B$260+$B$261)*(1+$B$221)^$B$254/$B$264</f>
-        <v>34.16203010909</v>
+        <v>34.1620301506064</v>
       </c>
       <c r="E279" s="121" t="n">
         <f aca="false">(($B$243*(SUMPRODUCT($C$117:$G$117,1/(1+$A279)^$C$118:$G$118)+$B$127*(1+E$274)/($A279-E$274)/(1+$A279)^$G$118)+$B$244*(SUMPRODUCT($C$117:$G$117,1/(1+$A279)^$C$118:$G$118)+$B$234*$G$71/(1+$A279)^$G$118))*(1+$A279)^$B$253+$B$257+$B$259+$B$260+$B$261)*(1+$B$221)^$B$254/$B$264</f>
-        <v>35.4160837169219</v>
+        <v>35.4160837630287</v>
       </c>
       <c r="F279" s="121" t="n">
         <f aca="false">(($B$243*(SUMPRODUCT($C$117:$G$117,1/(1+$A279)^$C$118:$G$118)+$B$127*(1+F$274)/($A279-F$274)/(1+$A279)^$G$118)+$B$244*(SUMPRODUCT($C$117:$G$117,1/(1+$A279)^$C$118:$G$118)+$B$234*$G$71/(1+$A279)^$G$118))*(1+$A279)^$B$253+$B$257+$B$259+$B$260+$B$261)*(1+$B$221)^$B$254/$B$264</f>
-        <v>36.8769820290247</v>
+        <v>36.8769820808619</v>
       </c>
     </row>
     <row r="280" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -18468,11 +18486,11 @@
       </c>
       <c r="B24" s="136" t="n">
         <f aca="false">WACC!B23</f>
-        <v>0.391908934023629</v>
+        <v>0.433755739210285</v>
       </c>
       <c r="C24" s="136" t="n">
         <f aca="false">'Proyección Final Soriana'!D219</f>
-        <v>0.328264593963907</v>
+        <v>0.328264601203422</v>
       </c>
       <c r="E24" s="132"/>
     </row>
@@ -18496,11 +18514,11 @@
       </c>
       <c r="B26" s="136" t="n">
         <f aca="false">B23*(1+(1-B25)*B24)</f>
-        <v>0.21730085753856</v>
+        <v>0.222295883488385</v>
       </c>
       <c r="C26" s="136" t="n">
         <f aca="false">C23*(1+(1-C25)*C24)</f>
-        <v>0.209703978189233</v>
+        <v>0.209703979053375</v>
       </c>
       <c r="E26" s="132"/>
     </row>
@@ -18538,11 +18556,11 @@
       </c>
       <c r="B29" s="139" t="n">
         <f aca="false">B27+B26*B28</f>
-        <v>0.104361826273881</v>
+        <v>0.104573115871559</v>
       </c>
       <c r="C29" s="139" t="n">
         <f aca="false">C27+C26*C28</f>
-        <v>0.104040478277405</v>
+        <v>0.104040478313958</v>
       </c>
       <c r="E29" s="132"/>
     </row>
@@ -18552,11 +18570,11 @@
       </c>
       <c r="B30" s="139" t="n">
         <f aca="false">WACC!B33</f>
-        <v>0.100630184051038</v>
+        <v>0.10049964337765</v>
       </c>
       <c r="C30" s="139" t="n">
         <f aca="false">'Proyección Final Soriana'!B126</f>
-        <v>0.0956277841268195</v>
+        <v>0.0956277840146585</v>
       </c>
       <c r="E30" s="132"/>
     </row>
@@ -18639,15 +18657,15 @@
       </c>
       <c r="B37" s="136" t="n">
         <f aca="false">Validación!H14</f>
-        <v>0.907086203708222</v>
+        <v>0.907086220409621</v>
       </c>
       <c r="C37" s="136" t="n">
         <f aca="false">Validación!F14</f>
-        <v>0.209703978189233</v>
+        <v>0.209703979053375</v>
       </c>
       <c r="D37" s="136" t="n">
         <f aca="false">C37-B37</f>
-        <v>-0.697382225518989</v>
+        <v>-0.697382241356246</v>
       </c>
       <c r="E37" s="130"/>
     </row>
@@ -18657,15 +18675,15 @@
       </c>
       <c r="B38" s="139" t="n">
         <f aca="false">Validación!H13</f>
-        <v>0.133539746416858</v>
+        <v>0.133539747123327</v>
       </c>
       <c r="C38" s="139" t="n">
         <f aca="false">Validación!F13</f>
-        <v>0.104040478277405</v>
+        <v>0.104040478313958</v>
       </c>
       <c r="D38" s="139" t="n">
         <f aca="false">C38-B38</f>
-        <v>-0.029499268139453</v>
+        <v>-0.029499268809369</v>
       </c>
       <c r="E38" s="130"/>
     </row>
@@ -18675,15 +18693,15 @@
       </c>
       <c r="B39" s="139" t="n">
         <f aca="false">Validación!H12</f>
-        <v>0.113837026578705</v>
+        <v>0.113837026020324</v>
       </c>
       <c r="C39" s="139" t="n">
         <f aca="false">Validación!F12</f>
-        <v>0.0956277841268195</v>
+        <v>0.0956277840146585</v>
       </c>
       <c r="D39" s="139" t="n">
         <f aca="false">C39-B39</f>
-        <v>-0.0182092424518855</v>
+        <v>-0.0182092420056655</v>
       </c>
       <c r="E39" s="130"/>
     </row>
@@ -18693,15 +18711,15 @@
       </c>
       <c r="B40" s="139" t="n">
         <f aca="false">Validación!H15</f>
-        <v>0.120748041823037</v>
+        <v>0.120479269946713</v>
       </c>
       <c r="C40" s="139" t="n">
         <f aca="false">Validación!F15</f>
-        <v>0.100630184051038</v>
+        <v>0.10049964337765</v>
       </c>
       <c r="D40" s="139" t="n">
         <f aca="false">C40-B40</f>
-        <v>-0.020117857771999</v>
+        <v>-0.019979626569063</v>
       </c>
       <c r="E40" s="130"/>
     </row>
@@ -18711,15 +18729,15 @@
       </c>
       <c r="B41" s="139" t="n">
         <f aca="false">Validación!H16</f>
-        <v>0.132364052240143</v>
+        <v>0.133219020132231</v>
       </c>
       <c r="C41" s="139" t="n">
         <f aca="false">Validación!F16</f>
-        <v>0.104361826273881</v>
+        <v>0.104573115871559</v>
       </c>
       <c r="D41" s="139" t="n">
         <f aca="false">C41-B41</f>
-        <v>-0.028002225966262</v>
+        <v>-0.028645904260672</v>
       </c>
       <c r="E41" s="130"/>
     </row>
@@ -18729,15 +18747,15 @@
       </c>
       <c r="B42" s="172" t="n">
         <f aca="false">Validación!H11</f>
-        <v>67198.4289751488</v>
+        <v>67198.4292769918</v>
       </c>
       <c r="C42" s="172" t="n">
         <f aca="false">Validación!F11</f>
-        <v>79382.6971683179</v>
+        <v>79382.6972619287</v>
       </c>
       <c r="D42" s="172" t="n">
         <f aca="false">C42-B42</f>
-        <v>12184.2681931691</v>
+        <v>12184.2679849369</v>
       </c>
       <c r="E42" s="130"/>
     </row>
@@ -18747,15 +18765,15 @@
       </c>
       <c r="B43" s="172" t="n">
         <f aca="false">Validación!H10</f>
-        <v>56910.4022601389</v>
+        <v>56910.4025795714</v>
       </c>
       <c r="C43" s="172" t="n">
         <f aca="false">Validación!F10</f>
-        <v>69012.1409597606</v>
+        <v>69012.1410564443</v>
       </c>
       <c r="D43" s="172" t="n">
         <f aca="false">C43-B43</f>
-        <v>12101.7386996217</v>
+        <v>12101.7384768729</v>
       </c>
       <c r="E43" s="130"/>
     </row>
@@ -18765,15 +18783,15 @@
       </c>
       <c r="B44" s="173" t="n">
         <f aca="false">Validación!H9</f>
-        <v>31.6168901445216</v>
+        <v>31.6168903219841</v>
       </c>
       <c r="C44" s="173" t="n">
         <f aca="false">Validación!F9</f>
-        <v>38.3400783109781</v>
+        <v>38.3400783646913</v>
       </c>
       <c r="D44" s="173" t="n">
         <f aca="false">C44-B44</f>
-        <v>6.7231881664565</v>
+        <v>6.7231880427072</v>
       </c>
       <c r="E44" s="130"/>
     </row>
@@ -18783,15 +18801,15 @@
       </c>
       <c r="B45" s="173" t="n">
         <f aca="false">Validación!H19</f>
-        <v>32.5548654995095</v>
+        <v>32.5548655882407</v>
       </c>
       <c r="C45" s="173" t="n">
         <f aca="false">Validación!F19</f>
-        <v>35.9164595827377</v>
+        <v>35.9164596095943</v>
       </c>
       <c r="D45" s="173" t="n">
         <f aca="false">C45-B45</f>
-        <v>3.3615940832282</v>
+        <v>3.3615940213536</v>
       </c>
       <c r="E45" s="130"/>
     </row>
@@ -20686,7 +20704,7 @@
       <c r="C76" s="198"/>
       <c r="D76" s="200" t="n">
         <f aca="false">Valuación!B42</f>
-        <v>33.48</v>
+        <v>30.25</v>
       </c>
     </row>
     <row r="77" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -20697,7 +20715,7 @@
       <c r="C77" s="198"/>
       <c r="D77" s="207" t="n">
         <f aca="false">D73/D76-1</f>
-        <v>0.000383538067423972</v>
+        <v>0.107201350561896</v>
       </c>
     </row>
     <row r="78" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -21593,7 +21611,7 @@
       </c>
       <c r="B4" s="231" t="n">
         <f aca="false">'Proyección Final Soriana'!B265</f>
-        <v>38.3400783109781</v>
+        <v>38.3400783646913</v>
       </c>
       <c r="C4" s="232" t="n">
         <v>0.5</v>
@@ -21604,7 +21622,7 @@
       </c>
       <c r="E4" s="231" t="n">
         <f aca="false">IF(ISNUMBER(B4),B4*C4,0)</f>
-        <v>19.1700391554891</v>
+        <v>19.1700391823456</v>
       </c>
       <c r="F4" s="234" t="s">
         <v>974</v>
@@ -21710,7 +21728,7 @@
       </c>
       <c r="B9" s="237" t="n">
         <f aca="false">IF(ABS(C7-1)&gt;0.000000001,"Los pesos deben sumar 100%",IF(SUMPRODUCT((C4:C6&gt;0)*(1-ISNUMBER(B4:B6)))&gt;0,"NA: método con peso sin precio",SUMPRODUCT(B4:B6,C4:C6)))</f>
-        <v>35.9164595827377</v>
+        <v>35.9164596095943</v>
       </c>
       <c r="C9" s="238"/>
       <c r="D9" s="238"/>
@@ -21726,7 +21744,7 @@
       </c>
       <c r="B10" s="231" t="n">
         <f aca="false">Valuación!B42</f>
-        <v>33.48</v>
+        <v>30.25</v>
       </c>
       <c r="C10" s="238"/>
       <c r="D10" s="238"/>
@@ -21742,7 +21760,7 @@
       </c>
       <c r="B11" s="231" t="n">
         <f aca="false">B9-B10</f>
-        <v>2.43645958273775</v>
+        <v>5.66645960959431</v>
       </c>
       <c r="C11" s="238"/>
       <c r="D11" s="238"/>
@@ -21758,7 +21776,7 @@
       </c>
       <c r="B12" s="240" t="n">
         <f aca="false">B9/B10-1</f>
-        <v>0.0727735837137917</v>
+        <v>0.187320978829564</v>
       </c>
       <c r="C12" s="238"/>
       <c r="D12" s="238"/>
@@ -21785,7 +21803,7 @@
       </c>
       <c r="B14" s="231" t="n">
         <f aca="false">SUMPRODUCT(B4:B6,D4:D6)/D7</f>
-        <v>31.8592397579363</v>
+        <v>31.8592397758407</v>
       </c>
       <c r="C14" s="35"/>
       <c r="D14" s="35"/>
@@ -21842,15 +21860,15 @@
       </c>
       <c r="B18" s="231" t="n">
         <f aca="false">MIN(Validación!E9:G9)</f>
-        <v>37.9348536027754</v>
+        <v>37.934853657986</v>
       </c>
       <c r="C18" s="231" t="n">
         <f aca="false">B4</f>
-        <v>38.3400783109781</v>
+        <v>38.3400783646913</v>
       </c>
       <c r="D18" s="231" t="n">
         <f aca="false">MAX(Validación!E9:G9)</f>
-        <v>39.1434242577885</v>
+        <v>39.1434243086755</v>
       </c>
       <c r="E18" s="35"/>
       <c r="F18" s="35"/>
@@ -25512,7 +25530,7 @@
       </c>
       <c r="G50" s="120" t="n">
         <f aca="false">IFERROR(F50/'Valuación Combinada'!$B$10-1,"NM")</f>
-        <v>-0.848355366387893</v>
+        <v>-0.832163228650138</v>
       </c>
       <c r="H50" s="256" t="str">
         <f aca="false">IF(ISNUMBER(D50),IF(D50*Multiplos!$B$18+Multiplos!$B$30&gt;0,(D50*Multiplos!$B$18+Multiplos!$B$30)/Multiplos!$B$23,"NM"),"NA")</f>
@@ -25541,7 +25559,7 @@
       </c>
       <c r="G51" s="120" t="n">
         <f aca="false">IFERROR(F51/'Valuación Combinada'!$B$10-1,"NM")</f>
-        <v>-0.390239228021705</v>
+        <v>-0.325130887741047</v>
       </c>
       <c r="H51" s="256" t="n">
         <f aca="false">IF(ISNUMBER(D51),IF(D51*Multiplos!$B$18+Multiplos!$B$30&gt;0,(D51*Multiplos!$B$18+Multiplos!$B$30)/Multiplos!$B$23,"NM"),"NA")</f>
@@ -25570,7 +25588,7 @@
       </c>
       <c r="G52" s="120" t="n">
         <f aca="false">IFERROR(F52/'Valuación Combinada'!$B$10-1,"NM")</f>
-        <v>0.244753836494425</v>
+        <v>0.377664742011019</v>
       </c>
       <c r="H52" s="256" t="n">
         <f aca="false">IF(ISNUMBER(D52),IF(D52*Multiplos!$B$18+Multiplos!$B$30&gt;0,(D52*Multiplos!$B$18+Multiplos!$B$30)/Multiplos!$B$23,"NM"),"NA")</f>
@@ -25599,7 +25617,7 @@
       </c>
       <c r="G53" s="120" t="n">
         <f aca="false">IFERROR(F53/'Valuación Combinada'!$B$10-1,"NM")</f>
-        <v>-0.290776579798885</v>
+        <v>-0.21504793030303</v>
       </c>
       <c r="H53" s="256" t="n">
         <f aca="false">IF(ISNUMBER(D53),IF(D53*Multiplos!$B$18+Multiplos!$B$30&gt;0,(D53*Multiplos!$B$18+Multiplos!$B$30)/Multiplos!$B$23,"NM"),"NA")</f>
@@ -25628,7 +25646,7 @@
       </c>
       <c r="G54" s="120" t="n">
         <f aca="false">IFERROR(F54/'Valuación Combinada'!$B$10-1,"NM")</f>
-        <v>0.469157249726205</v>
+        <v>0.626029246969697</v>
       </c>
       <c r="H54" s="256" t="n">
         <f aca="false">IF(ISNUMBER(D54),IF(D54*Multiplos!$B$18+Multiplos!$B$30&gt;0,(D54*Multiplos!$B$18+Multiplos!$B$30)/Multiplos!$B$23,"NM"),"NA")</f>
@@ -25657,7 +25675,7 @@
       </c>
       <c r="G55" s="120" t="n">
         <f aca="false">IFERROR(F55/'Valuación Combinada'!$B$10-1,"NM")</f>
-        <v>2.89692780117483</v>
+        <v>3.31302951349862</v>
       </c>
       <c r="H55" s="256" t="n">
         <f aca="false">IF(ISNUMBER(D55),IF(D55*Multiplos!$B$18+Multiplos!$B$30&gt;0,(D55*Multiplos!$B$18+Multiplos!$B$30)/Multiplos!$B$23,"NM"),"NA")</f>
@@ -25754,7 +25772,7 @@
       </c>
       <c r="G60" s="120" t="n">
         <f aca="false">IFERROR(F60/'Valuación Combinada'!$B$10-1,"NM")</f>
-        <v>-0.13412815845992</v>
+        <v>-0.0416730824872101</v>
       </c>
       <c r="H60" s="256" t="n">
         <f aca="false">IF(ISNUMBER(D60),IF(D60*Multiplos!$B$18+Multiplos!$B$30&gt;0,(D60*Multiplos!$B$18+Multiplos!$B$30)/Multiplos!$B$23,"NM"),"NA")</f>
@@ -25783,7 +25801,7 @@
       </c>
       <c r="G61" s="120" t="n">
         <f aca="false">IFERROR(F61/'Valuación Combinada'!$B$10-1,"NM")</f>
-        <v>-0.303515638191955</v>
+        <v>-0.229147225344353</v>
       </c>
     </row>
     <row r="62" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -26089,11 +26107,11 @@
       </c>
       <c r="C85" s="256" t="n">
         <f aca="false">'Valuación Combinada'!B4</f>
-        <v>38.3400783109781</v>
+        <v>38.3400783646913</v>
       </c>
       <c r="D85" s="120" t="n">
         <f aca="false">C85/$C$93-1</f>
-        <v>0.145163629360159</v>
+        <v>0.267440607097232</v>
       </c>
       <c r="E85" s="36" t="s">
         <v>1203</v>
@@ -26109,7 +26127,7 @@
       </c>
       <c r="D86" s="120" t="n">
         <f aca="false">C86/$C$93-1</f>
-        <v>0.000383538067423972</v>
+        <v>0.107201350561896</v>
       </c>
       <c r="E86" s="36" t="s">
         <v>1204</v>
@@ -26125,7 +26143,7 @@
       </c>
       <c r="D87" s="120" t="n">
         <f aca="false">C87/$C$93-1</f>
-        <v>0.21649925826364</v>
+        <v>0.346393228650137</v>
       </c>
       <c r="E87" s="36" t="s">
         <v>1206</v>
@@ -26141,7 +26159,7 @@
       </c>
       <c r="D88" s="120" t="n">
         <f aca="false">C88/$C$93-1</f>
-        <v>-0.290776579798885</v>
+        <v>-0.21504793030303</v>
       </c>
       <c r="E88" s="36" t="s">
         <v>1208</v>
@@ -26157,7 +26175,7 @@
       </c>
       <c r="D89" s="120" t="n">
         <f aca="false">C89/$C$93-1</f>
-        <v>-0.13412815845992</v>
+        <v>-0.0416730824872101</v>
       </c>
       <c r="E89" s="36" t="s">
         <v>1210</v>
@@ -26173,7 +26191,7 @@
       </c>
       <c r="D90" s="120" t="n">
         <f aca="false">C90/$C$93-1</f>
-        <v>-0.302359617682198</v>
+        <v>-0.227867768595041</v>
       </c>
       <c r="E90" s="0" t="str">
         <f aca="false">"Expertos: "&amp;Comparativo!B19&amp;" — sesgo vendedor."</f>
@@ -26186,11 +26204,11 @@
       </c>
       <c r="C91" s="256" t="n">
         <f aca="false">'Valuación Combinada'!B9</f>
-        <v>35.9164595827377</v>
+        <v>35.9164596095943</v>
       </c>
       <c r="D91" s="120" t="n">
         <f aca="false">C91/$C$93-1</f>
-        <v>0.0727735837137917</v>
+        <v>0.187320978829564</v>
       </c>
       <c r="E91" s="36" t="s">
         <v>1213</v>
@@ -26202,11 +26220,11 @@
       </c>
       <c r="C92" s="256" t="n">
         <f aca="false">AVERAGE(C85,C86,C88)</f>
-        <v>31.8592397579363</v>
+        <v>31.8592397758407</v>
       </c>
       <c r="D92" s="120" t="n">
         <f aca="false">C92/$C$93-1</f>
-        <v>-0.0484098041237673</v>
+        <v>0.0531980091186992</v>
       </c>
       <c r="E92" s="36" t="s">
         <v>1215</v>
@@ -26218,7 +26236,7 @@
       </c>
       <c r="C93" s="256" t="n">
         <f aca="false">'Valuación Combinada'!B10</f>
-        <v>33.48</v>
+        <v>30.25</v>
       </c>
     </row>
     <row r="95" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -26259,7 +26277,7 @@
       </c>
       <c r="C98" s="261" t="n">
         <f aca="false">C91</f>
-        <v>35.9164595827377</v>
+        <v>35.9164596095943</v>
       </c>
     </row>
     <row r="99" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -26268,7 +26286,7 @@
       </c>
       <c r="C99" s="120" t="n">
         <f aca="false">C98/C93-1</f>
-        <v>0.0727735837137917</v>
+        <v>0.187320978829564</v>
       </c>
     </row>
     <row r="100" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -26304,7 +26322,7 @@
       </c>
       <c r="C103" s="256" t="n">
         <f aca="false">MAX(C85,C86,C89)</f>
-        <v>38.3400783109781</v>
+        <v>38.3400783646913</v>
       </c>
     </row>
     <row r="104" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -26418,26 +26436,26 @@
       </c>
       <c r="E5" s="263" t="n">
         <f aca="false">'Proyección Final Soriana'!B265</f>
-        <v>38.3400783109781</v>
+        <v>38.3400783646913</v>
       </c>
       <c r="F5" s="263" t="n">
         <f aca="false">'Valuación Combinada'!B18</f>
-        <v>37.9348536027754</v>
+        <v>37.934853657986</v>
       </c>
       <c r="G5" s="263" t="n">
         <f aca="false">'Valuación Combinada'!D18</f>
-        <v>39.1434242577885</v>
+        <v>39.1434243086755</v>
       </c>
       <c r="H5" s="263" t="n">
         <f aca="false">'Valuación Combinada'!B10</f>
-        <v>33.48</v>
+        <v>30.25</v>
       </c>
       <c r="I5" s="36" t="s">
         <v>1242</v>
       </c>
       <c r="J5" s="120" t="n">
         <f aca="false">IF(AND(ISNUMBER(E5),ISNUMBER(H5)),E5/H5-1,"NA")</f>
-        <v>0.145163629360159</v>
+        <v>0.267440607097232</v>
       </c>
       <c r="K5" s="36" t="s">
         <v>1243</v>
@@ -26463,7 +26481,7 @@
         <v>1247</v>
       </c>
       <c r="D6" s="0" t="s">
-        <v>1248</v>
+        <v>1242</v>
       </c>
       <c r="E6" s="263" t="n">
         <f aca="false">'Valuación Combinada'!B5</f>
@@ -26479,20 +26497,20 @@
       </c>
       <c r="H6" s="263" t="n">
         <f aca="false">'Valuación Combinada'!B10</f>
-        <v>33.48</v>
+        <v>30.25</v>
       </c>
       <c r="I6" s="36" t="s">
         <v>1242</v>
       </c>
       <c r="J6" s="120" t="n">
         <f aca="false">IF(AND(ISNUMBER(E6),ISNUMBER(H6)),E6/H6-1,"NA")</f>
-        <v>0.000383538067423972</v>
+        <v>0.107201350561896</v>
       </c>
       <c r="K6" s="36" t="s">
+        <v>1248</v>
+      </c>
+      <c r="L6" s="36" t="s">
         <v>1249</v>
-      </c>
-      <c r="L6" s="36" t="s">
-        <v>1250</v>
       </c>
       <c r="M6" s="36" t="s">
         <v>1245</v>
@@ -26503,16 +26521,16 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="0" t="s">
-        <v>1251</v>
+        <v>1250</v>
       </c>
       <c r="B7" s="0" t="s">
         <v>1239</v>
       </c>
       <c r="C7" s="0" t="s">
+        <v>1251</v>
+      </c>
+      <c r="D7" s="0" t="s">
         <v>1252</v>
-      </c>
-      <c r="D7" s="0" t="s">
-        <v>1253</v>
       </c>
       <c r="E7" s="263" t="n">
         <f aca="false">'Valuación Combinada'!B6</f>
@@ -26528,23 +26546,23 @@
       </c>
       <c r="H7" s="263" t="n">
         <f aca="false">'Valuación Combinada'!B10</f>
-        <v>33.48</v>
+        <v>30.25</v>
       </c>
       <c r="I7" s="36" t="s">
         <v>1242</v>
       </c>
       <c r="J7" s="120" t="n">
         <f aca="false">IF(AND(ISNUMBER(E7),ISNUMBER(H7)),E7/H7-1,"NA")</f>
-        <v>-0.290776579798885</v>
+        <v>-0.21504793030303</v>
       </c>
       <c r="K7" s="36" t="s">
+        <v>1253</v>
+      </c>
+      <c r="L7" s="36" t="s">
         <v>1254</v>
       </c>
-      <c r="L7" s="36" t="s">
+      <c r="M7" s="36" t="s">
         <v>1255</v>
-      </c>
-      <c r="M7" s="36" t="s">
-        <v>1256</v>
       </c>
       <c r="N7" s="36" t="s">
         <v>587</v>
@@ -26552,13 +26570,13 @@
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="0" t="s">
-        <v>1257</v>
+        <v>1256</v>
       </c>
       <c r="B8" s="0" t="s">
         <v>1239</v>
       </c>
       <c r="C8" s="0" t="s">
-        <v>1258</v>
+        <v>1257</v>
       </c>
       <c r="D8" s="0" t="s">
         <v>587</v>
@@ -26577,23 +26595,23 @@
       </c>
       <c r="H8" s="263" t="n">
         <f aca="false">'Valuación Combinada'!B10</f>
-        <v>33.48</v>
+        <v>30.25</v>
       </c>
       <c r="I8" s="36" t="s">
         <v>1242</v>
       </c>
       <c r="J8" s="120" t="n">
         <f aca="false">IF(AND(ISNUMBER(E8),ISNUMBER(H8)),E8/H8-1,"NA")</f>
-        <v>0.21649925826364</v>
+        <v>0.346393228650137</v>
       </c>
       <c r="K8" s="36" t="s">
+        <v>1258</v>
+      </c>
+      <c r="L8" s="36" t="s">
         <v>1259</v>
       </c>
-      <c r="L8" s="36" t="s">
+      <c r="M8" s="36" t="s">
         <v>1260</v>
-      </c>
-      <c r="M8" s="36" t="s">
-        <v>1261</v>
       </c>
       <c r="N8" s="36" t="s">
         <v>587</v>
@@ -26601,40 +26619,40 @@
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="0" t="s">
-        <v>1262</v>
+        <v>1261</v>
       </c>
       <c r="B9" s="0" t="s">
         <v>1239</v>
       </c>
       <c r="C9" s="0" t="s">
-        <v>1263</v>
+        <v>1262</v>
       </c>
       <c r="D9" s="0" t="s">
         <v>1241</v>
       </c>
       <c r="E9" s="263" t="n">
         <f aca="false">'Valuación Combinada'!B9</f>
-        <v>35.9164595827377</v>
+        <v>35.9164596095943</v>
       </c>
       <c r="H9" s="263" t="n">
         <f aca="false">'Valuación Combinada'!B10</f>
-        <v>33.48</v>
+        <v>30.25</v>
       </c>
       <c r="I9" s="36" t="s">
         <v>1242</v>
       </c>
       <c r="J9" s="120" t="n">
         <f aca="false">IF(AND(ISNUMBER(E9),ISNUMBER(H9)),E9/H9-1,"NA")</f>
-        <v>0.0727735837137917</v>
+        <v>0.187320978829564</v>
       </c>
       <c r="K9" s="36" t="s">
-        <v>1264</v>
+        <v>1263</v>
       </c>
       <c r="L9" s="36" t="s">
         <v>587</v>
       </c>
       <c r="M9" s="36" t="s">
-        <v>1265</v>
+        <v>1264</v>
       </c>
       <c r="N9" s="36" t="s">
         <v>587</v>
@@ -26642,16 +26660,16 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="0" t="s">
+        <v>1265</v>
+      </c>
+      <c r="B10" s="0" t="s">
         <v>1266</v>
-      </c>
-      <c r="B10" s="0" t="s">
-        <v>1267</v>
       </c>
       <c r="C10" s="0" t="s">
         <v>990</v>
       </c>
       <c r="D10" s="0" t="s">
-        <v>1268</v>
+        <v>1267</v>
       </c>
       <c r="E10" s="264" t="n">
         <v>39.21</v>
@@ -26666,37 +26684,37 @@
         <v>33.1</v>
       </c>
       <c r="I10" s="36" t="s">
-        <v>1268</v>
+        <v>1267</v>
       </c>
       <c r="J10" s="120" t="n">
         <f aca="false">IF(AND(ISNUMBER(E10),ISNUMBER(H10)),E10/H10-1,"NA")</f>
         <v>0.184592145015106</v>
       </c>
       <c r="K10" s="36" t="s">
+        <v>1268</v>
+      </c>
+      <c r="L10" s="36" t="s">
         <v>1269</v>
       </c>
-      <c r="L10" s="36" t="s">
+      <c r="M10" s="36" t="s">
         <v>1270</v>
       </c>
-      <c r="M10" s="36" t="s">
+      <c r="N10" s="36" t="s">
         <v>1271</v>
-      </c>
-      <c r="N10" s="36" t="s">
-        <v>1272</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="0" t="s">
+        <v>1272</v>
+      </c>
+      <c r="B11" s="0" t="s">
         <v>1273</v>
       </c>
-      <c r="B11" s="0" t="s">
+      <c r="C11" s="0" t="s">
         <v>1274</v>
       </c>
-      <c r="C11" s="0" t="s">
-        <v>1275</v>
-      </c>
       <c r="D11" s="0" t="s">
-        <v>1268</v>
+        <v>1267</v>
       </c>
       <c r="E11" s="264" t="n">
         <v>36.35</v>
@@ -26705,31 +26723,31 @@
         <v>33.1</v>
       </c>
       <c r="I11" s="36" t="s">
-        <v>1268</v>
+        <v>1267</v>
       </c>
       <c r="J11" s="120" t="n">
         <f aca="false">IF(AND(ISNUMBER(E11),ISNUMBER(H11)),E11/H11-1,"NA")</f>
         <v>0.0981873111782476</v>
       </c>
       <c r="K11" s="36" t="s">
-        <v>1264</v>
+        <v>1263</v>
       </c>
       <c r="L11" s="36" t="s">
+        <v>1275</v>
+      </c>
+      <c r="M11" s="36" t="s">
         <v>1276</v>
       </c>
-      <c r="M11" s="36" t="s">
+      <c r="N11" s="36" t="s">
         <v>1277</v>
-      </c>
-      <c r="N11" s="36" t="s">
-        <v>1278</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="0" t="s">
+        <v>1278</v>
+      </c>
+      <c r="B12" s="0" t="s">
         <v>1279</v>
-      </c>
-      <c r="B12" s="0" t="s">
-        <v>1280</v>
       </c>
       <c r="C12" s="0" t="s">
         <v>990</v>
@@ -26750,7 +26768,7 @@
         <v>33.48</v>
       </c>
       <c r="I12" s="36" t="s">
-        <v>1242</v>
+        <v>1280</v>
       </c>
       <c r="J12" s="120" t="n">
         <f aca="false">IF(AND(ISNUMBER(E12),ISNUMBER(H12)),E12/H12-1,"NA")</f>
@@ -26763,7 +26781,7 @@
         <v>1282</v>
       </c>
       <c r="M12" s="36" t="s">
-        <v>1261</v>
+        <v>1260</v>
       </c>
       <c r="N12" s="36" t="s">
         <v>1283</v>
@@ -26780,7 +26798,7 @@
         <v>1286</v>
       </c>
       <c r="D13" s="0" t="s">
-        <v>1253</v>
+        <v>1252</v>
       </c>
       <c r="E13" s="264" t="n">
         <v>38.27</v>
@@ -26795,7 +26813,7 @@
         <v>33.1</v>
       </c>
       <c r="I13" s="36" t="s">
-        <v>1268</v>
+        <v>1267</v>
       </c>
       <c r="J13" s="120" t="n">
         <f aca="false">IF(AND(ISNUMBER(E13),ISNUMBER(H13)),E13/H13-1,"NA")</f>
@@ -26808,7 +26826,7 @@
         <v>1288</v>
       </c>
       <c r="M13" s="36" t="s">
-        <v>1277</v>
+        <v>1276</v>
       </c>
       <c r="N13" s="36" t="s">
         <v>1289</v>
@@ -26825,7 +26843,7 @@
         <v>1292</v>
       </c>
       <c r="D14" s="0" t="s">
-        <v>1253</v>
+        <v>1252</v>
       </c>
       <c r="E14" s="264" t="n">
         <v>29.7</v>
@@ -26840,7 +26858,7 @@
         <v>33.1</v>
       </c>
       <c r="I14" s="36" t="s">
-        <v>1268</v>
+        <v>1267</v>
       </c>
       <c r="J14" s="120" t="n">
         <f aca="false">IF(AND(ISNUMBER(E14),ISNUMBER(H14)),E14/H14-1,"NA")</f>
@@ -26853,7 +26871,7 @@
         <v>1294</v>
       </c>
       <c r="M14" s="36" t="s">
-        <v>1277</v>
+        <v>1276</v>
       </c>
       <c r="N14" s="36" t="s">
         <v>1295</v>
@@ -26870,7 +26888,7 @@
         <v>1297</v>
       </c>
       <c r="D15" s="0" t="s">
-        <v>1253</v>
+        <v>1252</v>
       </c>
       <c r="E15" s="264" t="n">
         <v>28.54</v>
@@ -26885,7 +26903,7 @@
         <v>33.1</v>
       </c>
       <c r="I15" s="36" t="s">
-        <v>1268</v>
+        <v>1267</v>
       </c>
       <c r="J15" s="120" t="n">
         <f aca="false">IF(AND(ISNUMBER(E15),ISNUMBER(H15)),E15/H15-1,"NA")</f>
@@ -26898,7 +26916,7 @@
         <v>1299</v>
       </c>
       <c r="M15" s="36" t="s">
-        <v>1277</v>
+        <v>1276</v>
       </c>
       <c r="N15" s="36" t="s">
         <v>1300</v>
@@ -26915,7 +26933,7 @@
         <v>1302</v>
       </c>
       <c r="D16" s="0" t="s">
-        <v>1253</v>
+        <v>1252</v>
       </c>
       <c r="E16" s="264" t="n">
         <v>33.98</v>
@@ -26924,7 +26942,7 @@
         <v>33.1</v>
       </c>
       <c r="I16" s="36" t="s">
-        <v>1268</v>
+        <v>1267</v>
       </c>
       <c r="J16" s="120" t="n">
         <f aca="false">IF(AND(ISNUMBER(E16),ISNUMBER(H16)),E16/H16-1,"NA")</f>
@@ -26937,7 +26955,7 @@
         <v>1304</v>
       </c>
       <c r="M16" s="36" t="s">
-        <v>1277</v>
+        <v>1276</v>
       </c>
       <c r="N16" s="36" t="s">
         <v>1305</v>
@@ -26954,7 +26972,7 @@
         <v>1307</v>
       </c>
       <c r="D17" s="0" t="s">
-        <v>1253</v>
+        <v>1252</v>
       </c>
       <c r="E17" s="264" t="n">
         <v>23.36</v>
@@ -26969,7 +26987,7 @@
         <v>33.1</v>
       </c>
       <c r="I17" s="36" t="s">
-        <v>1268</v>
+        <v>1267</v>
       </c>
       <c r="J17" s="120" t="n">
         <f aca="false">IF(AND(ISNUMBER(E17),ISNUMBER(H17)),E17/H17-1,"NA")</f>
@@ -26982,7 +27000,7 @@
         <v>1309</v>
       </c>
       <c r="M17" s="36" t="s">
-        <v>1277</v>
+        <v>1276</v>
       </c>
       <c r="N17" s="36" t="s">
         <v>1310</v>
@@ -26999,7 +27017,7 @@
         <v>1307</v>
       </c>
       <c r="D18" s="0" t="s">
-        <v>1253</v>
+        <v>1252</v>
       </c>
       <c r="E18" s="264" t="n">
         <v>22.42</v>
@@ -27008,7 +27026,7 @@
         <v>33.1</v>
       </c>
       <c r="I18" s="36" t="s">
-        <v>1268</v>
+        <v>1267</v>
       </c>
       <c r="J18" s="120" t="n">
         <f aca="false">IF(AND(ISNUMBER(E18),ISNUMBER(H18)),E18/H18-1,"NA")</f>
@@ -27021,7 +27039,7 @@
         <v>1314</v>
       </c>
       <c r="M18" s="36" t="s">
-        <v>1277</v>
+        <v>1276</v>
       </c>
       <c r="N18" s="36" t="s">
         <v>1315</v>
@@ -27038,7 +27056,7 @@
         <v>1318</v>
       </c>
       <c r="D19" s="0" t="s">
-        <v>1253</v>
+        <v>1252</v>
       </c>
       <c r="E19" s="264" t="n">
         <v>51</v>
@@ -27053,7 +27071,7 @@
         <v>33.1</v>
       </c>
       <c r="I19" s="36" t="s">
-        <v>1268</v>
+        <v>1267</v>
       </c>
       <c r="J19" s="120" t="n">
         <f aca="false">IF(AND(ISNUMBER(E19),ISNUMBER(H19)),E19/H19-1,"NA")</f>
@@ -27066,7 +27084,7 @@
         <v>1320</v>
       </c>
       <c r="M19" s="36" t="s">
-        <v>1277</v>
+        <v>1276</v>
       </c>
       <c r="N19" s="36" t="s">
         <v>1321</v>
@@ -27226,22 +27244,22 @@
         <v>1341</v>
       </c>
       <c r="C9" s="266" t="n">
-        <v>30.9318856931226</v>
+        <v>30.9318859027253</v>
       </c>
       <c r="D9" s="266" t="n">
-        <v>38.8228171407462</v>
+        <v>38.8228171926553</v>
       </c>
       <c r="E9" s="266" t="n">
-        <v>37.9348536027754</v>
+        <v>37.934853657986</v>
       </c>
       <c r="F9" s="266" t="n">
-        <v>38.3400783109781</v>
+        <v>38.3400783646913</v>
       </c>
       <c r="G9" s="266" t="n">
-        <v>39.1434242577885</v>
+        <v>39.1434243086755</v>
       </c>
       <c r="H9" s="266" t="n">
-        <v>31.6168901445216</v>
+        <v>31.6168903219841</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -27252,22 +27270,22 @@
         <v>1342</v>
       </c>
       <c r="C10" s="267" t="n">
-        <v>55677.3942476206</v>
+        <v>55677.3946249056</v>
       </c>
       <c r="D10" s="267" t="n">
-        <v>69881.0708533432</v>
+        <v>69881.0709467796</v>
       </c>
       <c r="E10" s="267" t="n">
-        <v>68282.7364849957</v>
+        <v>68282.7365843747</v>
       </c>
       <c r="F10" s="267" t="n">
-        <v>69012.1409597606</v>
+        <v>69012.1410564443</v>
       </c>
       <c r="G10" s="267" t="n">
-        <v>70458.1636640194</v>
+        <v>70458.1637556159</v>
       </c>
       <c r="H10" s="267" t="n">
-        <v>56910.4022601389</v>
+        <v>56910.4025795714</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -27278,22 +27296,22 @@
         <v>1343</v>
       </c>
       <c r="C11" s="267" t="n">
-        <v>65877.1203514794</v>
+        <v>65877.120705858</v>
       </c>
       <c r="D11" s="267" t="n">
-        <v>80190.5010810303</v>
+        <v>80190.5011714968</v>
       </c>
       <c r="E11" s="267" t="n">
-        <v>78704.5866448527</v>
+        <v>78704.5867410738</v>
       </c>
       <c r="F11" s="267" t="n">
-        <v>79382.6971683179</v>
+        <v>79382.6972619287</v>
       </c>
       <c r="G11" s="267" t="n">
-        <v>80727.0213270136</v>
+        <v>80727.0214156981</v>
       </c>
       <c r="H11" s="267" t="n">
-        <v>67198.4289751488</v>
+        <v>67198.4292769918</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -27304,22 +27322,22 @@
         <v>1344</v>
       </c>
       <c r="C12" s="268" t="n">
-        <v>0.117703264055937</v>
+        <v>0.117703263356543</v>
       </c>
       <c r="D12" s="268" t="n">
-        <v>0.0956853555538548</v>
+        <v>0.0956853554465444</v>
       </c>
       <c r="E12" s="268" t="n">
-        <v>0.0955790842123724</v>
+        <v>0.0955790840960861</v>
       </c>
       <c r="F12" s="268" t="n">
-        <v>0.0956277841268195</v>
+        <v>0.0956277840146585</v>
       </c>
       <c r="G12" s="268" t="n">
-        <v>0.0957222086238604</v>
+        <v>0.0957222085193786</v>
       </c>
       <c r="H12" s="268" t="n">
-        <v>0.113837026578705</v>
+        <v>0.113837026020324</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -27330,22 +27348,22 @@
         <v>1345</v>
       </c>
       <c r="C13" s="268" t="n">
-        <v>0.140162655262051</v>
+        <v>0.140162656276711</v>
       </c>
       <c r="D13" s="268" t="n">
-        <v>0.104021768141081</v>
+        <v>0.104021768175859</v>
       </c>
       <c r="E13" s="268" t="n">
-        <v>0.104056387187952</v>
+        <v>0.10405638722603</v>
       </c>
       <c r="F13" s="268" t="n">
-        <v>0.104040478277405</v>
+        <v>0.104040478313958</v>
       </c>
       <c r="G13" s="268" t="n">
-        <v>0.10400984596747</v>
+        <v>0.10400984600121</v>
       </c>
       <c r="H13" s="268" t="n">
-        <v>0.133539746416858</v>
+        <v>0.133539747123327</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -27356,22 +27374,22 @@
         <v>1346</v>
       </c>
       <c r="C14" s="155" t="n">
-        <v>1.06365615276715</v>
+        <v>1.06365617675439</v>
       </c>
       <c r="D14" s="155" t="n">
-        <v>0.209261658181595</v>
+        <v>0.209261659003758</v>
       </c>
       <c r="E14" s="155" t="n">
-        <v>0.210080075365293</v>
+        <v>0.210080076265473</v>
       </c>
       <c r="F14" s="155" t="n">
-        <v>0.209703978189233</v>
+        <v>0.209703979053375</v>
       </c>
       <c r="G14" s="155" t="n">
-        <v>0.208979810105667</v>
+        <v>0.208979810903308</v>
       </c>
       <c r="H14" s="155" t="n">
-        <v>0.907086203708222</v>
+        <v>0.907086220409621</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -27382,22 +27400,22 @@
         <v>1347</v>
       </c>
       <c r="C15" s="268" t="n">
-        <v>0.125008009155719</v>
+        <v>0.124709966746939</v>
       </c>
       <c r="D15" s="268" t="n">
-        <v>0.100630184051038</v>
+        <v>0.10049964337765</v>
       </c>
       <c r="E15" s="268" t="n">
-        <v>0.100630184051038</v>
+        <v>0.10049964337765</v>
       </c>
       <c r="F15" s="268" t="n">
-        <v>0.100630184051038</v>
+        <v>0.10049964337765</v>
       </c>
       <c r="G15" s="268" t="n">
-        <v>0.100630184051038</v>
+        <v>0.10049964337765</v>
       </c>
       <c r="H15" s="268" t="n">
-        <v>0.120748041823037</v>
+        <v>0.120479269946713</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -27408,22 +27426,22 @@
         <v>1348</v>
       </c>
       <c r="C16" s="268" t="n">
-        <v>0.138293538829152</v>
+        <v>0.139284805950413</v>
       </c>
       <c r="D16" s="268" t="n">
-        <v>0.104361826273881</v>
+        <v>0.104573115871559</v>
       </c>
       <c r="E16" s="268" t="n">
-        <v>0.104361826273881</v>
+        <v>0.104573115871559</v>
       </c>
       <c r="F16" s="268" t="n">
-        <v>0.104361826273881</v>
+        <v>0.104573115871559</v>
       </c>
       <c r="G16" s="268" t="n">
-        <v>0.104361826273881</v>
+        <v>0.104573115871559</v>
       </c>
       <c r="H16" s="268" t="n">
-        <v>0.132364052240143</v>
+        <v>0.133219020132231</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -27486,22 +27504,22 @@
         <v>1353</v>
       </c>
       <c r="C19" s="266" t="n">
-        <v>32.21236327381</v>
+        <v>32.2123633786113</v>
       </c>
       <c r="D19" s="266" t="n">
-        <v>36.1578289976218</v>
+        <v>36.1578290235764</v>
       </c>
       <c r="E19" s="266" t="n">
-        <v>35.7138472286364</v>
+        <v>35.7138472562417</v>
       </c>
       <c r="F19" s="266" t="n">
-        <v>35.9164595827377</v>
+        <v>35.9164596095943</v>
       </c>
       <c r="G19" s="266" t="n">
-        <v>36.3181325561429</v>
+        <v>36.3181325815864</v>
       </c>
       <c r="H19" s="266" t="n">
-        <v>32.5548654995095</v>
+        <v>32.5548655882407</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -27573,7 +27591,7 @@
       </c>
       <c r="B24" s="269" t="n">
         <f aca="false">'Proyección Final Soriana'!B126-'Proyección Final Soriana'!B123</f>
-        <v>0.0606277841268195</v>
+        <v>0.0606277840146585</v>
       </c>
       <c r="C24" s="269" t="s">
         <v>1362</v>
@@ -27592,14 +27610,14 @@
       </c>
       <c r="B25" s="269" t="n">
         <f aca="false">ABS('Proyección Final Soriana'!G219-'Proyección Final Soriana'!G218)</f>
-        <v>4.8664896321049E-008</v>
+        <v>4.74056967569858E-008</v>
       </c>
       <c r="C25" s="269" t="n">
         <v>0</v>
       </c>
       <c r="D25" s="270" t="n">
         <f aca="false">IF(AND(ISNUMBER(B25),ISNUMBER(C25)),B25-C25,"n/a")</f>
-        <v>4.8664896321049E-008</v>
+        <v>4.74056967569858E-008</v>
       </c>
       <c r="E25" s="0" t="n">
         <v>1E-006</v>
@@ -27618,11 +27636,11 @@
       </c>
       <c r="B26" s="269" t="n">
         <f aca="false">'Proyección Final Soriana'!B134</f>
-        <v>23547.3812562396</v>
+        <v>23547.3812632515</v>
       </c>
       <c r="C26" s="269" t="n">
         <f aca="false">SUMPRODUCT('Proyección Final Soriana'!C117:G117,'Proyección Final Soriana'!C119:G119)</f>
-        <v>23547.3812562396</v>
+        <v>23547.3812632515</v>
       </c>
       <c r="D26" s="270" t="n">
         <f aca="false">IF(AND(ISNUMBER(B26),ISNUMBER(C26)),B26-C26,"n/a")</f>
@@ -27645,11 +27663,11 @@
       </c>
       <c r="B27" s="269" t="n">
         <f aca="false">'Proyección Final Soriana'!G119</f>
-        <v>0.633409853102093</v>
+        <v>0.633409853426309</v>
       </c>
       <c r="C27" s="269" t="n">
         <f aca="false">1/(1+'Proyección Final Soriana'!B126)^5</f>
-        <v>0.633409853102093</v>
+        <v>0.633409853426309</v>
       </c>
       <c r="D27" s="270" t="n">
         <f aca="false">IF(AND(ISNUMBER(B27),ISNUMBER(C27)),B27-C27,"n/a")</f>
@@ -27672,11 +27690,11 @@
       </c>
       <c r="B28" s="269" t="n">
         <f aca="false">'Proyección Final Soriana'!B129</f>
-        <v>99025.313510992</v>
+        <v>99025.3136941883</v>
       </c>
       <c r="C28" s="269" t="n">
         <f aca="false">('Proyección Final Soriana'!G73*(1-'Proyección Final Soriana'!G55)+'Proyección Final Soriana'!G116)*(1+'Proyección Final Soriana'!B123)/('Proyección Final Soriana'!B126-'Proyección Final Soriana'!B123)</f>
-        <v>99025.3135109921</v>
+        <v>99025.3136941883</v>
       </c>
       <c r="D28" s="270" t="n">
         <f aca="false">IF(AND(ISNUMBER(B28),ISNUMBER(C28)),B28-C28,"n/a")</f>
@@ -27726,11 +27744,11 @@
       </c>
       <c r="B30" s="269" t="n">
         <f aca="false">'Proyección Final Soriana'!B262</f>
-        <v>67306.9403540494</v>
+        <v>67306.9404477808</v>
       </c>
       <c r="C30" s="269" t="n">
         <f aca="false">'Proyección Final Soriana'!B258-(Datos!F25+Datos!F26)-(Datos!F27+Datos!F28)+Datos!F17</f>
-        <v>67306.9403540494</v>
+        <v>67306.9404477808</v>
       </c>
       <c r="D30" s="270" t="n">
         <f aca="false">IF(AND(ISNUMBER(B30),ISNUMBER(C30)),B30-C30,"n/a")</f>
@@ -27780,11 +27798,11 @@
       </c>
       <c r="B32" s="269" t="n">
         <f aca="false">'Proyección Final Soriana'!B265</f>
-        <v>38.3400783109781</v>
+        <v>38.3400783646913</v>
       </c>
       <c r="C32" s="269" t="n">
         <f aca="false">'Proyección Final Soriana'!B263/WACC!B17</f>
-        <v>38.3400783109781</v>
+        <v>38.3400783646913</v>
       </c>
       <c r="D32" s="270" t="n">
         <f aca="false">IF(AND(ISNUMBER(B32),ISNUMBER(C32)),B32-C32,"n/a")</f>
@@ -27807,11 +27825,11 @@
       </c>
       <c r="B33" s="269" t="n">
         <f aca="false">'Proyección Final Soriana'!B265</f>
-        <v>38.3400783109781</v>
+        <v>38.3400783646913</v>
       </c>
       <c r="C33" s="269" t="n">
         <f aca="false">IF(AND(Inflación!$E$6=0,'Beta y Kd'!$B$18=0),C9,IF(AND(Inflación!$E$6=0,'Beta y Kd'!$B$18=2),D9,IF(AND(Inflación!$E$6=1,'Beta y Kd'!$B$18=2),E9,IF(AND(Inflación!$E$6=2,'Beta y Kd'!$B$18=2),F9,IF(AND(Inflación!$E$6=3,'Beta y Kd'!$B$18=2),G9,IF(AND(Inflación!$E$6=2,'Beta y Kd'!$B$18=1),H9,"sin registro"))))))</f>
-        <v>38.3400783109781</v>
+        <v>38.3400783646913</v>
       </c>
       <c r="D33" s="270" t="n">
         <f aca="false">IF(AND(ISNUMBER(B33),ISNUMBER(C33)),B33-C33,"n/a")</f>
@@ -27834,14 +27852,14 @@
       </c>
       <c r="B34" s="269" t="n">
         <f aca="false">C9</f>
-        <v>30.9318856931226</v>
+        <v>30.9318859027253</v>
       </c>
       <c r="C34" s="269" t="n">
         <v>30.9318856931226</v>
       </c>
       <c r="D34" s="270" t="n">
         <f aca="false">IF(AND(ISNUMBER(B34),ISNUMBER(C34)),B34-C34,"n/a")</f>
-        <v>0</v>
+        <v>2.09602699641209E-007</v>
       </c>
       <c r="E34" s="0" t="n">
         <v>1E-006</v>
@@ -27940,11 +27958,11 @@
       </c>
       <c r="B38" s="269" t="n">
         <f aca="false">WACC!B28</f>
-        <v>0.21730085753856</v>
+        <v>0.222295883488385</v>
       </c>
       <c r="C38" s="269" t="n">
         <f aca="false">WACC!B9*(1+(1-WACC!B10)*WACC!B23)</f>
-        <v>0.21730085753856</v>
+        <v>0.222295883488385</v>
       </c>
       <c r="D38" s="270" t="n">
         <f aca="false">IF(AND(ISNUMBER(B38),ISNUMBER(C38)),B38-C38,"n/a")</f>
@@ -27967,11 +27985,11 @@
       </c>
       <c r="B39" s="269" t="n">
         <f aca="false">'Proyección Final Soriana'!E219</f>
-        <v>0.209703978189233</v>
+        <v>0.209703979053375</v>
       </c>
       <c r="C39" s="269" t="n">
         <f aca="false">'Proyección Final Soriana'!B212*(1+(1-'Proyección Final Soriana'!B207)*'Proyección Final Soriana'!B209/'Proyección Final Soriana'!C219)</f>
-        <v>0.209703978189233</v>
+        <v>0.209703979053375</v>
       </c>
       <c r="D39" s="270" t="n">
         <f aca="false">IF(AND(ISNUMBER(B39),ISNUMBER(C39)),B39-C39,"n/a")</f>
@@ -27994,11 +28012,11 @@
       </c>
       <c r="B40" s="269" t="n">
         <f aca="false">'Proyección Final Soriana'!F219</f>
-        <v>0.104040478277405</v>
+        <v>0.104040478313958</v>
       </c>
       <c r="C40" s="269" t="n">
         <f aca="false">'Proyección Final Soriana'!B210+'Proyección Final Soriana'!E219*'Proyección Final Soriana'!B211</f>
-        <v>0.104040478277405</v>
+        <v>0.104040478313958</v>
       </c>
       <c r="D40" s="270" t="n">
         <f aca="false">IF(AND(ISNUMBER(B40),ISNUMBER(C40)),B40-C40,"n/a")</f>
@@ -28445,11 +28463,11 @@
       </c>
       <c r="B57" s="269" t="n">
         <f aca="false">'Valuación Combinada'!B9</f>
-        <v>35.9164595827377</v>
+        <v>35.9164596095943</v>
       </c>
       <c r="C57" s="269" t="n">
         <f aca="false">'Valuación Combinada'!B4*'Valuación Combinada'!C4+'Valuación Combinada'!B5*'Valuación Combinada'!C5+IF(ISNUMBER('Valuación Combinada'!B6),'Valuación Combinada'!B6*'Valuación Combinada'!C6,0)</f>
-        <v>35.9164595827377</v>
+        <v>35.9164596095943</v>
       </c>
       <c r="D57" s="270" t="n">
         <f aca="false">IF(AND(ISNUMBER(B57),ISNUMBER(C57)),B57-C57,"n/a")</f>
@@ -28818,11 +28836,11 @@
       </c>
       <c r="B71" s="121" t="n">
         <f aca="false">'Proyección Final Soriana'!D277</f>
-        <v>38.3400783109781</v>
+        <v>38.3400783646913</v>
       </c>
       <c r="C71" s="274" t="n">
         <f aca="false">'Proyección Final Soriana'!B265</f>
-        <v>38.3400783109781</v>
+        <v>38.3400783646913</v>
       </c>
       <c r="D71" s="36" t="n">
         <f aca="false">IF(AND(ISNUMBER(B71),ISNUMBER(C71)),B71-C71,"n/a")</f>
@@ -28951,7 +28969,7 @@
         <v>1468</v>
       </c>
       <c r="D6" s="132" t="s">
-        <v>1268</v>
+        <v>1267</v>
       </c>
       <c r="E6" s="132" t="s">
         <v>1469</v>
@@ -28974,7 +28992,7 @@
         <v>1474</v>
       </c>
       <c r="D7" s="132" t="s">
-        <v>1268</v>
+        <v>1267</v>
       </c>
       <c r="E7" s="132" t="s">
         <v>1469</v>
@@ -28997,7 +29015,7 @@
         <v>1478</v>
       </c>
       <c r="D8" s="132" t="s">
-        <v>1268</v>
+        <v>1267</v>
       </c>
       <c r="E8" s="132" t="s">
         <v>1469</v>
@@ -29136,7 +29154,7 @@
         <v>1507</v>
       </c>
       <c r="D14" s="277" t="s">
-        <v>1242</v>
+        <v>1280</v>
       </c>
       <c r="E14" s="132" t="s">
         <v>1469</v>
@@ -29205,7 +29223,7 @@
         <v>1519</v>
       </c>
       <c r="D17" s="132" t="s">
-        <v>1248</v>
+        <v>1242</v>
       </c>
       <c r="E17" s="132" t="s">
         <v>1494</v>
@@ -29251,7 +29269,7 @@
         <v>1528</v>
       </c>
       <c r="D19" s="132" t="s">
-        <v>1248</v>
+        <v>1242</v>
       </c>
       <c r="E19" s="132" t="s">
         <v>1529</v>
@@ -29297,7 +29315,7 @@
         <v>1537</v>
       </c>
       <c r="D21" s="248" t="s">
-        <v>1253</v>
+        <v>1252</v>
       </c>
       <c r="E21" s="248" t="s">
         <v>1538</v>
@@ -29320,7 +29338,7 @@
         <v>1542</v>
       </c>
       <c r="D22" s="248" t="s">
-        <v>1253</v>
+        <v>1252</v>
       </c>
       <c r="E22" s="248" t="s">
         <v>1543</v>
@@ -29517,7 +29535,7 @@
       </c>
       <c r="B12" s="16" t="n">
         <f aca="false">WACC!B18</f>
-        <v>60264</v>
+        <v>54450</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -29914,7 +29932,7 @@
       </c>
       <c r="B56" s="10" t="n">
         <f aca="false">WACC!B13/(Datos!G13/WACC!B17)</f>
-        <v>18.0755848830234</v>
+        <v>16.3317336532693</v>
       </c>
     </row>
     <row r="57" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -29932,7 +29950,7 @@
       </c>
       <c r="B58" s="10" t="n">
         <f aca="false">WACC!B13/B57</f>
-        <v>0.711230703866308</v>
+        <v>0.642614360572157</v>
       </c>
     </row>
     <row r="59" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -29977,7 +29995,7 @@
       </c>
       <c r="B63" s="4" t="n">
         <f aca="false">B62/WACC!B13</f>
-        <v>0.016594982078853</v>
+        <v>0.0183669421487603</v>
       </c>
     </row>
     <row r="64" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -30073,7 +30091,7 @@
       </c>
       <c r="B74" s="22" t="n">
         <f aca="false">B24/WACC!B13-1</f>
-        <v>-0.302359617682198</v>
+        <v>-0.227867768595041</v>
       </c>
     </row>
     <row r="75" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -30109,7 +30127,7 @@
       </c>
       <c r="B78" s="6" t="n">
         <f aca="false">WACC!B13</f>
-        <v>33.48</v>
+        <v>30.25</v>
       </c>
     </row>
     <row r="79" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -30196,7 +30214,7 @@
       </c>
       <c r="B89" s="6" t="n">
         <f aca="false">WACC!B13</f>
-        <v>33.48</v>
+        <v>30.25</v>
       </c>
       <c r="C89" s="6" t="n">
         <f aca="false">WACC!C13</f>
@@ -30217,7 +30235,7 @@
       </c>
       <c r="B90" s="10" t="n">
         <f aca="false">B56</f>
-        <v>18.0755848830234</v>
+        <v>16.3317336532693</v>
       </c>
       <c r="C90" s="10" t="n">
         <f aca="false">WACC!C13/(Datos!G39/WACC!C17)</f>
@@ -30238,7 +30256,7 @@
       </c>
       <c r="B91" s="11" t="n">
         <f aca="false">B63</f>
-        <v>0.016594982078853</v>
+        <v>0.0183669421487603</v>
       </c>
       <c r="C91" s="11" t="n">
         <v>0.0253</v>
@@ -30391,7 +30409,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:G20"/>
+  <dimension ref="A1:G21"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="4"/>
@@ -30781,7 +30799,7 @@
         <v>1630</v>
       </c>
     </row>
-    <row r="20" customFormat="false" ht="55.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="20" customFormat="false" ht="68.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="0" t="n">
         <v>16</v>
       </c>
@@ -30802,6 +30820,29 @@
       </c>
       <c r="G20" s="132" t="s">
         <v>587</v>
+      </c>
+    </row>
+    <row r="21" customFormat="false" ht="82.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A21" s="0" t="n">
+        <v>17</v>
+      </c>
+      <c r="B21" s="132" t="s">
+        <v>1635</v>
+      </c>
+      <c r="C21" s="132" t="s">
+        <v>1636</v>
+      </c>
+      <c r="D21" s="132" t="s">
+        <v>1637</v>
+      </c>
+      <c r="E21" s="132" t="s">
+        <v>1638</v>
+      </c>
+      <c r="F21" s="132" t="s">
+        <v>1639</v>
+      </c>
+      <c r="G21" s="132" t="s">
+        <v>1640</v>
       </c>
     </row>
   </sheetData>
@@ -35724,7 +35765,8 @@
         <v>205</v>
       </c>
       <c r="B13" s="38" t="n">
-        <v>33.48</v>
+        <f aca="false">Inflación!B183</f>
+        <v>30.25</v>
       </c>
       <c r="C13" s="38" t="n">
         <v>46.6</v>
@@ -35741,7 +35783,7 @@
         <v>206</v>
       </c>
       <c r="B14" s="39" t="n">
-        <v>46290</v>
+        <v>46203</v>
       </c>
       <c r="C14" s="40" t="n">
         <v>46266</v>
@@ -35814,7 +35856,7 @@
       </c>
       <c r="B18" s="5" t="n">
         <f aca="false">B17*B13</f>
-        <v>60264</v>
+        <v>54450</v>
       </c>
       <c r="C18" s="5" t="n">
         <f aca="false">C17*C13</f>
@@ -35897,7 +35939,7 @@
       </c>
       <c r="B23" s="41" t="n">
         <f aca="false">B21/B18</f>
-        <v>0.391908934023629</v>
+        <v>0.433755739210285</v>
       </c>
       <c r="C23" s="10" t="n">
         <f aca="false">C21/C18</f>
@@ -35918,7 +35960,7 @@
       </c>
       <c r="B24" s="4" t="n">
         <f aca="false">B21/(B21+B18)</f>
-        <v>0.281562194511337</v>
+        <v>0.302531126710048</v>
       </c>
       <c r="C24" s="4" t="n">
         <f aca="false">C21/(C21+C18)</f>
@@ -35939,7 +35981,7 @@
       </c>
       <c r="B25" s="4" t="n">
         <f aca="false">B18/(B21+B18)</f>
-        <v>0.718437805488663</v>
+        <v>0.697468873289952</v>
       </c>
       <c r="C25" s="4" t="n">
         <f aca="false">C18/(C21+C18)</f>
@@ -35980,7 +36022,7 @@
       </c>
       <c r="B28" s="24" t="n">
         <f aca="false">B9*(1+(1-B10)*B23)</f>
-        <v>0.21730085753856</v>
+        <v>0.222295883488385</v>
       </c>
       <c r="C28" s="24" t="n">
         <f aca="false">C9*(1+(1-C10)*C23)</f>
@@ -36001,7 +36043,7 @@
       </c>
       <c r="B29" s="4" t="n">
         <f aca="false">B5+B28*B8</f>
-        <v>0.104361826273881</v>
+        <v>0.104573115871559</v>
       </c>
       <c r="C29" s="4" t="n">
         <f aca="false">C5+C28*C8</f>
@@ -36085,7 +36127,7 @@
       </c>
       <c r="B33" s="4" t="n">
         <f aca="false">B25*B29+B24*B32</f>
-        <v>0.100630184051038</v>
+        <v>0.10049964337765</v>
       </c>
       <c r="C33" s="4" t="n">
         <f aca="false">C25*C29+C24*C32</f>
@@ -36114,7 +36156,7 @@
       </c>
       <c r="B36" s="4" t="n">
         <f aca="false">'Proyección Final Soriana'!B126</f>
-        <v>0.0956277841268195</v>
+        <v>0.0956277840146585</v>
       </c>
       <c r="C36" s="4"/>
       <c r="D36" s="4"/>
@@ -36125,7 +36167,7 @@
       </c>
       <c r="B37" s="4" t="n">
         <f aca="false">B33</f>
-        <v>0.100630184051038</v>
+        <v>0.10049964337765</v>
       </c>
       <c r="C37" s="4"/>
       <c r="D37" s="4"/>
@@ -36136,7 +36178,7 @@
       </c>
       <c r="B38" s="4" t="n">
         <f aca="false">B37-B36</f>
-        <v>0.00500239992421848</v>
+        <v>0.00487185936299141</v>
       </c>
       <c r="C38" s="4"/>
       <c r="D38" s="4"/>
@@ -36354,7 +36396,7 @@
       </c>
       <c r="B15" s="4" t="n">
         <f aca="false">WACC!B33</f>
-        <v>0.100630184051038</v>
+        <v>0.10049964337765</v>
       </c>
       <c r="C15" s="27"/>
       <c r="D15" s="27"/>
@@ -36663,23 +36705,23 @@
       <c r="B28" s="46"/>
       <c r="C28" s="46" t="n">
         <f aca="false">1/(1+$B$15)^C19</f>
-        <v>0.908570394025854</v>
+        <v>0.908678168155333</v>
       </c>
       <c r="D28" s="46" t="n">
         <f aca="false">1/(1+$B$15)^D19</f>
-        <v>0.825500160900296</v>
+        <v>0.825696013282131</v>
       </c>
       <c r="E28" s="46" t="n">
         <f aca="false">1/(1+$B$15)^E19</f>
-        <v>0.750025006457588</v>
+        <v>0.750291940802368</v>
       </c>
       <c r="F28" s="46" t="n">
         <f aca="false">1/(1+$B$15)^F19</f>
-        <v>0.681450515646415</v>
+        <v>0.681773906350006</v>
       </c>
       <c r="G28" s="46" t="n">
         <f aca="false">1/(1+$B$15)^G19</f>
-        <v>0.619145763509984</v>
+        <v>0.619513064318229</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -36689,23 +36731,23 @@
       <c r="B29" s="5"/>
       <c r="C29" s="5" t="n">
         <f aca="false">C27*C28</f>
-        <v>6240.84647099001</v>
+        <v>6241.58675682811</v>
       </c>
       <c r="D29" s="5" t="n">
         <f aca="false">D27*D28</f>
-        <v>5868.70702900433</v>
+        <v>5870.09939729735</v>
       </c>
       <c r="E29" s="5" t="n">
         <f aca="false">E27*E28</f>
-        <v>5518.75812878653</v>
+        <v>5520.72225807879</v>
       </c>
       <c r="F29" s="5" t="n">
         <f aca="false">F27*F28</f>
-        <v>5189.67655627114</v>
+        <v>5192.13938095819</v>
       </c>
       <c r="G29" s="5" t="n">
         <f aca="false">G27*G28</f>
-        <v>4880.21800017393</v>
+        <v>4883.11313104862</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -36722,7 +36764,7 @@
       </c>
       <c r="B31" s="5" t="n">
         <f aca="false">SUM(C29:G29)</f>
-        <v>27698.2061852259</v>
+        <v>27707.6609242111</v>
       </c>
       <c r="C31" s="47"/>
       <c r="D31" s="47"/>
@@ -36745,7 +36787,7 @@
       </c>
       <c r="B33" s="5" t="n">
         <f aca="false">B32/(B15-B16)</f>
-        <v>124303.410482692</v>
+        <v>124551.146959902</v>
       </c>
       <c r="C33" s="2"/>
       <c r="D33" s="2"/>
@@ -36759,7 +36801,7 @@
       </c>
       <c r="B34" s="5" t="n">
         <f aca="false">B33*G28</f>
-        <v>76961.9299902015</v>
+        <v>77161.0627174786</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -36768,7 +36810,7 @@
       </c>
       <c r="B35" s="5" t="n">
         <f aca="false">B31+B34</f>
-        <v>104660.136175427</v>
+        <v>104868.72364169</v>
       </c>
       <c r="C35" s="2"/>
       <c r="D35" s="2"/>
@@ -36809,7 +36851,7 @@
       </c>
       <c r="B39" s="5" t="n">
         <f aca="false">B35+B36+B37</f>
-        <v>90337.1361754274</v>
+        <v>90545.7236416897</v>
       </c>
       <c r="C39" s="2"/>
       <c r="D39" s="2"/>
@@ -36832,7 +36874,7 @@
       </c>
       <c r="B41" s="49" t="n">
         <f aca="false">B39/B40</f>
-        <v>50.1872978752374</v>
+        <v>50.3031798009387</v>
       </c>
       <c r="C41" s="50"/>
       <c r="D41" s="51" t="s">
@@ -36840,7 +36882,7 @@
       </c>
       <c r="E41" s="52" t="n">
         <f aca="false">'Proyección Soriana'!B85</f>
-        <v>50.1811650263689</v>
+        <v>50.2970347293132</v>
       </c>
       <c r="F41" s="2"/>
       <c r="G41" s="2"/>
@@ -36851,7 +36893,7 @@
       </c>
       <c r="B42" s="49" t="n">
         <f aca="false">WACC!B13</f>
-        <v>33.48</v>
+        <v>30.25</v>
       </c>
       <c r="C42" s="53"/>
       <c r="D42" s="51" t="s">
@@ -36859,7 +36901,7 @@
       </c>
       <c r="E42" s="54" t="n">
         <f aca="false">B41-E41</f>
-        <v>0.00613284886858168</v>
+        <v>0.00614507162552513</v>
       </c>
     </row>
     <row r="43" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -36868,7 +36910,7 @@
       </c>
       <c r="B43" s="55" t="n">
         <f aca="false">B41/B42-1</f>
-        <v>0.499023234027403</v>
+        <v>0.662915034741776</v>
       </c>
       <c r="C43" s="53"/>
       <c r="D43" s="51" t="s">
@@ -36876,7 +36918,7 @@
       </c>
       <c r="E43" s="56" t="n">
         <f aca="false">B41/E41-1</f>
-        <v>0.000122214158745804</v>
+        <v>0.000122175624439835</v>
       </c>
     </row>
     <row r="44" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -36885,7 +36927,7 @@
       </c>
       <c r="B44" s="7" t="n">
         <f aca="false">B34/B35</f>
-        <v>0.735350944520087</v>
+        <v>0.735787182660092</v>
       </c>
     </row>
     <row r="46" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -39217,23 +39259,23 @@
       <c r="B15" s="7"/>
       <c r="C15" s="7" t="n">
         <f aca="false">Valuación!$B$15</f>
-        <v>0.100630184051038</v>
+        <v>0.10049964337765</v>
       </c>
       <c r="D15" s="7" t="n">
         <f aca="false">Valuación!$B$15</f>
-        <v>0.100630184051038</v>
+        <v>0.10049964337765</v>
       </c>
       <c r="E15" s="7" t="n">
         <f aca="false">Valuación!$B$15</f>
-        <v>0.100630184051038</v>
+        <v>0.10049964337765</v>
       </c>
       <c r="F15" s="7" t="n">
         <f aca="false">Valuación!$B$15</f>
-        <v>0.100630184051038</v>
+        <v>0.10049964337765</v>
       </c>
       <c r="G15" s="7" t="n">
         <f aca="false">Valuación!$B$15</f>
-        <v>0.100630184051038</v>
+        <v>0.10049964337765</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -40561,23 +40603,23 @@
       <c r="B67" s="3"/>
       <c r="C67" s="46" t="n">
         <f aca="false">1/(1+C15)^C66</f>
-        <v>0.908570394025854</v>
+        <v>0.908678168155333</v>
       </c>
       <c r="D67" s="46" t="n">
         <f aca="false">1/(1+D15)^D66</f>
-        <v>0.825500160900296</v>
+        <v>0.825696013282131</v>
       </c>
       <c r="E67" s="46" t="n">
         <f aca="false">1/(1+E15)^E66</f>
-        <v>0.750025006457588</v>
+        <v>0.750291940802368</v>
       </c>
       <c r="F67" s="46" t="n">
         <f aca="false">1/(1+F15)^F66</f>
-        <v>0.681450515646415</v>
+        <v>0.681773906350006</v>
       </c>
       <c r="G67" s="46" t="n">
         <f aca="false">1/(1+G15)^G66</f>
-        <v>0.619145763509984</v>
+        <v>0.619513064318229</v>
       </c>
     </row>
     <row r="68" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -40587,23 +40629,23 @@
       <c r="B68" s="3"/>
       <c r="C68" s="5" t="n">
         <f aca="false">C65*C67</f>
-        <v>6240.18821173953</v>
+        <v>6240.92841949528</v>
       </c>
       <c r="D68" s="5" t="n">
         <f aca="false">D65*D67</f>
-        <v>5868.08802151742</v>
+        <v>5869.48024294906</v>
       </c>
       <c r="E68" s="5" t="n">
         <f aca="false">E65*E67</f>
-        <v>5518.17603249457</v>
+        <v>5520.13995461842</v>
       </c>
       <c r="F68" s="5" t="n">
         <f aca="false">F65*F67</f>
-        <v>5189.12917017281</v>
+        <v>5191.59173509108</v>
       </c>
       <c r="G68" s="5" t="n">
         <f aca="false">G65*G67</f>
-        <v>4879.70325451277</v>
+        <v>4882.59808002076</v>
       </c>
     </row>
     <row r="69" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -40634,7 +40676,7 @@
       </c>
       <c r="B71" s="5" t="n">
         <f aca="false">SUM(C68:G68)</f>
-        <v>27695.2846904371</v>
+        <v>27704.7384321746</v>
       </c>
       <c r="C71" s="35"/>
       <c r="D71" s="35"/>
@@ -40662,7 +40704,7 @@
       </c>
       <c r="B73" s="5" t="n">
         <f aca="false">B72/(G15-G16)</f>
-        <v>124290.299461584</v>
+        <v>124538.009808551</v>
       </c>
       <c r="C73" s="35"/>
       <c r="D73" s="35"/>
@@ -40676,7 +40718,7 @@
       </c>
       <c r="B74" s="5" t="n">
         <f aca="false">B73*G67</f>
-        <v>76953.8123570269</v>
+        <v>77152.9240805892</v>
       </c>
       <c r="C74" s="35"/>
       <c r="D74" s="35"/>
@@ -40690,7 +40732,7 @@
       </c>
       <c r="B75" s="5" t="n">
         <f aca="false">B71+B74</f>
-        <v>104649.097047464</v>
+        <v>104857.662512764</v>
       </c>
       <c r="C75" s="35"/>
       <c r="D75" s="35"/>
@@ -40704,7 +40746,7 @@
       </c>
       <c r="B76" s="7" t="n">
         <f aca="false">B74/B75</f>
-        <v>0.735350944520087</v>
+        <v>0.735787182660092</v>
       </c>
       <c r="C76" s="35"/>
       <c r="D76" s="35"/>
@@ -40740,7 +40782,7 @@
       </c>
       <c r="B79" s="5" t="n">
         <f aca="false">B75</f>
-        <v>104649.097047464</v>
+        <v>104857.662512764</v>
       </c>
       <c r="C79" s="35"/>
       <c r="D79" s="35"/>
@@ -40796,7 +40838,7 @@
       </c>
       <c r="B83" s="5" t="n">
         <f aca="false">SUM(B79:B82)</f>
-        <v>90326.0970474639</v>
+        <v>90534.6625127637</v>
       </c>
       <c r="C83" s="35"/>
       <c r="D83" s="35"/>
@@ -40824,7 +40866,7 @@
       </c>
       <c r="B85" s="24" t="n">
         <f aca="false">B83/B84</f>
-        <v>50.1811650263689</v>
+        <v>50.2970347293132</v>
       </c>
       <c r="C85" s="35"/>
       <c r="D85" s="35"/>
@@ -40838,7 +40880,7 @@
       </c>
       <c r="B86" s="24" t="n">
         <f aca="false">Valuación!B42</f>
-        <v>33.48</v>
+        <v>30.25</v>
       </c>
       <c r="C86" s="35"/>
       <c r="D86" s="35"/>
@@ -40852,7 +40894,7 @@
       </c>
       <c r="B87" s="7" t="n">
         <f aca="false">B85/B86-1</f>
-        <v>0.498840054551041</v>
+        <v>0.662711891878122</v>
       </c>
       <c r="C87" s="35"/>
       <c r="D87" s="35"/>

</xml_diff>